<commit_message>
Hero, Method, Thinking posts, cover photos, favicon, ES/EN
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/database/hipernova-portafolio-db.xlsx
+++ b/database/hipernova-portafolio-db.xlsx
@@ -12,6 +12,7 @@
     <sheet name="Experience" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Pages" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Config" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Translations" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -430,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q48"/>
+  <dimension ref="A1:U48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -450,6 +451,10 @@
     <col width="40" customWidth="1" min="15" max="15"/>
     <col width="50" customWidth="1" min="16" max="16"/>
     <col width="60" customWidth="1" min="17" max="17"/>
+    <col width="44" customWidth="1" min="18" max="18"/>
+    <col width="44" customWidth="1" min="19" max="19"/>
+    <col width="40" customWidth="1" min="20" max="20"/>
+    <col width="60" customWidth="1" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -536,6 +541,26 @@
       <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>body_html</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>title_es</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>sub_es</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>excerpt_es</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>body_html_es</t>
         </is>
       </c>
     </row>
@@ -618,6 +643,18 @@
 &lt;p&gt;The Sprint transformed a complex operational challenge into a validated product concept, a prioritized backlog, and a clear path toward implementation. The team aligned around a shared vision for a more standardized, traceable, and scalable process, with five core modules and more than 20 key functionalities defined during the engagement. Most importantly, the work reframed automation not simply as a way to reduce manual effort, but as a means to free analysts to focus on judgment, operational insight, and stronger decision-making.&lt;/p&gt;</t>
         </is>
       </c>
+      <c r="R2" s="2" t="inlineStr">
+        <is>
+          <t>Sprint de diseño de tarifas OPEX</t>
+        </is>
+      </c>
+      <c r="S2" s="2" t="inlineStr">
+        <is>
+          <t>De cálculos fragmentados a un sistema de decisión más confiable</t>
+        </is>
+      </c>
+      <c r="T2" s="2" t="inlineStr"/>
+      <c r="U2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -699,6 +736,18 @@
 &lt;p&gt;The work also reframed one of the company’s most important assets: its operational footprint was not simply evidence of scale, but the foundation of an intelligence advantage that could inform both client decisions and future differentiation.&lt;/p&gt;</t>
         </is>
       </c>
+      <c r="R3" s="2" t="inlineStr">
+        <is>
+          <t>Connected Compass</t>
+        </is>
+      </c>
+      <c r="S3" s="2" t="inlineStr">
+        <is>
+          <t>Convertir la experiencia operativa en un sistema estratégico de crecimiento</t>
+        </is>
+      </c>
+      <c r="T3" s="2" t="inlineStr"/>
+      <c r="U3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -779,6 +828,18 @@
 &lt;p&gt;Four strategic territories of opportunity were identified, along with corresponding lines of action, such as &lt;strong&gt;improving governance, fostering collaboration, and optimizing talent management.&lt;/strong&gt; These outcomes laid the groundwork for VTI to become a more credible, integrated, and strategically aligned partner within Ecopetrol. Additionally, the initiative highlighted the importance of closing gaps between business and technology, ensuring that VTI evolves from a service provider to a strategic enabler in Ecopetrol’s energy transition journey.&lt;/p&gt;</t>
         </is>
       </c>
+      <c r="R4" s="2" t="inlineStr">
+        <is>
+          <t>Transformar la VTI en un habilitador estratégico</t>
+        </is>
+      </c>
+      <c r="S4" s="2" t="inlineStr">
+        <is>
+          <t>Alinear innovación y tecnología con la visión 2040 de Ecopetrol</t>
+        </is>
+      </c>
+      <c r="T4" s="2" t="inlineStr"/>
+      <c r="U4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -852,6 +913,18 @@
 &lt;p&gt;The workshop resulted in a clear articulation of GIP’s purpose: to orchestrate and drive innovation and technological transformation across Ecopetrol, contributing to a more sustainable, competitive, and prosperous energy future. Eight critical capabilities were identified, providing a foundation for GIP’s strategic framework. The session also highlighted key barriers, such as siloed operations and resistance to change, and emphasized the need for cultural shifts to foster innovation. Moving forward, the outcomes will guide the development of strategic priorities, roadmaps, and activation models to ensure GIP’s alignment with Ecopetrol’s 2040 goals while maximizing value for stakeholders.&lt;/p&gt;</t>
         </is>
       </c>
+      <c r="R5" s="2" t="inlineStr">
+        <is>
+          <t>Redefinir las capacidades clave</t>
+        </is>
+      </c>
+      <c r="S5" s="2" t="inlineStr">
+        <is>
+          <t>Prioridades estratégicas para la innovación y la gestión de portafolio en Ecopetrol</t>
+        </is>
+      </c>
+      <c r="T5" s="2" t="inlineStr"/>
+      <c r="U5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -920,6 +993,14 @@
 &lt;p&gt;As the CX Lead, my role was to accompany and guide the team throughout the strategic definition of Itaú’s new customer experience. I provided coaching to the internal designer to enhance their leadership and strategic thinking, while also offering experience frameworks, inspirational cases, and competitive benchmarks to enrich the design process. I supported the identification of experience drivers and the construction of a transformation model that considered the business, the customer, and the competitive landscape. My involvement was also key in aligning cross-functional teams—business, UX, tech—around a shared vision, and in shaping a clear narrative that connected the current challenges with the desired future state for Itaú’s experience.&lt;/p&gt;</t>
         </is>
       </c>
+      <c r="R6" s="2" t="inlineStr">
+        <is>
+          <t>Transformación estratégica de CX para Itaú Colombia</t>
+        </is>
+      </c>
+      <c r="S6" s="2" t="inlineStr"/>
+      <c r="T6" s="2" t="inlineStr"/>
+      <c r="U6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -1013,6 +1094,18 @@
 &lt;p&gt;&lt;strong&gt;Key learning:&lt;/strong&gt; Successful technology foresight transformation requires simultaneous intervention across strategy alignment, governance structure, intelligence systems, methodological frameworks, and cultural change—achieved through collaborative co-creation that builds shared ownership and clear evolutionary pathway from core competencies toward comprehensive anticipation capabilities.&lt;/p&gt;</t>
         </is>
       </c>
+      <c r="R7" s="2" t="inlineStr">
+        <is>
+          <t>FARO CT+I</t>
+        </is>
+      </c>
+      <c r="S7" s="2" t="inlineStr">
+        <is>
+          <t>Modelo de prospectiva tecnológica estratégica para Ecopetrol</t>
+        </is>
+      </c>
+      <c r="T7" s="2" t="inlineStr"/>
+      <c r="U7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -1092,6 +1185,18 @@
 &lt;p&gt;The project laid the foundation to transform a fragmented digital landscape into a &lt;strong&gt;coherent, user-centered, and governable ecosystem&lt;/strong&gt;. The experience strategy enabled prioritization of key services and a structure rooted in real user needs. The governance model introduced clear ownership, cross-functional coordination, and mechanisms for sustained evolution. A key learning was that digital transformation isn’t just about platforms—it requires alignment between vision, operations, and organizational culture.&lt;/p&gt;</t>
         </is>
       </c>
+      <c r="R8" s="2" t="inlineStr">
+        <is>
+          <t>Transformar el ecosistema digital de la CCB</t>
+        </is>
+      </c>
+      <c r="S8" s="2" t="inlineStr">
+        <is>
+          <t>De portales fragmentados a una experiencia unificada</t>
+        </is>
+      </c>
+      <c r="T8" s="2" t="inlineStr"/>
+      <c r="U8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -1174,6 +1279,18 @@
 &lt;p&gt;Educators and families gain simple, repeatable strategies that extend from the classroom into the home. The Caldas pilot establishes the first node in a larger vision: a MERAKI network of sensory spaces, rooted in equity, science, and care—positioned to scale across new communities in the years ahead.&lt;/p&gt;</t>
         </is>
       </c>
+      <c r="R9" s="2" t="inlineStr">
+        <is>
+          <t>MERAKI</t>
+        </is>
+      </c>
+      <c r="S9" s="2" t="inlineStr">
+        <is>
+          <t>Entornos sensoriales inclusivos para la primera infancia (programa de voluntariado)</t>
+        </is>
+      </c>
+      <c r="T9" s="2" t="inlineStr"/>
+      <c r="U9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -1258,6 +1375,14 @@
 &lt;p&gt;This initiative transformed cash flow management at Ecopetrol. The platform enabled real-time insights, reduced manual data handling, and improved forecast accuracy. It also supported strategic decision-making with simulation and optimization tools. Beyond the technical benefits, the project fostered a cultural shift toward agility, user-centered thinking, and innovation—laying the groundwork for a smarter, more resilient financial future.&lt;/p&gt;</t>
         </is>
       </c>
+      <c r="R10" s="2" t="inlineStr">
+        <is>
+          <t>Fortalecer la estrategia financiera de Ecopetrol con una solución digital de flujo de caja 360°</t>
+        </is>
+      </c>
+      <c r="S10" s="2" t="inlineStr"/>
+      <c r="T10" s="2" t="inlineStr"/>
+      <c r="U10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -1333,6 +1458,14 @@
 &lt;p&gt;At Ecopetrol's refineries, water from the Magdalena River must be clarified before entering the production cycle, leaving behind solid matter that was previously treated as waste. At Neture Impact (part of VML), we helped Ecopetrol transform this byproduct into sustainable bricks, turning what once was discarded material into a valuable commercial solution for the construction industry.&lt;/p&gt;</t>
         </is>
       </c>
+      <c r="R11" s="2" t="inlineStr">
+        <is>
+          <t>Explorar oportunidades de reutilización de subproductos de Ecopetrol en construcción sostenible con enfoque circular</t>
+        </is>
+      </c>
+      <c r="S11" s="2" t="inlineStr"/>
+      <c r="T11" s="2" t="inlineStr"/>
+      <c r="U11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -1401,6 +1534,14 @@
 &lt;ul&gt;&lt;li&gt;&lt;strong&gt;Structured Methodology:&lt;/strong&gt; A clear, five-stage methodology for characterizing the mega-challenges was created, providing a structured approach for analysis and decision-making.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Shared Understanding:&lt;/strong&gt; The workshop and subsequent report fostered a shared understanding of the challenges and the importance of a multidisciplinary approach.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Enhanced Collaboration:&lt;/strong&gt; The participatory process encouraged collaboration and knowledge sharing between different areas and subsidiaries within Ecopetrol.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Strategic Alignment:&lt;/strong&gt; The methodology ensured alignment with Ecopetrol's 2040 vision and strategic objectives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Actionable Framework:&lt;/strong&gt; The defined methodology and pilot project recommendation provided an actionable framework for moving forward with the characterization process.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Capacity Building:&lt;/strong&gt; The workshop and supporting materials contributed to capacity building within Ecopetrol on systems thinking and participatory methods.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Increased Efficiency:&lt;/strong&gt; The structured approach is expected to increase efficiency in resource allocation and project prioritization.&lt;/li&gt;&lt;/ul&gt;</t>
         </is>
       </c>
+      <c r="R12" s="2" t="inlineStr">
+        <is>
+          <t>Un enfoque sistémico para la estrategia de ciencia y tecnología de Ecopetrol basada en retos</t>
+        </is>
+      </c>
+      <c r="S12" s="2" t="inlineStr"/>
+      <c r="T12" s="2" t="inlineStr"/>
+      <c r="U12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -1482,6 +1623,14 @@
 &lt;p&gt;By addressing the technological and methodological gaps, the Design Sprint initiative has paved the way for more robust and scalable solutions, ultimately contributing to Ecopetrol's mission of generating sustainable value for its stakeholders.&lt;/p&gt;</t>
         </is>
       </c>
+      <c r="R13" s="2" t="inlineStr">
+        <is>
+          <t>Potenciar el análisis de precios en Ecopetrol</t>
+        </is>
+      </c>
+      <c r="S13" s="2" t="inlineStr"/>
+      <c r="T13" s="2" t="inlineStr"/>
+      <c r="U13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
@@ -1552,6 +1701,14 @@
 &lt;ul&gt;&lt;li&gt;Conducted a one-day intensive bootcamp where the agile design framework and its relevance in business contexts were introduced.&lt;/li&gt;&lt;li&gt;Defined long-term expectations and goals for the Analytics Hub team.&lt;/li&gt;&lt;li&gt;Identified key problems using the Challenge Map and HMW questions.&lt;/li&gt;&lt;li&gt;Generated creative solutions using techniques like Crazy 8.&lt;/li&gt;&lt;li&gt;Built rapid prototypes of the best-selected ideas.&lt;/li&gt;&lt;li&gt;Tested the prototypes with real users to gather feedback.&lt;/li&gt;&lt;li&gt;Summarized findings and planned the next steps to implement the developed solutions.&lt;/li&gt;&lt;/ul&gt;</t>
         </is>
       </c>
+      <c r="R14" s="2" t="inlineStr">
+        <is>
+          <t>Diseño e implementación de un bootcamp de diseño ágil en Ecopetrol</t>
+        </is>
+      </c>
+      <c r="S14" s="2" t="inlineStr"/>
+      <c r="T14" s="2" t="inlineStr"/>
+      <c r="U14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
@@ -1628,6 +1785,18 @@
 &lt;ul&gt;&lt;li&gt;Enhanced decision-making processes, enabling quicker and more informed responses to market fluctuations.&lt;/li&gt;&lt;li&gt;Improved operational efficiency through optimized manual processes and better interdepartmental coordination.&lt;/li&gt;&lt;li&gt;Increased commercial margins by aligning trading strategies with advanced analytics insights.&lt;/li&gt;&lt;li&gt;Boosted customer satisfaction by providing greater transparency, personalization, and faster transaction times.&lt;/li&gt;&lt;li&gt;Facilitated the adoption of new trading methodologies and tools among Ecopetrol's staff, ensuring a smooth transition to more advanced trading practices.&lt;/li&gt;&lt;/ul&gt;</t>
         </is>
       </c>
+      <c r="R15" s="2" t="inlineStr">
+        <is>
+          <t>Transformar el trading de petróleo</t>
+        </is>
+      </c>
+      <c r="S15" s="2" t="inlineStr">
+        <is>
+          <t>El salto de Ecopetrol hacia la analítica avanzada</t>
+        </is>
+      </c>
+      <c r="T15" s="2" t="inlineStr"/>
+      <c r="U15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
@@ -1714,6 +1883,18 @@
 &lt;p&gt;The project delivered Parque Explora’s first formal corporate strategy, fully co-created and approved by its leadership team. It established a strategic operating system that aligns its dual identities—museum and innovation partner—and positions it as a catalyst for collective learning and transformation. Personally, the project deepened my practice in strategic foresight, cultural systems design, and public innovation—reinforcing design as a driver of systemic change.&lt;/p&gt;</t>
         </is>
       </c>
+      <c r="R16" s="2" t="inlineStr">
+        <is>
+          <t>Futuros tangibles</t>
+        </is>
+      </c>
+      <c r="S16" s="2" t="inlineStr">
+        <is>
+          <t>Una estrategia con propósito para un centro de ciencia</t>
+        </is>
+      </c>
+      <c r="T16" s="2" t="inlineStr"/>
+      <c r="U16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
@@ -1791,6 +1972,14 @@
 &lt;p&gt;&lt;strong&gt;Ideation and Solution Development.&lt;/strong&gt; Held collaborative workshops to brainstorm and prioritize potential solutions. Developed detailed proposals for initiatives with the most potential impact.&lt;/p&gt;</t>
         </is>
       </c>
+      <c r="R17" s="2" t="inlineStr">
+        <is>
+          <t>Mejorar la experiencia de cliente en las tiendas Coppel</t>
+        </is>
+      </c>
+      <c r="S17" s="2" t="inlineStr"/>
+      <c r="T17" s="2" t="inlineStr"/>
+      <c r="U17" s="2" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
@@ -1879,6 +2068,18 @@
 &lt;p&gt;The project delivered a shared strategic vision, a prioritized roadmap, and a set of actionable growth drivers that both KOF and KO adopted as the foundation for the next evolution of the D2C channel. These definitions have informed subsequent investment decisions and served as the north star for digital, portfolio, and organizational transformation. For me, this project sharpened my ability to design in complexity—balancing user insight, business logic, and systemic change—while facilitating alignment across diverse executive audiences.&lt;/p&gt;</t>
         </is>
       </c>
+      <c r="R18" s="2" t="inlineStr">
+        <is>
+          <t>Definir las prioridades estratégicas de “Coca-Cola En Tu Hogar”</t>
+        </is>
+      </c>
+      <c r="S18" s="2" t="inlineStr">
+        <is>
+          <t>Canal D2C</t>
+        </is>
+      </c>
+      <c r="T18" s="2" t="inlineStr"/>
+      <c r="U18" s="2" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
@@ -1960,6 +2161,18 @@
 &lt;ol&gt;&lt;li&gt;&lt;strong&gt;Collaborative Research:&lt;/strong&gt; The CRC facilitates cutting-edge research in climate science, focusing on practical solutions that can be implemented in urban settings. It encourages collaboration between scientists, policymakers, and community leaders to address local climate issues effectively.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Education and Training:&lt;/strong&gt; The center offers extensive training programs and workshops aimed at building capacity among residents, professionals, and policymakers. These initiatives focus on climate literacy, sustainable practices, and innovative adaptation strategies.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Policy Advocacy:&lt;/strong&gt; By engaging in political advocacy, the CRC seeks to influence public policies and promote regulations that support climate resilience and social equity. It acts as a voice for vulnerable communities, ensuring their needs and perspectives are considered in decision-making processes.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Public Awareness and Outreach:&lt;/strong&gt; The CRC is dedicated to raising public awareness about the impacts of climate change and the importance of resilience. Through campaigns, seminars, and community events, it aims to foster a culture of proactive adaptation and environmental stewardship.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Innovation Hub:&lt;/strong&gt; The center serves as an incubator for climate-related innovations and entrepreneurial initiatives. It supports startups and projects that offer sustainable solutions to urban challenges, providing resources and mentorship to turn ideas into impactful actions.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Temporary Refuge for Climate Migrants:&lt;/strong&gt; Recognizing the growing issue of climate-induced migration, the CRC provides temporary shelter and support services for climate migrants. This initiative ensures that migrants have access to essential resources and integration programs.&lt;/li&gt;&lt;/ol&gt;</t>
         </is>
       </c>
+      <c r="R19" s="2" t="inlineStr">
+        <is>
+          <t>El futuro de la Ciudad de México</t>
+        </is>
+      </c>
+      <c r="S19" s="2" t="inlineStr">
+        <is>
+          <t>Construir resiliencia a través del Centro de Resiliencia Climática (concepto)</t>
+        </is>
+      </c>
+      <c r="T19" s="2" t="inlineStr"/>
+      <c r="U19" s="2" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
@@ -2037,6 +2250,14 @@
 &lt;p&gt;A core component of the process was a foresight exercise where participants envisioned ZooBaq’s long-term role in the conservation of the Caribbean region. This included co-defining a “North Star” vision and exploring plausible future scenarios around infrastructure, community engagement, and sustainability. These scenario explorations helped identify strategic tensions and informed the creation of a phased roadmap responsive to both current constraints and future possibilities.&lt;/p&gt;</t>
         </is>
       </c>
+      <c r="R20" s="2" t="inlineStr">
+        <is>
+          <t>Crear el futuro de la Fundación Botánica y Zoológica de Barranquilla (FBZB)</t>
+        </is>
+      </c>
+      <c r="S20" s="2" t="inlineStr"/>
+      <c r="T20" s="2" t="inlineStr"/>
+      <c r="U20" s="2" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
@@ -2116,6 +2337,14 @@
 &lt;ol&gt;&lt;li&gt;&lt;strong&gt;Increased Member Engagement:&lt;/strong&gt; Boost regular contributions by improving awareness of the benefits of formal employment and consistent savings.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Enhanced Financial Literacy:&lt;/strong&gt; Provide comprehensive financial education to empower members with better saving habits and informed decision-making.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Operational Efficiency:&lt;/strong&gt; Streamline processes and integrate data to improve internal workflows and customer service efficiency.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Sustainable Saving Practices:&lt;/strong&gt; Promote voluntary savings and reward good financial behaviors through innovative programs and incentives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Social Inclusion and Formal Employment:&lt;/strong&gt; Support inactive and informal workers in transitioning to formal employment, increasing their chances of securing a full pension.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Improved Customer Experience:&lt;/strong&gt; Enhance the overall member experience with personalized support, clear information, and responsive service throughout their savings journey.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Strengthened Community Trust:&lt;/strong&gt; Foster a sense of belonging and trust among affiliates towards AFORE Coppel, enhancing loyalty and long-term engagement.&lt;/li&gt;&lt;/ol&gt;</t>
         </is>
       </c>
+      <c r="R21" s="2" t="inlineStr">
+        <is>
+          <t>Mejorar el acceso a la pensión para los afiliados de AFORE Coppel</t>
+        </is>
+      </c>
+      <c r="S21" s="2" t="inlineStr"/>
+      <c r="T21" s="2" t="inlineStr"/>
+      <c r="U21" s="2" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
@@ -2190,6 +2419,14 @@
 &lt;p&gt;This Design Sprint not only transformed the financial asset management processes at Ecopetrol but also set a precedent for future innovation projects, highlighting the value of agile methodologies and user-centered design in driving organizational change.&lt;/p&gt;</t>
         </is>
       </c>
+      <c r="R22" s="2" t="inlineStr">
+        <is>
+          <t>Transformar la gestión de activos financieros en Ecopetrol a través del diseño estratégico</t>
+        </is>
+      </c>
+      <c r="S22" s="2" t="inlineStr"/>
+      <c r="T22" s="2" t="inlineStr"/>
+      <c r="U22" s="2" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
@@ -2261,6 +2498,18 @@
 &lt;p&gt;The workshop reached over 300 educators across Antioquia, fostering creative dialogue and new connections within a community still recovering from the pandemic. While designed as a sensitization exercise, it activated a mindset of experimentation and empowered teachers to see themselves as agents of transformation. A key takeaway: systemic change can begin with small, intentional hacks—especially when grounded in empathy and shared purpose.&lt;/p&gt;</t>
         </is>
       </c>
+      <c r="R23" s="2" t="inlineStr">
+        <is>
+          <t>Hackear el Aula</t>
+        </is>
+      </c>
+      <c r="S23" s="2" t="inlineStr">
+        <is>
+          <t>Explorando microintervenciones creativas para transformar el aprendizaje en el aula</t>
+        </is>
+      </c>
+      <c r="T23" s="2" t="inlineStr"/>
+      <c r="U23" s="2" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
@@ -2340,6 +2589,18 @@
 &lt;p&gt;The resulting proposal redefined the Planetarium not just as a science venue, but as a cultural space for critical reflection and collective imagination. It introduced new forms of accessibility, multisensory engagement, and narrative depth that were previously missing. A key takeaway: when designing for science, grounding complexity in human emotion and local context can create deeper, more transformative public experiences.&lt;/p&gt;</t>
         </is>
       </c>
+      <c r="R24" s="2" t="inlineStr">
+        <is>
+          <t>Planetario de Medellín</t>
+        </is>
+      </c>
+      <c r="S24" s="2" t="inlineStr">
+        <is>
+          <t>Estrategia de renovación</t>
+        </is>
+      </c>
+      <c r="T24" s="2" t="inlineStr"/>
+      <c r="U24" s="2" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
@@ -2422,6 +2683,14 @@
 &lt;ul&gt;&lt;li&gt;&lt;strong&gt;Heritage Revitalization:&lt;/strong&gt; The proposed intervention aims to value and preserve Puerto Colombia's cultural heritage, turning the museum into a reference for local history and identity.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Inclusion and Community Participation:&lt;/strong&gt; Involving various voices in the project's design and planning strengthens the sense of ownership and collaboration between the community and the museum.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Tourism and Cultural Attraction:&lt;/strong&gt; The museum's renovation and expansion position Puerto Colombia as a prominent tourist and cultural destination, boosting the local economy and fostering sustainable development.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Educational Innovation:&lt;/strong&gt; Creating educational and participatory experiences enriches the museum's cultural and educational offerings, benefiting students and visitors of all ages.&lt;/li&gt;&lt;/ul&gt;</t>
         </is>
       </c>
+      <c r="R25" s="2" t="inlineStr">
+        <is>
+          <t>Plan maestro para un sitio histórico en Puerto Colombia</t>
+        </is>
+      </c>
+      <c r="S25" s="2" t="inlineStr"/>
+      <c r="T25" s="2" t="inlineStr"/>
+      <c r="U25" s="2" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
@@ -2494,6 +2763,14 @@
 &lt;ul&gt;&lt;li&gt;&lt;strong&gt;Environmental Impact:&lt;/strong&gt; Shift to electric and renewable energy reduces carbon footprint; integration of solar panels and wind turbines supports sustainability.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Customer Experience:&lt;/strong&gt; Introduction of EV charging, rental services, and experience centers; interactive and entertaining elements improve customer visits.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Economic Benefits:&lt;/strong&gt; Services like EV rentals and home charging generate additional income; new services and technologies create employment opportunities.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Sustainable Mobility:&lt;/strong&gt; Expanded network of EV chargers supports electric vehicle adoption; home charging services and public infrastructure alleviate EV range concerns.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Technological Advancements:&lt;/strong&gt; Mobile apps for services and customer interaction enhance tech integration; efficient use of renewable energy sources.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Strategic Partnerships:&lt;/strong&gt; Public-private partnerships foster sustainable mobility solutions; collaboration with startups and tech companies drives innovation.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Consumer Preferences:&lt;/strong&gt; Data analytics provide customized services, enhancing satisfaction; green energy options meet environmentally conscious consumer expectations.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Business Viability:&lt;/strong&gt; Diversification ensures long-term business viability; multiple energy and service options make stations more resilient to market changes.&lt;/li&gt;&lt;/ul&gt;</t>
         </is>
       </c>
+      <c r="R26" s="2" t="inlineStr">
+        <is>
+          <t>El futuro de las estaciones de servicio en el contexto de la transición energética</t>
+        </is>
+      </c>
+      <c r="S26" s="2" t="inlineStr"/>
+      <c r="T26" s="2" t="inlineStr"/>
+      <c r="U26" s="2" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
@@ -2572,6 +2849,18 @@
 &lt;p&gt;Finally, we supported the integration of these new public functions by training CIAT scientists as science communicators and space mediators. Their presence and active participation enriched the visitor experience, allowing for real-time interpretation, dialogue, and connection. This human-centered approach helped bridge the gap between rigorous research and societal understanding, making the science come alive for everyone.&lt;/p&gt;</t>
         </is>
       </c>
+      <c r="R27" s="2" t="inlineStr">
+        <is>
+          <t>Semillas del futuro</t>
+        </is>
+      </c>
+      <c r="S27" s="2" t="inlineStr">
+        <is>
+          <t>Transformar un centro de investigación en una puerta pública a la biodiversidad</t>
+        </is>
+      </c>
+      <c r="T27" s="2" t="inlineStr"/>
+      <c r="U27" s="2" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
@@ -2657,6 +2946,14 @@
 &lt;ul&gt;&lt;li&gt;The network of spaces is now a reality known as &lt;em&gt;Alianza Biofilia&lt;/em&gt;.&lt;/li&gt;&lt;li&gt;Successfully implemented a flexible museographic system that celebrates Colombia’s biological and cultural diversity.&lt;/li&gt;&lt;li&gt;Strengthened strategic partnerships and local capacities in science communication.&lt;/li&gt;&lt;li&gt;Enabled meaningful public engagement with science in historically underserved regions.&lt;/li&gt;&lt;li&gt;Achieved seamless integration between physical and digital museum formats.&lt;/li&gt;&lt;li&gt;Established the project as a benchmark for museum innovation and strategic design in Latin America.&lt;/li&gt;&lt;li&gt;Demonstrated the power of collaborative design in addressing complex challenges with national impact.&lt;/li&gt;&lt;/ul&gt;</t>
         </is>
       </c>
+      <c r="R28" s="2" t="inlineStr">
+        <is>
+          <t>Crear una red nacional de sedes para el Museo de Historia Natural y Cultural de Colombia</t>
+        </is>
+      </c>
+      <c r="S28" s="2" t="inlineStr"/>
+      <c r="T28" s="2" t="inlineStr"/>
+      <c r="U28" s="2" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
@@ -2742,6 +3039,18 @@
 &lt;ul&gt;&lt;li&gt;&lt;strong&gt;Community Empowerment:&lt;/strong&gt; Empower local communities by involving them in the management and activities of the park, promoting social cohesion and a sense of ownership.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Cultural Preservation:&lt;/strong&gt; Integrate the rich cultural and historical heritage of the region into the park's narrative, preserving and celebrating local traditions and knowledge.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Health and Well-being:&lt;/strong&gt; Provide a serene and educational environment for visitors, contributing to mental and physical well-being through nature-based activities.&lt;/li&gt;&lt;/ul&gt;</t>
         </is>
       </c>
+      <c r="R29" s="2" t="inlineStr">
+        <is>
+          <t>Horizontes regenerativos</t>
+        </is>
+      </c>
+      <c r="S29" s="2" t="inlineStr">
+        <is>
+          <t>Cocreación de un parque de aves y agricultura en Colombia</t>
+        </is>
+      </c>
+      <c r="T29" s="2" t="inlineStr"/>
+      <c r="U29" s="2" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
@@ -2825,6 +3134,18 @@
 &lt;p&gt;Artista de Archivo’s digital relaunch successfully extended the museum’s reach during a time of physical closure, while preserving its interactive and educational essence. The project strengthened the institution’s digital presence and set a precedent for hybrid cultural experiences. For me, it was a clear demonstration of how design can mobilize memory, creativity, and civic participation—even in times of disruption.&lt;/p&gt;</t>
         </is>
       </c>
+      <c r="R30" s="2" t="inlineStr">
+        <is>
+          <t>Composiciones</t>
+        </is>
+      </c>
+      <c r="S30" s="2" t="inlineStr">
+        <is>
+          <t>adaptar una exhibición de museo a una experiencia digital</t>
+        </is>
+      </c>
+      <c r="T30" s="2" t="inlineStr"/>
+      <c r="U30" s="2" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
@@ -2904,6 +3225,18 @@
 &lt;ul&gt;&lt;li&gt;&lt;strong&gt;Educational and Cultural Enrichment:&lt;/strong&gt; Stimulate scientific curiosity, enhance educational outcomes, and promote cultural enrichment to foster a scientifically literate and culturally aware community.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Community Development:&lt;/strong&gt; Contribute to the social and economic development of the border region by creating opportunities for social interaction, community building, and economic growth through educational and cultural activities.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Cross-Border Integration:&lt;/strong&gt; Foster collaboration and integration between Colombia and Venezuela to strengthen cross-border relationships, promote mutual understanding, and create a shared sense of regional identity.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Environmental Awareness:&lt;/strong&gt; Promote environmental consciousness and sustainability by encouraging sustainable practices, raising awareness about environmental issues, and integrating ecological education into the community.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Strategic Vision and Stakeholder Engagement:&lt;/strong&gt; Develop a clear and shared vision for the EUREKA Science Center that aligns with regional development plans and community aspirations, ensuring that the center meets the needs and expectations of the community.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Community-Centric Design:&lt;/strong&gt; Ensure the design and planning of the center are grounded in the needs and expectations of the community, creating a welcoming, engaging, and relevant space that enhances the overall user experience and fosters long-term engagement.&lt;/li&gt;&lt;/ul&gt;</t>
         </is>
       </c>
+      <c r="R31" s="2" t="inlineStr">
+        <is>
+          <t>Centro de Ciencia EUREKA</t>
+        </is>
+      </c>
+      <c r="S31" s="2" t="inlineStr">
+        <is>
+          <t>Tender puentes entre fronteras a través del conocimiento, la cultura y la innovación</t>
+        </is>
+      </c>
+      <c r="T31" s="2" t="inlineStr"/>
+      <c r="U31" s="2" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
@@ -2972,6 +3305,14 @@
 &lt;p&gt;The "Compás Estratégico" initiative resulted in a clear framework of five strategic priorities: enhancing community impact, consolidating a transmedia ecosystem, strengthening alliances for sustainability, identifying critical resources and capacities, and becoming a more agile and resilient organization. These priorities were supported by actionable goals, such as expanding digital offerings, fostering inclusivity, and improving operational flexibility. The process also highlighted the importance of leveraging technology, forming new partnerships, and addressing barriers like resistance to change. By preparing for multiple scenarios, Parque Explora positioned itself to navigate uncertainty while reinforcing its role as a leader in education, culture, and science.&lt;/p&gt;</t>
         </is>
       </c>
+      <c r="R32" s="2" t="inlineStr">
+        <is>
+          <t>Transformación estratégica de Parque Explora en medio de la crisis del Covid</t>
+        </is>
+      </c>
+      <c r="S32" s="2" t="inlineStr"/>
+      <c r="T32" s="2" t="inlineStr"/>
+      <c r="U32" s="2" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
@@ -3049,6 +3390,14 @@
 &lt;ul&gt;&lt;li&gt;&lt;strong&gt;Visitor Safety and Confidence:&lt;/strong&gt; By ensuring strict adherence to health and safety protocols, the museum aims to rebuild visitor trust and confidence, creating a safe environment for public engagement.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Operational Resilience:&lt;/strong&gt; The flexible operational model is designed to withstand future disruptions, allowing the museum to adapt quickly to changing circumstances and maintain continuity.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Sustainable Engagement:&lt;/strong&gt; Enhanced digital content and phased reopening plans aim to sustain public interest and engagement, ensuring the museum remains relevant and accessible.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Community Support and Inclusion:&lt;/strong&gt; Active involvement of local communities and stakeholders in the planning and execution process fosters a sense of ownership and support for the museum's initiatives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Long-term Viability:&lt;/strong&gt; The comprehensive strategy, including financial planning and the creation of new revenue streams, aims to secure the museum's financial health and long-term sustainability.&lt;/li&gt;&lt;/ul&gt;</t>
         </is>
       </c>
+      <c r="R33" s="2" t="inlineStr">
+        <is>
+          <t>Modelo de reapertura de museos durante el Covid-19</t>
+        </is>
+      </c>
+      <c r="S33" s="2" t="inlineStr"/>
+      <c r="T33" s="2" t="inlineStr"/>
+      <c r="U33" s="2" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
@@ -3122,6 +3471,14 @@
 &lt;p&gt;This strategic initiative, spearheaded by MEN, OEI, and Parque Explora, represents a significant step towards transforming STEM education in Colombia. By addressing the challenges and leveraging the strengths of various stakeholders, the project aims to create a robust and inclusive STEM+ framework that prepares students for the future, fosters innovation, and promotes sustainable development. This collaborative effort not only enhances the quality of education but also contributes to the overall socio-economic growth of the country.&lt;/p&gt;</t>
         </is>
       </c>
+      <c r="R34" s="2" t="inlineStr">
+        <is>
+          <t>Crear una estrategia nacional de educación STEM en Colombia</t>
+        </is>
+      </c>
+      <c r="S34" s="2" t="inlineStr"/>
+      <c r="T34" s="2" t="inlineStr"/>
+      <c r="U34" s="2" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
@@ -3202,6 +3559,18 @@
 &lt;p&gt;MALVA became a fully designed and largely implemented integrated science center, successfully unifying two previously fragmented institutions into a coherent public experience. The project refreshed scientific narratives, modernized infrastructure, and introduced more participatory, family-oriented, and inclusive ways of engaging with science. Beyond physical transformation, MALVA enabled stronger institutional collaboration and positioned &lt;em&gt;La Manzana del Saber&lt;/em&gt; as a contemporary, future-facing science and learning ecosystem—demonstrating how strategic design can drive long-term public value.&lt;/p&gt;</t>
         </is>
       </c>
+      <c r="R35" s="2" t="inlineStr">
+        <is>
+          <t>MALVA</t>
+        </is>
+      </c>
+      <c r="S35" s="2" t="inlineStr">
+        <is>
+          <t>Experiencia integrada de centro de ciencia</t>
+        </is>
+      </c>
+      <c r="T35" s="2" t="inlineStr"/>
+      <c r="U35" s="2" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
@@ -3284,6 +3653,18 @@
 &lt;figure class="c-img"&gt;&lt;img src="https://portafolio.parqueexplora.org/_next/image?url=https%3A%2F%2Fimgix.cosmicjs.com%2F89adfbb0-87c2-11ee-a141-bf415eaf0a74-img-test-1.webp%3Ffit%3Dcrop%26h%3D683%26w%3D1105%26upscale%3Dtrue%26auto%3Dformat%2Ccompress&amp;w=3840&amp;q=75" alt="Panama Canal Experience Center" loading="lazy" onerror="this.parentNode.remove()"&gt;&lt;/figure&gt;</t>
         </is>
       </c>
+      <c r="R36" s="2" t="inlineStr">
+        <is>
+          <t>Diseñar un canal para todos</t>
+        </is>
+      </c>
+      <c r="S36" s="2" t="inlineStr">
+        <is>
+          <t>Un centro interactivo en el corazón de Panamá</t>
+        </is>
+      </c>
+      <c r="T36" s="2" t="inlineStr"/>
+      <c r="U36" s="2" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
@@ -3358,6 +3739,18 @@
 &lt;ul&gt;&lt;li&gt;Ocampo-Agudelo J., Maya J. (2021) Core Concepts Linking Exhibit Design and the Visitor Experience in Science Centers: An Early Framework. In: Rauterberg M. (eds) Culture and Computing. Design Thinking and Cultural Computing. HCII 2021. Lecture Notes in Computer Science, vol 12795. Springer, Cham. &lt;a href="https://doi.org/10.1007/978-3-030-77431-8_7" target="_blank" rel="noopener"&gt;doi.org/10.1007/978-3-030-77431-8_7&lt;/a&gt;&lt;/li&gt;&lt;li&gt;&lt;a href="https://www.researchgate.net/publication/328223899_The_Design_of_Experience-centered_Exhibits_in_Science_Museums" target="_blank" rel="noopener"&gt;The Design of Experience-centered Exhibits in Science Centers&lt;/a&gt; (2018). ASTC Conference. Hartford, United States.&lt;/li&gt;&lt;li&gt;Ocampo-Agudelo, Jose; Maya, Jorge; Roldán, Andrés (2017). &lt;a href="https://www.researchgate.net/publication/321135314_A_Tool_for_the_Design_of_Experience-Centered_Exhibits_in_Science_Centers" target="_blank" rel="noopener"&gt;“A Tool for the Design of Experience-Centered Exhibits in Science Centers”&lt;/a&gt;. Poster presentation at Science Centre World Summit. Tokyo, Japan.&lt;/li&gt;&lt;li&gt;Ocampo-Agudelo, J., &amp;amp; Maya, J. (2017). &lt;a href="https://www.researchgate.net/publication/319402257_Experiential_qualities_of_science_museum_exhibits_a_thematic_analysis" target="_blank" rel="noopener"&gt;Experiential qualities of science museum exhibits: a thematic analysis.&lt;/a&gt; In DS 87-8 Proceedings of the 21st International Conference on Engineering Design (ICED 17) Vol 8: Human Behaviour in Design, Vancouver, Canada (pp. 439-448).&lt;/li&gt;&lt;/ul&gt;</t>
         </is>
       </c>
+      <c r="R37" s="2" t="inlineStr">
+        <is>
+          <t>Del insight al impacto</t>
+        </is>
+      </c>
+      <c r="S37" s="2" t="inlineStr">
+        <is>
+          <t>Un marco de investigación para diseñar exhibiciones interactivas de museo</t>
+        </is>
+      </c>
+      <c r="T37" s="2" t="inlineStr"/>
+      <c r="U37" s="2" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
@@ -3436,6 +3829,18 @@
 &lt;p&gt;After the strategic design process Biblored decided to implement a pilot in one of the major public libraries in Bogotá.&lt;/p&gt;</t>
         </is>
       </c>
+      <c r="R38" s="2" t="inlineStr">
+        <is>
+          <t>Reimaginar las bibliotecas públicas</t>
+        </is>
+      </c>
+      <c r="S38" s="2" t="inlineStr">
+        <is>
+          <t>Diseñar centros creativos para la innovación colectiva en Bogotá</t>
+        </is>
+      </c>
+      <c r="T38" s="2" t="inlineStr"/>
+      <c r="U38" s="2" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
@@ -3513,6 +3918,14 @@
 &lt;p&gt;&lt;strong&gt;Allies:&lt;/strong&gt; Cité de l'espace, Embajada de Francia en Colombia, Instituto Francés.&lt;/p&gt;</t>
         </is>
       </c>
+      <c r="R39" s="2" t="inlineStr">
+        <is>
+          <t>El Niño y La Niña, historias superpuestas</t>
+        </is>
+      </c>
+      <c r="S39" s="2" t="inlineStr"/>
+      <c r="T39" s="2" t="inlineStr"/>
+      <c r="U39" s="2" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
@@ -3588,6 +4001,14 @@
 &lt;ul&gt;&lt;li&gt;"MUSIC: You are the Orchestra" was the bronze winner in the Onsite Digital Experience category at the 2019 Muse Awards, American Alliance of Museums.&lt;/li&gt;&lt;li&gt;“Musical Landscapes,” an experience in the music hall, was the silver winner in the Video, Film, Animation, and Live Media or Digital Performances category at the 2019 Muse Awards, American Alliance of Museums.&lt;/li&gt;&lt;/ul&gt;</t>
         </is>
       </c>
+      <c r="R40" s="2" t="inlineStr">
+        <is>
+          <t>Diseño estratégico para una exposición de música</t>
+        </is>
+      </c>
+      <c r="S40" s="2" t="inlineStr"/>
+      <c r="T40" s="2" t="inlineStr"/>
+      <c r="U40" s="2" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
@@ -3671,6 +4092,18 @@
 &lt;p&gt;This work established the strategic and experiential foundation for one of Medellín’s most ambitious civic transformations. The Claustro has since evolved into a reference point for cultural life in the city, with over 2.1 million visitors and 6,000+ public events hosted between 2023 and 2025. The project demonstrated how heritage spaces can be reactivated through purpose-driven design, and it shaped my ongoing approach to aligning physical transformation with institutional vision and user meaning.&lt;/p&gt;</t>
         </is>
       </c>
+      <c r="R41" s="2" t="inlineStr">
+        <is>
+          <t>Claustro San Ignacio</t>
+        </is>
+      </c>
+      <c r="S41" s="2" t="inlineStr">
+        <is>
+          <t>Plan maestro estratégico para la transformación cultural</t>
+        </is>
+      </c>
+      <c r="T41" s="2" t="inlineStr"/>
+      <c r="U41" s="2" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
@@ -3755,6 +4188,18 @@
 &lt;figure class="c-video"&gt;&lt;iframe src="https://www.youtube-nocookie.com/embed/sT1iB5tOBgY" title="Video" loading="lazy" allow="accelerometer; encrypted-media; picture-in-picture" allowfullscreen&gt;&lt;/iframe&gt;&lt;/figure&gt;</t>
         </is>
       </c>
+      <c r="R42" s="2" t="inlineStr">
+        <is>
+          <t>Molas</t>
+        </is>
+      </c>
+      <c r="S42" s="2" t="inlineStr">
+        <is>
+          <t>capas de sabiduría</t>
+        </is>
+      </c>
+      <c r="T42" s="2" t="inlineStr"/>
+      <c r="U42" s="2" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
@@ -3834,6 +4279,14 @@
 &lt;p&gt;&lt;strong&gt;Scalability and National Adoption.&lt;/strong&gt; Since publication, the guide has become a national reference. It was instrumental in shaping the vision and spatial strategies of the &lt;strong&gt;CIBI Science Center in Dosquebradas&lt;/strong&gt; and used as a diagnostic and planning tool in the &lt;strong&gt;Science Center of the Technological University of Pereira&lt;/strong&gt;. Many more initiatives across the country continue to draw from its framework.&lt;/p&gt;</t>
         </is>
       </c>
+      <c r="R43" s="2" t="inlineStr">
+        <is>
+          <t>Guía nacional para centros de ciencia en Colombia</t>
+        </is>
+      </c>
+      <c r="S43" s="2" t="inlineStr"/>
+      <c r="T43" s="2" t="inlineStr"/>
+      <c r="U43" s="2" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
@@ -3906,6 +4359,18 @@
 &lt;p&gt;Learning by doing and teaching by showing is a common methodological commitment that is defined in spatial relationships and ways of inhabiting the project. Criteria such as spatial simultaneity, gaps and transparencies, and the mix of activities allow the generation of more complex relationships by giving visibility to all the experiences that take place, finding a fertile environment for creation.&lt;/p&gt;</t>
         </is>
       </c>
+      <c r="R44" s="2" t="inlineStr">
+        <is>
+          <t>MOVA</t>
+        </is>
+      </c>
+      <c r="S44" s="2" t="inlineStr">
+        <is>
+          <t>Centro de innovación para docentes públicos</t>
+        </is>
+      </c>
+      <c r="T44" s="2" t="inlineStr"/>
+      <c r="U44" s="2" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
@@ -3967,6 +4432,14 @@
           <t>&lt;figure class="c-video"&gt;&lt;iframe src="https://www.youtube-nocookie.com/embed/9GzNzIdNakc" title="Video" loading="lazy" allow="accelerometer; encrypted-media; picture-in-picture" allowfullscreen&gt;&lt;/iframe&gt;&lt;/figure&gt;</t>
         </is>
       </c>
+      <c r="R45" s="2" t="inlineStr">
+        <is>
+          <t>MIND Science Truck</t>
+        </is>
+      </c>
+      <c r="S45" s="2" t="inlineStr"/>
+      <c r="T45" s="2" t="inlineStr"/>
+      <c r="U45" s="2" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
@@ -4033,6 +4506,18 @@
 &lt;figure class="c-video"&gt;&lt;iframe src="https://www.youtube-nocookie.com/embed/DPe9s-1SppQ" title="Video" loading="lazy" allow="accelerometer; encrypted-media; picture-in-picture" allowfullscreen&gt;&lt;/iframe&gt;&lt;/figure&gt;</t>
         </is>
       </c>
+      <c r="R46" s="2" t="inlineStr">
+        <is>
+          <t>En escena</t>
+        </is>
+      </c>
+      <c r="S46" s="2" t="inlineStr">
+        <is>
+          <t>historias detrás de las historias</t>
+        </is>
+      </c>
+      <c r="T46" s="2" t="inlineStr"/>
+      <c r="U46" s="2" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
@@ -4106,6 +4591,18 @@
 &lt;figure class="c-video"&gt;&lt;iframe src="https://www.youtube-nocookie.com/embed/ZcotQQtb2Gg" title="Video" loading="lazy" allow="accelerometer; encrypted-media; picture-in-picture" allowfullscreen&gt;&lt;/iframe&gt;&lt;/figure&gt;</t>
         </is>
       </c>
+      <c r="R47" s="2" t="inlineStr">
+        <is>
+          <t>Historias menores</t>
+        </is>
+      </c>
+      <c r="S47" s="2" t="inlineStr">
+        <is>
+          <t>experiencia interactiva</t>
+        </is>
+      </c>
+      <c r="T47" s="2" t="inlineStr"/>
+      <c r="U47" s="2" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
@@ -4190,6 +4687,18 @@
 &lt;figure class="c-video"&gt;&lt;iframe src="https://www.youtube-nocookie.com/embed/a5zf8eEe4wU" title="Video" loading="lazy" allow="accelerometer; encrypted-media; picture-in-picture" allowfullscreen&gt;&lt;/iframe&gt;&lt;/figure&gt;</t>
         </is>
       </c>
+      <c r="R48" s="2" t="inlineStr">
+        <is>
+          <t>Mind</t>
+        </is>
+      </c>
+      <c r="S48" s="2" t="inlineStr">
+        <is>
+          <t>el mundo interior</t>
+        </is>
+      </c>
+      <c r="T48" s="2" t="inlineStr"/>
+      <c r="U48" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4202,13 +4711,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
     <col width="32" customWidth="1" min="2" max="2"/>
     <col width="90" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="5" max="5"/>
+    <col width="90" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4232,6 +4743,16 @@
           <t>symbol</t>
         </is>
       </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>title_es</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>text_es</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -4252,6 +4773,16 @@
           <t>onda</t>
         </is>
       </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Narrativa como estrategia</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Destilo ideas complejas en narrativas claras y enfocadas que inspiran acción y transformación. A través de la narración conecto profundamente con las audiencias e impulso el cambio haciendo lo esencial visible y memorable.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -4272,6 +4803,16 @@
           <t>superposicion</t>
         </is>
       </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Cocreación a escala</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Entiendo el diseño como un proceso compartido: trabajo de cerca con las comunidades para construir soluciones arraigadas en sus realidades. Este enfoque inclusivo produce resultados más significativos, sostenibles y aceptados.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -4292,6 +4833,16 @@
           <t>orbita</t>
         </is>
       </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Pensamiento sistémico</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Desde el pensamiento sistémico diseño con conciencia del contexto más amplio, conectando las dinámicas organizacionales, las necesidades de las personas y las fuerzas sociales para lograr un impacto duradero y sistémico.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -4312,6 +4863,16 @@
           <t>campo</t>
         </is>
       </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Futuros y prospectiva</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Ayudo a las organizaciones a mirar más allá del presente, diseñando soluciones preparadas para el futuro que construyen resiliencia y aseguran relevancia en un mundo en constante cambio.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -4332,6 +4893,16 @@
           <t>vector</t>
         </is>
       </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Experimentar para generar impacto rápido</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>A través del prototipado rápido y las pruebas iterativas, convierto ideas en soluciones validadas con rapidez, acelerando el aprendizaje, la adaptación y una innovación medible.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -4350,6 +4921,16 @@
       <c r="D7" s="2" t="inlineStr">
         <is>
           <t>nucleo</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Diseño de marcos a la medida</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Diseño estrategias a la medida del reto, no plantillas. Al replantear los problemas e integrar un pensamiento sistémico y centrado en las personas, abro soluciones significativas y ajustadas al contexto.</t>
         </is>
       </c>
     </row>
@@ -4364,12 +4945,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
     <col width="120" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="120" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4388,6 +4971,16 @@
           <t>html</t>
         </is>
       </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>title_es</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>html_es</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -4403,6 +4996,16 @@
           <t>As Strategic Design &amp;amp; CX Lead and now Consulting Director at VML Colombia, I've led end-to-end transformation engagements for organizations navigating strategic inflection points. My work spans foresight model design, digital ecosystem strategy, operating model redesign, and customer experience innovation — always at the intersection of design rigor and business pragmatism. I currently lead the LATAM Consulting Center of Excellence, scaling our strategic design practice across Colombia, Mexico, Peru, Chile, and Puerto Rico.</t>
         </is>
       </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>En VML</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Como líder de Diseño Estratégico y CX y hoy Director de Consultoría en VML Colombia, he liderado proyectos de transformación de principio a fin para organizaciones en puntos de inflexión estratégica. Mi trabajo abarca el diseño de modelos de prospectiva, la estrategia de ecosistemas digitales, el rediseño de modelos operativos y la innovación en experiencia de cliente — siempre en la intersección entre el rigor del diseño y el pragmatismo del negocio. Actualmente lidero el Centro de Excelencia de Consultoría para LATAM, escalando nuestra práctica de diseño estratégico en Colombia, México, Perú, Chile y Puerto Rico.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -4416,6 +5019,16 @@
       <c r="C3" s="2" t="inlineStr">
         <is>
           <t>Over 11 years at Parque Explora, I built my practice from the ground up — starting as an exhibition designer and growing into Head of Innovation. I led the institution's most ambitious transformation projects: a full Science Center renovation, the design of immersive learning environments for national and international clients, and the development of Parque Explora's innovation methodology, published as &lt;em&gt;Compás de Diseño&lt;/em&gt;. Work from this period earned recognition at the American Alliance of Museums (Muse Awards 2017) and the Ibero-American Design Biennial in Madrid.</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Antes de VML</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Durante más de 11 años en Parque Explora construí mi práctica desde cero — empecé como diseñador de exposiciones y llegué a ser Jefe de Innovación. Lideré los proyectos de transformación más ambiciosos de la institución: la renovación completa de un centro de ciencia, el diseño de entornos de aprendizaje inmersivos para clientes nacionales e internacionales y el desarrollo de la metodología de innovación de Parque Explora, publicada como &lt;em&gt;Compás de Diseño&lt;/em&gt;. El trabajo de esta etapa recibió reconocimiento de la American Alliance of Museums (Muse Awards 2017) y de la Bienal Iberoamericana de Diseño en Madrid.</t>
         </is>
       </c>
     </row>
@@ -4430,11 +5043,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="140" customWidth="1" min="2" max="2"/>
+    <col width="120" customWidth="1" min="2" max="2"/>
+    <col width="120" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4448,88 +5062,205 @@
           <t>value</t>
         </is>
       </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>value_es</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>home.lead</t>
+          <t>home.hero</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>I help organizations turn complexity into strategic clarity, and vision into action.</t>
+          <t>I help people, brands and organizations to</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Ayudo a personas, marcas y organizaciones a</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>home.bio</t>
+          <t>home.phrases</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Strategic Design &amp; CX Transformation Director with 15+ years building the conditions for organizations to navigate complexity, redesign how they operate, and create long-term value. I lead at the intersection of foresight, systems thinking, and human-centered design, translating strategic ambiguity into new operating models, digital ecosystems, and organizational capabilities. My work spans energy, financial services, retail, and public sector across Latin America.</t>
+          <t>see what we couldn't see before.
+change course.
+question the rules we were given.
+do things differently.
+turn limits into possibilities.
+imagine other futures.
+let something new emerge.
+discover new possibilities.
+shift the way they look at things.
+break with the predictable.
+reimagine what already exists.
+create from another place.
+change the context.
+redesign the conditions.
+open new paths.
+change the questions.
+challenge what was taken for granted.
+inhabit new scenarios.
+start new conversations.
+expand what seemed possible.
+connect what was separate.
+create new ways of relating.
+give shape to what doesn't exist yet.
+turn uncertainty into possibility.
+try out other futures.
+make the invisible visible.</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>ver lo que antes no veían.
+cambiar de rumbo.
+cuestionar las reglas dadas.
+hacer las cosas de otra manera.
+convertir los límites en posibilidades.
+imaginar otros futuros.
+hacer emerger algo nuevo.
+descubrir nuevas posibilidades.
+cambiar la forma de mirar.
+romper con lo predecible.
+reimaginar lo que ya existe.
+crear desde otro lugar.
+cambiar el contexto.
+rediseñar las condiciones.
+abrir nuevos caminos.
+cambiar las preguntas.
+desafiar lo que se daba por hecho.
+habitar nuevos escenarios.
+activar nuevas conversaciones.
+expandir lo que parecía posible.
+conectar lo que estaba separado.
+crear nuevas formas de relacionarse.
+dar forma a lo que aún no existe.
+convertir la incertidumbre en posibilidad.
+ensayar otros futuros.
+hacer visible lo invisible.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>approach.lead</t>
+          <t>home.lead</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Every engagement starts with a question, not a solution. My practice is built on six principles that guide how I work with organizations facing strategic complexity — from reframing the right problem to designing the conditions for lasting change.</t>
-        </is>
-      </c>
+          <t>I help organizations turn complexity into strategic clarity, and vision into action.</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>about.intro</t>
+          <t>home.bio</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>I'm a Strategic Design &amp; Transformation Director with 15+ years building the conditions for organizations to navigate complexity, reimagine how they operate, and create long-term value. My practice sits at the intersection of foresight, systems thinking, service design, and human-centered co-creation — translating strategic ambiguity into actionable frameworks, new operating models, and organizational capabilities that endure.</t>
+          <t>Strategic Design &amp; CX Transformation Director with 15+ years building the conditions for organizations to navigate complexity, redesign how they operate, and create long-term value. I lead at the intersection of foresight, systems thinking, and human-centered design, translating strategic ambiguity into new operating models, digital ecosystems, and organizational capabilities. My work spans energy, financial services, retail, and public sector across Latin America.</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Director de Diseño Estratégico y Transformación de CX con más de 15 años construyendo las condiciones para que las organizaciones naveguen la complejidad, rediseñen cómo operan y creen valor a largo plazo. Lidero en la intersección de la prospectiva, el pensamiento sistémico y el diseño centrado en las personas, traduciendo la ambigüedad estratégica en nuevos modelos operativos, ecosistemas digitales y capacidades organizacionales. Mi trabajo abarca energía, servicios financieros, retail y sector público en América Latina.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>about.quote</t>
+          <t>approach.lead</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>I believe complexity is not a problem to be solved — it's a condition to be navigated. The organizations I work with don't need simpler answers. They need better questions, clearer models, and the organizational capability to act with intention under uncertainty.</t>
+          <t>Every engagement starts with a question, not a solution. My practice is built on six principles that guide how I work with organizations facing strategic complexity — from reframing the right problem to designing the conditions for lasting change.</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Todo proyecto empieza con una pregunta, no con una solución. Mi práctica se apoya en seis principios que guían cómo trabajo con organizaciones que enfrentan complejidad estratégica — desde replantear el problema correcto hasta diseñar las condiciones para un cambio duradero.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
+          <t>about.intro</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>I'm a Strategic Design &amp; Transformation Director with 15+ years building the conditions for organizations to navigate complexity, reimagine how they operate, and create long-term value. My practice sits at the intersection of foresight, systems thinking, service design, and human-centered co-creation — translating strategic ambiguity into actionable frameworks, new operating models, and organizational capabilities that endure.</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Soy Director de Diseño Estratégico y Transformación, con más de 15 años construyendo las condiciones para que las organizaciones naveguen la complejidad, reimaginen cómo operan y creen valor a largo plazo. Mi práctica se ubica en la intersección de la prospectiva, el pensamiento sistémico, el diseño de servicios y la cocreación centrada en las personas — traduciendo la ambigüedad estratégica en marcos accionables, nuevos modelos operativos y capacidades organizacionales que perduran.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>about.quote</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>I believe complexity is not a problem to be solved — it's a condition to be navigated. The organizations I work with don't need simpler answers. They need better questions, clearer models, and the organizational capability to act with intention under uncertainty.</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Creo que la complejidad no es un problema por resolver — es una condición que hay que navegar. Las organizaciones con las que trabajo no necesitan respuestas más simples. Necesitan mejores preguntas, modelos más claros y la capacidad organizacional de actuar con intención en la incertidumbre.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
           <t>about.education</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>Master’s in Engineering (2015–2017) — EAFIT University
 Product Design Engineering (2004–2010) — EAFIT University
 Academic Exchange — Delft University of Technology (TU Delft), Netherlands (2008–2009)</t>
         </is>
       </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Maestría en Ingeniería (2015–2017) — Universidad EAFIT
+Ingeniería en Diseño de Producto (2004–2010) — Universidad EAFIT
+Intercambio académico — Universidad Tecnológica de Delft (TU Delft), Países Bajos (2008–2009)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>about.certifications</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>Systemic Design for Tackling Complexity — Service Design College, 2025
 Branding and Customer Experience — IE University, 2024
@@ -4538,14 +5269,23 @@
 Strategic Management and Innovation — Copenhagen Business School, 2021</t>
         </is>
       </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Diseño sistémico para abordar la complejidad — Service Design College, 2025
+Branding y experiencia de cliente — IE University, 2024
+Design Futures — CENTRO, 2023
+Diseño de servicios — IxDF, 2023
+Gestión estratégica e innovación — Copenhagen Business School, 2021</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>about.disciplines</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>Strategic Design
 Service Design
@@ -4558,62 +5298,95 @@
 Transition Design</t>
         </is>
       </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>about.teaching</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>11+ years of university teaching in experience design, interaction design, design thinking, and design-driven innovation at EAFIT University and Universidad Pontificia Bolivariana.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>thinking.lead</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>A collection of my articles, podcasts, and writings, reflecting my passion for design, methodologies, and experiences. Here, I share insights and reflections on innovative design practices and the creation of meaningful user experiences.</t>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Diseño estratégico
+Diseño de servicios
+Pensamiento sistémico
+Prospectiva de diseño
+Diseño centrado en las personas
+Diseño de modelos operativos
+Estrategia de ecosistemas digitales
+Sprints de diseño
+Diseño de transición</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>thinking.substack</t>
+          <t>about.teaching</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Hipernova is a space to explore the frontiers of creativity, design, technology, and purposeful living. It's not a technical blog, nor a personal diary, nor a step-by-step consultancy guide. It's a crossroads: the practice of meaningful design, the energy of transformation, the wisdom of books, and the human experiences that show us new ways of relating to the world.</t>
+          <t>11+ years of university teaching in experience design, interaction design, design thinking, and design-driven innovation at EAFIT University and Universidad Pontificia Bolivariana.</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Más de 11 años de docencia universitaria en diseño de experiencias, diseño de interacción, design thinking e innovación guiada por el diseño en la Universidad EAFIT y la Universidad Pontificia Bolivariana.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>thinking.medium</t>
+          <t>thinking.lead</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Writing for IxDF (Interaction Design Foundation) South America.</t>
+          <t>A collection of my articles, podcasts, and writings, reflecting my passion for design, methodologies, and experiences. Here, I share insights and reflections on innovative design practices and the creation of meaningful user experiences.</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Una colección de mis artículos, podcasts y escritos, que refleja mi pasión por el diseño, las metodologías y las experiencias. Aquí comparto ideas y reflexiones sobre prácticas de diseño innovadoras y la creación de experiencias de usuario con sentido.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
+          <t>thinking.substack</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Hipernova is a space to explore the frontiers of creativity, design, technology, and purposeful living. It's not a technical blog, nor a personal diary, nor a step-by-step consultancy guide. It's a crossroads: the practice of meaningful design, the energy of transformation, the wisdom of books, and the human experiences that show us new ways of relating to the world.</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Hipernova es un espacio para explorar las fronteras de la creatividad, el diseño, la tecnología y una vida con propósito. No es un blog técnico, ni un diario personal, ni una guía de consultoría paso a paso. Es una encrucijada: la práctica del diseño con sentido, la energía de la transformación, la sabiduría de los libros y las experiencias humanas que nos muestran nuevas formas de relacionarnos con el mundo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>thinking.medium</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Writing for IxDF (Interaction Design Foundation) South America.</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Escribo para IxDF (Interaction Design Foundation) Sudamérica.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
           <t>thinking.publications</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="B16" s="2" t="inlineStr">
         <is>
           <t>Ocampo-Agudelo J., Maya J. (2021) &lt;strong&gt;Core Concepts Linking Exhibit Design and the Visitor Experience in Science Centers: An Early Framework.&lt;/strong&gt; In: Rauterberg M. (eds) Culture and Computing. HCII 2021. Lecture Notes in Computer Science, vol 12795. Springer, Cham. &lt;a href="https://doi.org/10.1007/978-3-030-77431-8_7" target="_blank" rel="noopener"&gt;doi.org/10.1007/978-3-030-77431-8_7&lt;/a&gt;
 Ministerio de Educación Nacional (2020). &lt;strong&gt;Visión STEM+A: Educación Expandida para la vida.&lt;/strong&gt; Documento de trabajo del MEN.
@@ -4628,6 +5401,7 @@
 Ocampo A., Jose Augusto (2014). &lt;strong&gt;Design of Interactions for Social Appropriation of Knowledge.&lt;/strong&gt; Proceedings of the 9th International Conference on Design &amp;amp; Emotion. Bogotá. Ediciones Uniandes. &lt;a href="https://www.researchgate.net/publication/286048784_Design_of_interactions_for_social_appropriation_of_knowledge" target="_blank" rel="noopener"&gt;researchgate.net&lt;/a&gt;</t>
         </is>
       </c>
+      <c r="C16" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4640,11 +5414,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="80" customWidth="1" min="2" max="2"/>
+    <col width="80" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4658,6 +5433,11 @@
           <t>value</t>
         </is>
       </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>value_es</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -4670,6 +5450,7 @@
           <t>Jose Augusto Ocampo</t>
         </is>
       </c>
+      <c r="C2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -4682,6 +5463,7 @@
           <t>Strategic Design &amp; Transformation Director</t>
         </is>
       </c>
+      <c r="C3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -4694,6 +5476,11 @@
           <t>Strategic Design | Design Futures | Transformation Design | CX Strategy</t>
         </is>
       </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Diseño estratégico | Prospectiva de diseño | Diseño de transformación | Estrategia de CX</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -4702,6 +5489,7 @@
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr"/>
+      <c r="C5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -4710,6 +5498,7 @@
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr"/>
+      <c r="C6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -4718,6 +5507,7 @@
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr"/>
+      <c r="C7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -4728,6 +5518,1729 @@
       <c r="B8" s="2" t="inlineStr">
         <is>
           <t>08.10.2026</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B142"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="60" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>es</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Skip to content</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Saltar al contenido</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Menu</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Menú</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Work</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Trabajo</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Approach</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Enfoque</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>About</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Sobre mí</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Thinking</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Pensamiento</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>See the work</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Ver el trabajo</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>How I work</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Cómo trabajo</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>People · Systems · Futures</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Personas · Sistemas · Futuros</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Projects</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Proyectos</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Industries</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Industrias</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Clientes</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Years</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Años</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Years of work</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Años de trayectoria</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>01 — Highlights</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>01 — Destacados</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Selected work.</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Trabajo seleccionado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>02 — Practice</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>02 — Práctica</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Turning strategic ambiguity into operating models.</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Convertir la ambigüedad estratégica en modelos operativos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>03 — Principles</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>03 — Principios</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Six principles.</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Seis principios.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>One practice.</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Una práctica.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Read the approach</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Leer el enfoque</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>04 — Clients &amp; partners</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>04 — Clientes y aliados</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Who I've worked with.</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Con quién he trabajado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>05 — Next</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>05 — Siguiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>Let's design what comes next.</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Diseñemos lo que viene.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>Explore the work</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Explorar el trabajo</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>About me</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>Sobre mí</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>Write to me</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>Escríbeme</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>People.</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Personas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>Systems.</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>Sistemas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>Futures.</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>Futuros.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>HIPERNOVA | Design-Driven Transformation | By ©Jose Augusto Ocampo</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>HIPERNOVA | Transformación guiada por el diseño | Por ©Jose Augusto Ocampo</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>Work.</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>Trabajo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>Strategy, transformation and experience design across energy, financial services, retail, culture, education and the public sector — from science centers to operating models.</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>Estrategia, transformación y diseño de experiencias en energía, servicios financieros, retail, cultura, educación y sector público — desde centros de ciencia hasta modelos operativos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>Industry</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>Industria</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>grid</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>cuadrícula</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>index</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>índice</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>← Work / Index</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>← Trabajo / Índice</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>Client</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>Cliente</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>Año</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>Role</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>Rol</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>Country</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>País</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>Visit project</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>Ver proyecto</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>02 — Approach</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>02 — Enfoque</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>A question,</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>Una pregunta,</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>not a solution.</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>no una solución.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>01 — Method · System</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>01 — Método · Sistema</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>A cycle of four movements.</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>Un ciclo de cuatro movimientos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>OBSERVE</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>OBSERVAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>EXPAND</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>EXPANDIR</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>RECONFIGURE</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>RECONFIGURAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVATE</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>CYCLE</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>CICLO</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>Make visible what the system stopped seeing.</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>Hacer visible lo que el sistema dejó de ver.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>Bring in other perspectives, futures and questions.</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>Introducir otras perspectivas, futuros y preguntas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>Explore new relationships between the elements of the system.</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>Explorar nuevas relaciones entre los elementos del sistema.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>Turn possibilities into experiments, decisions and actions.</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>Convertir las posibilidades en experimentos, decisiones y acciones.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>02 — Six principles</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>02 — Seis principios</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>Reframe the problem.</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>Reformula el problema.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>Design the conditions.</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>Diseña las condiciones.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>Make change last.</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>Haz que el cambio perdure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>See it in practice</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>Verlo en la práctica</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>03 — About</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>03 — Sobre mí</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>Complexity is a condition</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>La complejidad es una condición</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>to be navigated.</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>que hay que navegar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>01 — Belief</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="inlineStr">
+        <is>
+          <t>01 — Convicción</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>02 — Experience</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>02 — Experiencia</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>Relevant experience.</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="inlineStr">
+        <is>
+          <t>Experiencia relevante.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>03 — Education</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>03 — Educación</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>Education.</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="inlineStr">
+        <is>
+          <t>Educación.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>04 — Certifications</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>04 — Certificaciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>Certifications.</t>
+        </is>
+      </c>
+      <c r="B77" s="2" t="inlineStr">
+        <is>
+          <t>Certificaciones.</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>05 — Disciplines</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>05 — Disciplinas</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="inlineStr">
+        <is>
+          <t>Disciplines &amp; frameworks.</t>
+        </is>
+      </c>
+      <c r="B79" s="2" t="inlineStr">
+        <is>
+          <t>Disciplinas y marcos de trabajo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>06 — Teaching</t>
+        </is>
+      </c>
+      <c r="B80" s="2" t="inlineStr">
+        <is>
+          <t>06 — Docencia</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="inlineStr">
+        <is>
+          <t>Teaching.</t>
+        </is>
+      </c>
+      <c r="B81" s="2" t="inlineStr">
+        <is>
+          <t>Docencia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>07 — Next</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>07 — Siguiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="inlineStr">
+        <is>
+          <t>Let's talk.</t>
+        </is>
+      </c>
+      <c r="B83" s="2" t="inlineStr">
+        <is>
+          <t>Hablemos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>Read my thinking</t>
+        </is>
+      </c>
+      <c r="B84" s="2" t="inlineStr">
+        <is>
+          <t>Leer mis ideas</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="inlineStr">
+        <is>
+          <t>04 — Thinking</t>
+        </is>
+      </c>
+      <c r="B85" s="2" t="inlineStr">
+        <is>
+          <t>04 — Pensamiento</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t>Thinking.</t>
+        </is>
+      </c>
+      <c r="B86" s="2" t="inlineStr">
+        <is>
+          <t>Pensamiento.</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="inlineStr">
+        <is>
+          <t>01 — Substack</t>
+        </is>
+      </c>
+      <c r="B87" s="2" t="inlineStr">
+        <is>
+          <t>01 — Substack</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="inlineStr">
+        <is>
+          <t>Read on Substack</t>
+        </is>
+      </c>
+      <c r="B88" s="2" t="inlineStr">
+        <is>
+          <t>Leer en Substack</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="inlineStr">
+        <is>
+          <t>Read on Substack ↗</t>
+        </is>
+      </c>
+      <c r="B89" s="2" t="inlineStr">
+        <is>
+          <t>Leer en Substack ↗</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="inlineStr">
+        <is>
+          <t>02 — Medium</t>
+        </is>
+      </c>
+      <c r="B90" s="2" t="inlineStr">
+        <is>
+          <t>02 — Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="inlineStr">
+        <is>
+          <t>03 — Publications</t>
+        </is>
+      </c>
+      <c r="B91" s="2" t="inlineStr">
+        <is>
+          <t>03 — Publicaciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="inlineStr">
+        <is>
+          <t>Publications.</t>
+        </is>
+      </c>
+      <c r="B92" s="2" t="inlineStr">
+        <is>
+          <t>Publicaciones.</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="inlineStr">
+        <is>
+          <t>Loading articles…</t>
+        </is>
+      </c>
+      <c r="B93" s="2" t="inlineStr">
+        <is>
+          <t>Cargando artículos…</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="inlineStr">
+        <is>
+          <t>Read them on Substack ↗</t>
+        </is>
+      </c>
+      <c r="B94" s="2" t="inlineStr">
+        <is>
+          <t>Léelos en Substack ↗</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="inlineStr">
+        <is>
+          <t>Couldn't load the articles right now.</t>
+        </is>
+      </c>
+      <c r="B95" s="2" t="inlineStr">
+        <is>
+          <t>No pude cargar los artículos en este momento.</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="inlineStr">
+        <is>
+          <t>404 — Signal lost</t>
+        </is>
+      </c>
+      <c r="B96" s="2" t="inlineStr">
+        <is>
+          <t>404 — Señal perdida</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="inlineStr">
+        <is>
+          <t>Not found.</t>
+        </is>
+      </c>
+      <c r="B97" s="2" t="inlineStr">
+        <is>
+          <t>No encontrado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="2" t="inlineStr">
+        <is>
+          <t>Back home</t>
+        </is>
+      </c>
+      <c r="B98" s="2" t="inlineStr">
+        <is>
+          <t>Volver al inicio</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="2" t="inlineStr">
+        <is>
+          <t>This case is available in English only for now.</t>
+        </is>
+      </c>
+      <c r="B99" s="2" t="inlineStr">
+        <is>
+          <t>Este caso está disponible solo en inglés por ahora.</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="2" t="inlineStr">
+        <is>
+          <t>CPG</t>
+        </is>
+      </c>
+      <c r="B100" s="2" t="inlineStr">
+        <is>
+          <t>Bienes de consumo</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="2" t="inlineStr">
+        <is>
+          <t>Culture &amp; Museums</t>
+        </is>
+      </c>
+      <c r="B101" s="2" t="inlineStr">
+        <is>
+          <t>Cultura y museos</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="2" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="B102" s="2" t="inlineStr">
+        <is>
+          <t>Educación</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="2" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="B103" s="2" t="inlineStr">
+        <is>
+          <t>Energía</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="2" t="inlineStr">
+        <is>
+          <t>Financial Services</t>
+        </is>
+      </c>
+      <c r="B104" s="2" t="inlineStr">
+        <is>
+          <t>Servicios financieros</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="2" t="inlineStr">
+        <is>
+          <t>Goverment / Public</t>
+        </is>
+      </c>
+      <c r="B105" s="2" t="inlineStr">
+        <is>
+          <t>Gobierno / Público</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="2" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="B106" s="2" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="2" t="inlineStr">
+        <is>
+          <t>Science - Research</t>
+        </is>
+      </c>
+      <c r="B107" s="2" t="inlineStr">
+        <is>
+          <t>Ciencia - Investigación</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="2" t="inlineStr">
+        <is>
+          <t>Third Sector / NGOs</t>
+        </is>
+      </c>
+      <c r="B108" s="2" t="inlineStr">
+        <is>
+          <t>Tercer sector / ONG</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="2" t="inlineStr">
+        <is>
+          <t>CX Strategy</t>
+        </is>
+      </c>
+      <c r="B109" s="2" t="inlineStr">
+        <is>
+          <t>Estrategia de CX</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="2" t="inlineStr">
+        <is>
+          <t>Creative space</t>
+        </is>
+      </c>
+      <c r="B110" s="2" t="inlineStr">
+        <is>
+          <t>Espacio creativo</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="2" t="inlineStr">
+        <is>
+          <t>Customer Experience and Innovation</t>
+        </is>
+      </c>
+      <c r="B111" s="2" t="inlineStr">
+        <is>
+          <t>Experiencia de cliente e innovación</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="2" t="inlineStr">
+        <is>
+          <t>Data visualization</t>
+        </is>
+      </c>
+      <c r="B112" s="2" t="inlineStr">
+        <is>
+          <t>Visualización de datos</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="2" t="inlineStr">
+        <is>
+          <t>Digital experience</t>
+        </is>
+      </c>
+      <c r="B113" s="2" t="inlineStr">
+        <is>
+          <t>Experiencia digital</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="2" t="inlineStr">
+        <is>
+          <t>Digital product</t>
+        </is>
+      </c>
+      <c r="B114" s="2" t="inlineStr">
+        <is>
+          <t>Producto digital</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="2" t="inlineStr">
+        <is>
+          <t>Exhibition</t>
+        </is>
+      </c>
+      <c r="B115" s="2" t="inlineStr">
+        <is>
+          <t>Exposición</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="2" t="inlineStr">
+        <is>
+          <t>Immersive media</t>
+        </is>
+      </c>
+      <c r="B116" s="2" t="inlineStr">
+        <is>
+          <t>Medios inmersivos</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="2" t="inlineStr">
+        <is>
+          <t>Interactives</t>
+        </is>
+      </c>
+      <c r="B117" s="2" t="inlineStr">
+        <is>
+          <t>Interactivos</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="2" t="inlineStr">
+        <is>
+          <t>Learning environment</t>
+        </is>
+      </c>
+      <c r="B118" s="2" t="inlineStr">
+        <is>
+          <t>Entorno de aprendizaje</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="2" t="inlineStr">
+        <is>
+          <t>Master Planning</t>
+        </is>
+      </c>
+      <c r="B119" s="2" t="inlineStr">
+        <is>
+          <t>Plan maestro</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="2" t="inlineStr">
+        <is>
+          <t>Policy making</t>
+        </is>
+      </c>
+      <c r="B120" s="2" t="inlineStr">
+        <is>
+          <t>Política pública</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="2" t="inlineStr">
+        <is>
+          <t>Product Design and Strategy</t>
+        </is>
+      </c>
+      <c r="B121" s="2" t="inlineStr">
+        <is>
+          <t>Diseño y estrategia de producto</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="2" t="inlineStr">
+        <is>
+          <t>Purpose-driven strategy</t>
+        </is>
+      </c>
+      <c r="B122" s="2" t="inlineStr">
+        <is>
+          <t>Estrategia con propósito</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="2" t="inlineStr">
+        <is>
+          <t>Science center</t>
+        </is>
+      </c>
+      <c r="B123" s="2" t="inlineStr">
+        <is>
+          <t>Centro de ciencia</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="2" t="inlineStr">
+        <is>
+          <t>Strategy</t>
+        </is>
+      </c>
+      <c r="B124" s="2" t="inlineStr">
+        <is>
+          <t>Estrategia</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="2" t="inlineStr">
+        <is>
+          <t>Sustainable Futures</t>
+        </is>
+      </c>
+      <c r="B125" s="2" t="inlineStr">
+        <is>
+          <t>Futuros sostenibles</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="2" t="inlineStr">
+        <is>
+          <t>Temporary exhibition</t>
+        </is>
+      </c>
+      <c r="B126" s="2" t="inlineStr">
+        <is>
+          <t>Exposición temporal</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="2" t="inlineStr">
+        <is>
+          <t>Transformation</t>
+        </is>
+      </c>
+      <c r="B127" s="2" t="inlineStr">
+        <is>
+          <t>Transformación</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="2" t="inlineStr">
+        <is>
+          <t>Traveling exhibition</t>
+        </is>
+      </c>
+      <c r="B128" s="2" t="inlineStr">
+        <is>
+          <t>Exposición itinerante</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="2" t="inlineStr">
+        <is>
+          <t>Ux</t>
+        </is>
+      </c>
+      <c r="B129" s="2" t="inlineStr">
+        <is>
+          <t>UX</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="2" t="inlineStr">
+        <is>
+          <t>Workshop / Bootcamp</t>
+        </is>
+      </c>
+      <c r="B130" s="2" t="inlineStr">
+        <is>
+          <t>Taller / Bootcamp</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="2" t="inlineStr">
+        <is>
+          <t>Author</t>
+        </is>
+      </c>
+      <c r="B131" s="2" t="inlineStr">
+        <is>
+          <t>Autor</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="2" t="inlineStr">
+        <is>
+          <t>Creative director</t>
+        </is>
+      </c>
+      <c r="B132" s="2" t="inlineStr">
+        <is>
+          <t>Director creativo</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="2" t="inlineStr">
+        <is>
+          <t>Exhibition Designer</t>
+        </is>
+      </c>
+      <c r="B133" s="2" t="inlineStr">
+        <is>
+          <t>Diseñador de exposiciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="2" t="inlineStr">
+        <is>
+          <t>Interior designer</t>
+        </is>
+      </c>
+      <c r="B134" s="2" t="inlineStr">
+        <is>
+          <t>Diseñador de interiores</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="2" t="inlineStr">
+        <is>
+          <t>Project leader</t>
+        </is>
+      </c>
+      <c r="B135" s="2" t="inlineStr">
+        <is>
+          <t>Líder de proyecto</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="2" t="inlineStr">
+        <is>
+          <t>Researcher</t>
+        </is>
+      </c>
+      <c r="B136" s="2" t="inlineStr">
+        <is>
+          <t>Investigador</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="2" t="inlineStr">
+        <is>
+          <t>Senior Exhibition Designer</t>
+        </is>
+      </c>
+      <c r="B137" s="2" t="inlineStr">
+        <is>
+          <t>Diseñador sénior de exposiciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="2" t="inlineStr">
+        <is>
+          <t>Senior designer</t>
+        </is>
+      </c>
+      <c r="B138" s="2" t="inlineStr">
+        <is>
+          <t>Diseñador sénior</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="2" t="inlineStr">
+        <is>
+          <t>Strategic Design &amp; CX Lead</t>
+        </is>
+      </c>
+      <c r="B139" s="2" t="inlineStr">
+        <is>
+          <t>Líder de diseño estratégico y CX</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="2" t="inlineStr">
+        <is>
+          <t>Strategic Design Consultant</t>
+        </is>
+      </c>
+      <c r="B140" s="2" t="inlineStr">
+        <is>
+          <t>Consultor de diseño estratégico</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="2" t="inlineStr">
+        <is>
+          <t>Strategy Consulting Director</t>
+        </is>
+      </c>
+      <c r="B141" s="2" t="inlineStr">
+        <is>
+          <t>Director de consultoría estratégica</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="2" t="inlineStr">
+        <is>
+          <t>Volunteer</t>
+        </is>
+      </c>
+      <c r="B142" s="2" t="inlineStr">
+        <is>
+          <t>Voluntario</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Spanish bodies for all 47 cases
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/database/hipernova-portafolio-db.xlsx
+++ b/database/hipernova-portafolio-db.xlsx
@@ -654,7 +654,22 @@
         </is>
       </c>
       <c r="T2" s="2" t="inlineStr"/>
-      <c r="U2" s="2" t="inlineStr"/>
+      <c r="U2" s="2" t="inlineStr">
+        <is>
+          <t>&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;01 —&lt;/span&gt;Situación — El desafío&lt;/h2&gt;
+&lt;p&gt;El proceso de cálculo de tarifas OPEX de Ecopetrol dependía en gran medida del trabajo manual, de fuentes de datos fragmentadas, de hojas de cálculo individuales y de criterios de cálculo distintos entre equipos. Esto hacía que el proceso fuera más difícil de trazar, estandarizar y escalar, y limitaba el tiempo que los analistas podían dedicar a análisis de mayor valor. El desafío era repensar una parte crítica del proceso y explorar cómo una única herramienta, más confiable, podía conectar datos, estandarizar cálculos, fortalecer la trazabilidad y apoyar mejor los procesos de Portafolio, Reservas y FMV.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;02 —&lt;/span&gt;Tarea — Mi rol&lt;/h2&gt;
+&lt;p&gt;Lideré el proyecto de principio a fin, dirigiendo al equipo multidisciplinario responsable de la investigación, la síntesis, la facilitación, el prototipado y la definición estratégica. Diseñé y facilité el Design Sprint de tres días con Ecopetrol, guiando a un grupo de más de 20 participantes a través del encuadre del problema, la priorización, la ideación, el desarrollo de conceptos y la validación. También lideré la integración de las necesidades de los usuarios, los requerimientos del proceso, las consideraciones de gobernanza y la factibilidad técnica en una solución coherente y una hoja de ruta de implementación.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;03 —&lt;/span&gt;Acción — El proceso&lt;/h2&gt;
+&lt;p&gt;&lt;strong&gt;Inmersión y mapeo del proceso.&lt;/strong&gt; Lideré al equipo en una fase inicial de planeación que incluyó 13 entrevistas con stakeholders de Ecopetrol, un mapeo detallado del proceso de cálculo de tarifas OPEX y una revisión de las principales herramientas involucradas, entre ellas SAP, VALNAV, Spotfire y Planning Space. Esto nos permitió identificar las principales barreras en torno al trabajo manual, el acceso a los datos, la trazabilidad, la consistencia metodológica, la escalabilidad y la ausencia de una única fuente de verdad.&lt;/p&gt;
+&lt;p&gt;&lt;strong&gt;Design Sprint y encuadre del problema.&lt;/strong&gt; Facilité un Design Sprint de tres días en Bogotá con más de 20 participantes de Ecopetrol. El primer día alineamos al grupo en torno al desafío, definimos la meta de largo plazo y el foco del Sprint, exploramos referentes relevantes y generamos los primeros conceptos. Esto dio como resultado cinco módulos de solución priorizados: precomparación, normalización, escalamiento, visualización de tarifas y reportería.&lt;/p&gt;
+&lt;p&gt;&lt;strong&gt;Co-diseño y prototipado.&lt;/strong&gt; Guié al equipo en el desarrollo detallado de los cinco módulos, definiendo flujos, lógica de interacción y decisiones clave de diseño. En paralelo, trabajamos con el equipo de tecnología en consideraciones de factibilidad y arquitectura, mientras otra línea de trabajo exploraba la gobernanza del proceso, los roles, la continuidad del conocimiento y la gestión de datos. Estos insumos se consolidaron en un prototipo de alta fidelidad que representaba una experiencia de punta a punta más integrada y trazable.&lt;/p&gt;
+&lt;p&gt;&lt;strong&gt;Validación con stakeholders.&lt;/strong&gt; El último día probamos el prototipo con stakeholders clave de distintas áreas de Ecopetrol y usamos sus comentarios para refinar la solución. La validación reforzó el valor de reducir el esfuerzo operativo para que los analistas pudieran dedicar más tiempo a cuestionar supuestos, trabajar más cerca de la operación y fortalecer el aseguramiento del proceso, en lugar de gestionar consolidaciones manuales.&lt;/p&gt;
+&lt;p&gt;&lt;strong&gt;Del prototipo a la implementación.&lt;/strong&gt; Después del Sprint, lideré la consolidación del prototipo final, el backlog y la hoja de ruta de implementación. La solución se estructuró en tres olas: un MVP centrado en el flujo central de cálculo, una expansión funcional que incluía visualización y reportería, y una fase complementaria que introducía capacidades asistidas por IA y mayor automatización.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;04 —&lt;/span&gt;Resultado&lt;/h2&gt;
+&lt;p&gt;El Sprint transformó un desafío operativo complejo en un concepto de producto validado, un backlog priorizado y un camino claro hacia la implementación. El equipo se alineó en torno a una visión compartida de un proceso más estandarizado, trazable y escalable, con cinco módulos centrales y más de 20 funcionalidades clave definidas durante el proyecto. Lo más importante es que el trabajo replanteó la automatización no solo como una forma de reducir el esfuerzo manual, sino como un medio para liberar a los analistas y que se concentren en el criterio, la comprensión operativa y una toma de decisiones más sólida.&lt;/p&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -747,7 +762,23 @@
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr"/>
-      <c r="U3" s="2" t="inlineStr"/>
+      <c r="U3" s="2" t="inlineStr">
+        <is>
+          <t>&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;01 —&lt;/span&gt;Situación — El desafío&lt;/h2&gt;
+&lt;p&gt;MTS LATAM había construido una posición sólida administrando activos inmobiliarios en cinco mercados latinoamericanos, respaldada por décadas de experiencia operativa, una amplia base de clientes institucionales y millones de metros cuadrados bajo administración. Sin embargo, buena parte de esa experiencia permanecía invisible: los clientes reconocían a MTS principalmente por su capacidad de ejecución, mientras que su conocimiento estratégico, sus datos operativos propios y su portafolio más amplio de servicios eran menos visibles. El desafío era aclarar dónde tenía la compañía un derecho a ganar defendible y traducir sus fortalezas existentes en un camino enfocado de crecimiento a largo plazo.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;02 —&lt;/span&gt;Tarea — Mi rol&lt;/h2&gt;
+&lt;p&gt;Participé en una inmersión estratégica de cinco semanas diseñada para ayudar al liderazgo de MTS a tomar decisiones más claras sobre dónde jugar, cómo ganar y qué capacidades se requerirían para sostener su siguiente etapa de crecimiento. Mi trabajo conectó la investigación, las perspectivas del liderazgo, la estrategia de negocio, el posicionamiento de marca y las implicaciones organizacionales en un marco estratégico coherente. También ayudé a traducir esas decisiones en un sistema que pudiera guiar la priorización entre mercados, capacidades y activación de marketing.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;03 —&lt;/span&gt;Acción&lt;/h2&gt;
+&lt;p&gt;&lt;strong&gt;Descubrimiento y diagnóstico estratégico.&lt;/strong&gt; Empezamos revisando los planes comerciales y de marketing internos, los benchmarks de la competencia y los materiales estratégicos existentes. Esto se complementó con entrevistas a profundidad con líderes de la gerencia ejecutiva y de las áreas comercial, de operaciones, de talento y de administración de activos, lo que nos permitió sacar a la luz tensiones recurrentes en torno al posicionamiento, el crecimiento, los hábitos organizacionales, la tecnología y las relaciones con los clientes.&lt;/p&gt;
+&lt;p&gt;&lt;strong&gt;Cocreación con el liderazgo.&lt;/strong&gt; Reunimos al equipo de liderazgo de LATAM en un taller de cocreación de un día completo, seguido de sesiones de trabajo enfocadas con las áreas comercial, de operaciones, de talento, de marketing y otras funciones del negocio. En lugar de tratar el proyecto como un diagnóstico externo, el proceso usó la propia experiencia de la organización para convertir las tensiones en decisiones estratégicas explícitas y generar una apropiación compartida de la dirección.&lt;/p&gt;
+&lt;p&gt;&lt;strong&gt;Decisiones estratégicas y posicionamiento.&lt;/strong&gt; El trabajo aclaró los perfiles de clientes y los mercados prioritarios, las áreas que la compañía debía evitar deliberadamente y una posición competitiva diferenciada: ni un operador tradicional ni una firma de asesoría distante, sino un &lt;strong&gt;operador estratégico&lt;/strong&gt; que combina la ejecución con inteligencia para la toma de decisiones. También conectamos esta posición con los datos operativos y la plataforma tecnológica de MTS, replanteándolos: de infraestructura de apoyo a evidencia de una ventaja competitiva más difícil de replicar.&lt;/p&gt;
+&lt;p&gt;&lt;strong&gt;Diseño del sistema de crecimiento.&lt;/strong&gt; Sintetizamos la estrategia en un &lt;strong&gt;Property Intelligence Flywheel&lt;/strong&gt; de cinco partes: proteger la base operativa, transformar los datos en inteligencia, usar esa inteligencia para guiar las decisiones, capturar el valor creado y ampliar el alcance de la compañía. Cuatro aceleradores en paralelo —datos más profundos, costos de cambio crecientes, reputación acumulada y capital relacional institucionalizado— mostraron cómo el sistema podía fortalecerse con el tiempo en lugar de operar como un plan estratégico lineal.&lt;/p&gt;
+&lt;p&gt;&lt;strong&gt;De la estrategia a la activación.&lt;/strong&gt; Finalmente, tradujimos el modelo en tres horizontes: fortalecer el núcleo establecido, expandirse en mercados validados y tratar las oportunidades de nuevos mercados como experimentos disciplinados. También revisamos el plan de marketing existente frente a la nueva estrategia e identificamos brechas en las prioridades geográficas, la segmentación de audiencias, la arquitectura narrativa, la activación tecnológica, la medición y la gobernanza. Esto creó un puente más claro entre la intención estratégica y la ejecución.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;04 —&lt;/span&gt;Resultado — El impacto&lt;/h2&gt;
+&lt;p&gt;La Connected Compass le dio a MTS un lenguaje estratégico compartido para conectar las operaciones, el conocimiento propio, la marca, las prioridades de mercado y las capacidades organizacionales. En lugar de perseguir el crecimiento como un conjunto de iniciativas desconectadas, el liderazgo ganó un sistema coherente para decidir qué fortalecer ahora, qué expandir después y qué explorar con mayor disciplina.&lt;/p&gt;
+&lt;p&gt;El trabajo también replanteó uno de los activos más importantes de la compañía: su huella operativa no era simplemente evidencia de escala, sino la base de una ventaja de inteligencia capaz de informar tanto las decisiones de los clientes como la diferenciación futura.&lt;/p&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -839,7 +870,22 @@
         </is>
       </c>
       <c r="T4" s="2" t="inlineStr"/>
-      <c r="U4" s="2" t="inlineStr"/>
+      <c r="U4" s="2" t="inlineStr">
+        <is>
+          <t>&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;01 —&lt;/span&gt;Contexto&lt;/h2&gt;
+&lt;p&gt;En marzo de 2025, Ecopetrol se asoció con The Cocktail para realizar un taller de gerencia de dos días en Bucaramanga para los líderes de la Vicepresidencia de Tecnología e Innovación (VTI). El taller buscaba fortalecer la cohesión del equipo y definir prioridades estratégicas alineadas con la Estrategia 2040 de Ecopetrol. Dados los desafíos de la transición energética y la caída de los retornos del sector, fortalecer la posición de la VTI como motor clave de la transformación digital y tecnológica se volvió esencial.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;02 —&lt;/span&gt;El desafío&lt;/h2&gt;
+&lt;p&gt;El principal desafío era alinear las prioridades de la VTI con los objetivos estratégicos del Grupo Ecopetrol, abordando al mismo tiempo la baja rentabilidad, la desconfianza interna y la desconexión entre las unidades de negocio y tecnología. La VTI necesitaba posicionarse como un socio estratégico: uno capaz de anticipar desafíos, entregar valor tangible y marcar referentes en ciencia, tecnología e innovación.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;03 —&lt;/span&gt;El proceso&lt;/h2&gt;
+&lt;p&gt;El taller siguió una metodología de tres fases: planeación, ejecución y reporte. Durante la planeación, las entrevistas con stakeholders clave sirvieron de base para diseñar actividades interactivas a la medida de las necesidades de la VTI. A lo largo de dos días, los participantes realizaron ejercicios para alinearse en el propósito de la VTI, identificar desafíos transversales y cocrear soluciones.&lt;/p&gt;
+&lt;ul&gt;&lt;li&gt;El primer día se centró en comprender el contexto estratégico de Ecopetrol, definir la visión de la VTI y mapear las barreras en cinco áreas de enfoque estratégico.&lt;/li&gt;&lt;li&gt;El segundo día, estas barreras se agruparon en cuatro "territorios de oportunidad", como mejorar la confianza en la VTI y potenciar las sinergias entre negocio y tecnología.&lt;/li&gt;&lt;/ul&gt;
+&lt;p&gt;Luego, los participantes desarrollaron soluciones accionables y líneas de acción detalladas para abordar estas oportunidades. La fase final consistió en documentar los resultados, incluida una hoja de ruta de implementación y aprendizajes para orientar acciones futuras.&lt;/p&gt;
+&lt;ul&gt;&lt;li&gt;Realizamos entrevistas con stakeholders clave de Ecopetrol para afinar la metodología del taller.&lt;/li&gt;&lt;li&gt;Diseñamos y preparamos materiales del taller a la medida.&lt;/li&gt;&lt;li&gt;Facilitamos dos días de sesiones colaborativas presenciales con más de 17 gerentes y líderes.&lt;/li&gt;&lt;li&gt;Identificamos brechas organizacionales y mapeamos 17 áreas de oportunidad.&lt;/li&gt;&lt;li&gt;Consolidamos 4 territorios estratégicos de oportunidad de carácter transversal.&lt;/li&gt;&lt;li&gt;Cocreamos soluciones e iniciativas para cada área de oportunidad.&lt;/li&gt;&lt;li&gt;Definimos 12 líneas de acción con fichas de planeación detalladas para guiar los esfuerzos de la VTI en 2025.&lt;/li&gt;&lt;/ul&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;04 —&lt;/span&gt;El impacto&lt;/h2&gt;
+&lt;p&gt;El taller dio como resultado una articulación clara del propósito de la VTI: aprovechar la ciencia, la tecnología y la innovación para abordar los desafíos más críticos de Ecopetrol, impulsando al mismo tiempo la eficiencia, la competitividad y la sostenibilidad.&lt;/p&gt;
+&lt;p&gt;Se identificaron cuatro territorios estratégicos de oportunidad, junto con sus líneas de acción correspondientes, como &lt;strong&gt;mejorar la gobernanza, fomentar la colaboración y optimizar la gestión del talento.&lt;/strong&gt; Estos resultados sentaron las bases para que la VTI se convierta en un socio más creíble, integrado y alineado estratégicamente dentro de Ecopetrol. Además, la iniciativa resaltó la importancia de cerrar las brechas entre negocio y tecnología, asegurando que la VTI evolucione de proveedor de servicios a habilitador estratégico en el camino de transición energética de Ecopetrol.&lt;/p&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -924,7 +970,19 @@
         </is>
       </c>
       <c r="T5" s="2" t="inlineStr"/>
-      <c r="U5" s="2" t="inlineStr"/>
+      <c r="U5" s="2" t="inlineStr">
+        <is>
+          <t>&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;01 —&lt;/span&gt;El contexto&lt;/h2&gt;
+&lt;p&gt;En febrero de 2025, Ecopetrol, en colaboración con The Cocktail, realizó un taller participativo para apoyar a la Gerencia de Innovación y Portafolio (GIP) en la alineación de su planeación estratégica con la visión 2040 de Ecopetrol. La iniciativa reunió a los tres departamentos centrales —Planeación y Portafolio, Arquitectura Tecnológica e Innovación— para definir colectivamente las capacidades críticas, reflexionar sobre sus roles y proponer una hoja de ruta para activar esas capacidades y potenciar la transformación tecnológica y la transición energética de Ecopetrol.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;02 —&lt;/span&gt;El desafío&lt;/h2&gt;
+&lt;p&gt;La GIP enfrentaba varios desafíos estratégicos: alinear sus iniciativas con la Estrategia 2040 de Ecopetrol, derribar los silos entre departamentos, identificar y fortalecer las capacidades críticas, y fomentar un propósito compartido. La fragmentación interna, las barreras burocráticas y la resistencia al cambio limitaban la efectividad y la agilidad necesarias para impulsar la innovación en toda la organización.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;03 —&lt;/span&gt;El proceso&lt;/h2&gt;
+&lt;p&gt;El taller siguió una metodología estructurada de tres fases: planeación, ejecución y reporte. Durante la planeación, las entrevistas con stakeholders y una revisión de los procesos existentes sirvieron de base para diseñar la agenda y los materiales del taller. La sesión de un día comenzó con una introducción a los roles de cada departamento, seguida de ejercicios colaborativos para definir el propósito de la GIP y cocrear sus capacidades centrales. Los participantes identificaron ocho capacidades críticas, como la visión de futuro, la exploración tecnológica y la conexión con el ecosistema, y analizaron sus habilitadores y barreras. La fase final consistió en documentar los resultados, incluidos el propósito definido, las capacidades y las prioridades iniciales, y en preparar recomendaciones para los próximos pasos.&lt;/p&gt;
+&lt;ul&gt;&lt;li&gt;Realizamos sesiones de alineación y de definición de expectativas con los stakeholders.&lt;/li&gt;&lt;li&gt;Revisamos los procesos actuales y las oportunidades de mejora.&lt;/li&gt;&lt;li&gt;Facilitamos un taller de cocreación con más de 50 participantes de los tres departamentos de la GIP.&lt;/li&gt;&lt;li&gt;Definimos un propósito unificado y cinco capacidades estratégicas clave para la GIP.&lt;/li&gt;&lt;li&gt;Mapeamos los habilitadores y las barreras para el desarrollo de las capacidades.&lt;/li&gt;&lt;/ul&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;04 —&lt;/span&gt;El impacto&lt;/h2&gt;
+&lt;p&gt;El taller dio como resultado una articulación clara del propósito de la GIP: orquestar e impulsar la innovación y la transformación tecnológica en todo Ecopetrol, contribuyendo a un futuro energético más sostenible, competitivo y próspero. Se identificaron ocho capacidades críticas, que ofrecen una base para el marco estratégico de la GIP. La sesión también puso de relieve barreras clave, como la operación en silos y la resistencia al cambio, y subrayó la necesidad de cambios culturales para fomentar la innovación. De cara al futuro, los resultados guiarán el desarrollo de prioridades estratégicas, hojas de ruta y modelos de activación para asegurar la alineación de la GIP con las metas 2040 de Ecopetrol, maximizando el valor para los stakeholders.&lt;/p&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -1000,7 +1058,18 @@
       </c>
       <c r="S6" s="2" t="inlineStr"/>
       <c r="T6" s="2" t="inlineStr"/>
-      <c r="U6" s="2" t="inlineStr"/>
+      <c r="U6" s="2" t="inlineStr">
+        <is>
+          <t>&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;01 —&lt;/span&gt;El contexto&lt;/h2&gt;
+&lt;p&gt;Itaú Colombia atraviesa un giro estratégico para convertirse en un banco "future-ready", donde la digitalización, la personalización y la competitividad son centrales para el crecimiento. Para respaldar esta visión, la organización emprendió un proceso de diagnóstico integral para evaluar su experiencia de cliente (CX) actual y definir una hoja de ruta para su transformación. Participé en este recorrido como CX Lead, apoyando el diseño estratégico y la coordinación de este esfuerzo de transformación.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;02 —&lt;/span&gt;El desafío&lt;/h2&gt;
+&lt;p&gt;A pesar de su sólido posicionamiento en la región, Itaú iba rezagado frente a competidores locales e internacionales en experiencia digital, particularmente en banca de personas. La inestabilidad de la app móvil, los problemas de UX y la falta de funcionalidades clave afectaban la satisfacción de los clientes. El desafío central era construir un modelo de transformación que integrara las necesidades del negocio, las expectativas de los clientes y los aprendizajes de la competencia para impulsar una estrategia de CX diferenciada.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;03 —&lt;/span&gt;El proceso&lt;/h2&gt;
+&lt;ul&gt;&lt;li&gt;Realizamos un diagnóstico estratégico de los productos digitales de Itaú y de su ecosistema de experiencia actual (AS-IS).&lt;/li&gt;&lt;li&gt;Hicimos un benchmark de más de 30 actores financieros (bancos tradicionales, fintechs y neobancos).&lt;/li&gt;&lt;li&gt;Definimos drivers de experiencia por segmento (personas y corporativo) para identificar oportunidades.&lt;/li&gt;&lt;li&gt;Mapeamos las brechas en el desempeño de CX y las contrastamos con las mejores prácticas y las necesidades de los usuarios.&lt;/li&gt;&lt;li&gt;Creamos un modelo de transformación de CX que integra personalización, multiexperiencia, agilidad e innovación.&lt;/li&gt;&lt;li&gt;Diseñamos una hoja de ruta orientada al futuro, basada en oportunidades estratégicas y prioridades del negocio.&lt;/li&gt;&lt;li&gt;Entregamos recomendaciones basadas en evidencia para la evolución de la experiencia en todos los canales y puntos de contacto.&lt;/li&gt;&lt;/ul&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;04 —&lt;/span&gt;Mi rol&lt;/h2&gt;
+&lt;p&gt;Como CX Lead, mi rol fue acompañar y guiar al equipo durante la definición estratégica de la nueva experiencia de cliente de Itaú. Brindé coaching al diseñador interno para fortalecer su liderazgo y su pensamiento estratégico, y aporté marcos de experiencia, casos inspiradores y benchmarks de la competencia para enriquecer el proceso de diseño. Apoyé la identificación de los drivers de experiencia y la construcción de un modelo de transformación que considerara el negocio, al cliente y el panorama competitivo. Mi participación también fue clave para alinear a los equipos multifuncionales —negocio, UX, tecnología— en torno a una visión compartida, y para dar forma a una narrativa clara que conectara los desafíos actuales con el estado futuro deseado para la experiencia de Itaú.&lt;/p&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -1105,7 +1174,35 @@
         </is>
       </c>
       <c r="T7" s="2" t="inlineStr"/>
-      <c r="U7" s="2" t="inlineStr"/>
+      <c r="U7" s="2" t="inlineStr">
+        <is>
+          <t>&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;01 —&lt;/span&gt;Situación&lt;/h2&gt;
+&lt;p&gt;Ecopetrol enfrentaba desafíos de transformación sin precedentes en el sector energético global, que exigían una diversificación estratégica hacia negocios de electrones y moléculas de bajas emisiones. Las definiciones estratégicas recientes de la compañía buscaban convertirla en un grupo empresarial enfocado en la rentabilidad, la eficiencia, el crecimiento y la sostenibilidad, lo que demanda enfoques cada vez más robustos para anticipar los cambios tecnológicos y de mercado.&lt;/p&gt;
+&lt;p&gt;La VTI (Vicepresidencia de Tecnología e Innovación) tenía un rol estratégico para el futuro de la compañía, pero necesitaba fortalecer sus capacidades de prospectiva y vigilancia tecnológica para conectar mejor las tendencias emergentes con las decisiones estratégicas de largo plazo.&lt;/p&gt;
+&lt;p&gt;El diagnóstico reveló una posición "vulnerable" de la VTI —operando en un entorno de alta volatilidad pero con una preparación insuficiente para el futuro—, caracterizada por una gobernanza fragmentada, mentalidades reactivas de corto plazo y una planeación estratégica desconectada entre la estrategia corporativa, las hojas de ruta tecnológicas y la gestión del portafolio.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;02 —&lt;/span&gt;Tarea&lt;/h2&gt;
+&lt;p&gt;Lideré el diseño y desarrollo de un modelo de prospectiva de CT+I (Ciencia, Tecnología e Innovación) accionable, que transformaría a la VTI en un habilitador clave de la estrategia de Ciencia y Tecnología de Ecopetrol. Mi rol abarcó la facilitación estratégica a lo largo de tres fases: inmersión y diagnóstico, definición colaborativa de la intención, y especificación detallada del modelo con su hoja de ruta de implementación.&lt;/p&gt;
+&lt;p&gt;Trabajando junto a equipos multifuncionales de la VTI, el ICPET y las unidades de negocio, orquesté un proceso colaborativo de transformación que involucró a más de 60 stakeholders mediante encuestas, entrevistas y talleres intensivos de cocreación, con el fin de institucionalizar capacidades sistemáticas de anticipación tecnológica y establecer un propósito transformador compartido.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;03 —&lt;/span&gt;Acción&lt;/h2&gt;
+&lt;p&gt;Primero, realizamos un análisis integral de las prácticas de prospectiva existentes mediante un diagnóstico multimétodo que combinó entrevistas con stakeholders, análisis documental y una encuesta organizacional.&lt;/p&gt;
+&lt;p&gt;Las más de 16 entrevistas a profundidad abarcaron roles clave del liderazgo de la VTI, entre ellos planeación y gestión de portafolio, arquitectura digital, equipos de innovación y socios de negocio, además de voces estratégicas del ICPET y de la estrategia corporativa. Estas conversaciones revelaron enfoques fragmentados de anticipación tecnológica, con cada área operando metodologías y tiempos distintos, sin una coordinación sistemática.&lt;/p&gt;
+&lt;p&gt;El análisis de más de 15 documentos estratégicos abarcó marcos de estrategia corporativa, hojas de ruta tecnológicas existentes, portafolios de innovación, planes quinquenales y ejercicios de prospectiva previos, y dejó al descubierto brechas significativas entre la intención estratégica y la ejecución operativa. Lo complementamos con una encuesta integral a 44 participantes de toda la organización para cuantificar las percepciones sobre las capacidades actuales de prospectiva e identificar las áreas prioritarias de mejora.&lt;/p&gt;
+&lt;p&gt;Esta síntesis diagnóstica reveló cinco territorios de oportunidad críticos que requerían intervención: conexión estratégica (vincular la estrategia corporativa con la ejecución tecnológica), gobernanza integrada (superar los silos organizacionales), inteligencia accionable (transformar datos dispersos en insights estratégicos), métodos prospectivos (institucionalizar prácticas sistemáticas de prospectiva) y mentalidades anticipatorias (fomentar una cultura orientada al futuro).&lt;/p&gt;
+&lt;p&gt;En paralelo, hicimos un benchmarking sistemático de 14 líderes de la industria en energía (Repsol, BP, Shell, Petrobras, TotalEnergies, Chevron), energías renovables (Iberdrola, Moeve, Oklo) y otros sectores (NVIDIA, BASF, Enel, Bosch, Siemens), evaluando seis capacidades centrales de prospectiva: liderazgo y gobernanza, inteligencia del entorno, exploración del futuro, visión y dirección estratégica, acción y experimentación, y cultura prospectiva. Este análisis mostró que las compañías líderes institucionalizan la prospectiva mediante mandatos al nivel del CEO, escaneo sistemático del entorno, desarrollo colaborativo de escenarios y mecanismos formales de experimentación, lo que pone de relieve la actual posición "vulnerable" de la VTI, que requiere una intervención estructurada en cinco territorios de oportunidad.&lt;/p&gt;
+&lt;p&gt;Creamos y facilitamos un taller intensivo de cocreación de un día en Bogotá, que reunió a 12 participantes de la VTI, las unidades de negocio y las áreas estratégicas. La sesión comenzó con un encuadre inspirador sobre el propósito organizacional como "actos de esperanza que abren realidades futuras". Mediante dinámicas colaborativas estructuradas, cocreamos el propósito transformador de FARO:&lt;/p&gt;
+&lt;blockquote class="c-quote"&gt;"Somos el Faro CT+I de inteligencia prospectiva que conecta el presente con el futuro tecnológico, habilitando al Grupo Empresarial para anticipar, interpretar y actuar en entornos de alta incertidumbre."&lt;/blockquote&gt;
+&lt;p&gt;Guiamos a los participantes en una exploración sistemática de cinco territorios estratégicos, generando 21 iniciativas accionables a lo largo de las dimensiones de oportunidad. Aplicamos la metodología "Transition by Design" para crear una hoja de ruta evolutiva de tres versiones (V1-V3), que parte de las áreas de influencia centrales de la VTI y se expande progresivamente. Facilitamos sesiones colaborativas de priorización, con votación por impacto y por stakeholders, para identificar las iniciativas de mayor valor para implementar de inmediato.&lt;/p&gt;
+&lt;p&gt;Luego, diseñamos un modelo operativo integral estructurado en cinco fases integradas: Enmarcar, Explorar, Proyectar, Definir y Transformar. Desarrollamos especificaciones detalladas para 10 iniciativas prioritarias en los distintos territorios estratégicos, cada una con sus requerimientos de implementación, equipos responsables, dependencias y métricas de éxito. Creamos una estructura de gobernanza que integra a los Business Partners, el ICPET y las unidades de negocio, con roles y procesos de toma de decisiones claros.&lt;/p&gt;
+&lt;p&gt;Adicionalmente, desarrollamos un completo Toolkit de Prospectiva FARO CT+I: una guía práctica que traduce el modelo teórico en metodologías accionables. Este playbook de más de 50 páginas estructura 20 herramientas específicas a lo largo de las cinco fases del modelo, desde el mapeo de stakeholders y el horizon scanning hasta la creación de escenarios y los design sprints, cada una con instrucciones paso a paso, plantillas y recursos descargables. El toolkit sirve como recurso interno de la VTI para el desarrollo de capacidades, y permite que los equipos apliquen las metodologías de prospectiva de manera sistemática y reduzcan su dependencia de consultores externos.&lt;/p&gt;
+&lt;p&gt;Finalmente, establecimos una hoja de ruta priorizada que se enfoca en las iniciativas de mayor impacto: un modelo integrado de estrategia-tecnología para sincronizar la estrategia corporativa con la ejecución tecnológica, un Radar Ejecutivo para la síntesis continua de inteligencia y un Centro de Inteligencia para democratizar el acceso a fuentes de información especializadas. Diseñamos un sistema de medición (FARO Impact Measurement) para demostrar el valor estratégico y guiar la mejora continua.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;04 —&lt;/span&gt;Resultado&lt;/h2&gt;
+&lt;p&gt;Entregamos un modelo operativo integral de prospectiva que posiciona a la VTI como el centro de anticipación tecnológica estratégica de Ecopetrol, con un alineamiento demostrado de los stakeholders y una ruta clara de implementación. El modelo FARO ofrece una metodología sistemática para conectar la visión estratégica de largo plazo con la ejecución tecnológica, con una gobernanza estructurada, una generación continua de inteligencia y capacidades prospectivas institucionalizadas.&lt;/p&gt;
+&lt;p&gt;El proceso colaborativo generó 10 iniciativas accionables organizadas en cinco territorios estratégicos, con una priorización clara y una hoja de ruta evolutiva que abarca un modelo mínimo viable centrado en tecnologías digitales, un modelo ampliado que incorpora tecnologías emergentes y un modelo consolidado que cubre todas las tecnologías críticas del Grupo. Se estableció una estructura de gobernanza con roles definidos entre los equipos de planeación, arquitectura e innovación, respaldada por sistemas de medición e iniciativas de transformación cultural.&lt;/p&gt;
+&lt;p&gt;El enfoque de cocreación aseguró la apropiación de la organización mediante la definición colaborativa del propósito, las prioridades y el enfoque de implementación. Surgieron seis grandes reflexiones:&lt;/p&gt;
+&lt;ul&gt;&lt;li&gt;Necesidad de una conexión más fuerte entre tecnología y estrategia&lt;/li&gt;&lt;li&gt;Evolución de una inteligencia reactiva a una continua&lt;/li&gt;&lt;li&gt;Establecimiento de un mandato claro que supere la fragmentación&lt;/li&gt;&lt;li&gt;Espacios de aprendizaje colaborativo&lt;/li&gt;&lt;li&gt;Resultados tempranos tangibles que permiten escalar&lt;/li&gt;&lt;li&gt;Capacidades internas fortalecidas mediante marcos comunes&lt;/li&gt;&lt;/ul&gt;
+&lt;p&gt;&lt;strong&gt;Aprendizaje clave:&lt;/strong&gt; Una transformación exitosa en prospectiva tecnológica requiere intervenir simultáneamente en la alineación estratégica, la estructura de gobernanza, los sistemas de inteligencia, los marcos metodológicos y el cambio cultural, lo cual se logra mediante una cocreación colaborativa que construye apropiación compartida y una ruta evolutiva clara desde las competencias centrales hacia capacidades integrales de anticipación.&lt;/p&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -1196,7 +1293,21 @@
         </is>
       </c>
       <c r="T8" s="2" t="inlineStr"/>
-      <c r="U8" s="2" t="inlineStr"/>
+      <c r="U8" s="2" t="inlineStr">
+        <is>
+          <t>&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;01 —&lt;/span&gt;Situación&lt;/h2&gt;
+&lt;p&gt;La Cámara de Comercio de Bogotá (CCB) es una de las instituciones empresariales más influyentes de Colombia y atiende a más de 400.000 empresarios y compañías de la región de Bogotá. Desempeña un papel central en la formalización empresarial, el desarrollo económico y la colaboración público-privada. Con el tiempo, la CCB había desarrollado más de 15 activos digitales —entre plataformas, sitios web y micrositios—, cada uno gestionado de forma independiente por distintos departamentos o proveedores. Esto resultó en una experiencia de usuario fragmentada, esfuerzos duplicados y una capacidad limitada para evolucionar estratégicamente. En el contexto de una transformación institucional más amplia, la CCB se propuso unificar su ecosistema digital en torno a una visión centrada en el usuario: mejorando el acceso, fortaleciendo la coherencia de marca y aumentando la eficiencia operativa.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;02 —&lt;/span&gt;Tarea&lt;/h2&gt;
+&lt;p&gt;Supervisé el proyecto de principio a fin, desde la elaboración de la propuesta comercial y el pitch hasta el logro de la aprobación de la alta dirección. Bajo mi liderazgo, un equipo multidisciplinario lideró la investigación, la estrategia de experiencia y la estructuración de la plataforma. Asumí un rol práctico en las fases críticas: consolidé personalmente el modelo de gobernanza, diseñé flujos de trabajo y definiciones clave, y presenté ante el comité ejecutivo y el presidente de la CCB para lograr su validación y aprobación. Mi objetivo fue asegurar que la visión institucional se tradujera en un marco coherente, accionable y preparado para el futuro.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;03 —&lt;/span&gt;Acción&lt;/h2&gt;
+&lt;p&gt;&lt;strong&gt;Descubrimiento y diagnóstico del ecosistema.&lt;/strong&gt; Comenzamos con un diagnóstico a profundidad del ecosistema digital de la CCB mediante entrevistas, auditorías, análisis de plataformas y benchmarking. El equipo identificó los problemas centrales: toma de decisiones en silos, experiencias de usuario inconsistentes, servicios redundantes y falta de estándares compartidos. Mapeamos más de 15 activos digitales activos, 8 dominios y 21 soluciones tecnológicas distintas, lo que hizo evidente la necesidad de integración.&lt;/p&gt;
+&lt;p&gt;&lt;strong&gt;Principios de experiencia y alineación estratégica.&lt;/strong&gt; Para guiar las decisiones futuras, definimos seis principios centrales de experiencia, entre ellos &lt;em&gt;Zero Friction&lt;/em&gt;, &lt;em&gt;One CCB&lt;/em&gt; y &lt;em&gt;Make It Easy&lt;/em&gt;. Estos sirvieron como norte para priorizar contenidos, estructurar la navegación y reorganizar los servicios. Desarrollamos arquetipos de usuario, journeys, árboles de decisión y modelos de roles de servicio para alinear el ecosistema futuro con las necesidades reales de los usuarios.&lt;/p&gt;
+&lt;p&gt;&lt;strong&gt;Estructura unificada para el ecosistema digital.&lt;/strong&gt; Propusimos una arquitectura centralizada y modular que reorganizó la presencia digital de la CCB en cinco puntos de entrada principales: necesidades de las personas, necesidades de las empresas, trámites, servicios destacados y el ciclo de vida empresarial. Esta estructura futura se validó mediante talleres colaborativos y análisis de benchmarks. Entregamos wireframes, arquitectura de información y una taxonomía unificada para apoyar la implementación.&lt;/p&gt;
+&lt;p&gt;&lt;strong&gt;Diseño del modelo de gobernanza.&lt;/strong&gt; A partir de la visión estratégica, consolidé y formalicé un modelo de gobernanza de tres niveles —&lt;strong&gt;estratégico, táctico y operativo&lt;/strong&gt;— para clarificar roles, agilizar las decisiones y sostener la calidad en el tiempo. Definí procesos clave de gobernanza, entre ellos flujos de ingreso de solicitudes, la "definición de listo" y matrices RACI. También lideré presentaciones ejecutivas ante la alta dirección de la organización y obtuve el respaldo del presidente. El modelo le dio a la CCB una forma sostenible de gestionar el crecimiento digital manteniendo la consistencia y la rendición de cuentas.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;04 —&lt;/span&gt;Resultado&lt;/h2&gt;
+&lt;p&gt;El proyecto sentó las bases para transformar un panorama digital fragmentado en un &lt;strong&gt;ecosistema coherente, centrado en el usuario y gobernable&lt;/strong&gt;. La estrategia de experiencia permitió priorizar los servicios clave y una estructura arraigada en las necesidades reales de los usuarios. El modelo de gobernanza introdujo una responsabilidad clara, coordinación multifuncional y mecanismos para una evolución sostenida. Un aprendizaje clave fue que la transformación digital no se trata solo de plataformas: requiere alineación entre la visión, las operaciones y la cultura organizacional.&lt;/p&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -1290,7 +1401,24 @@
         </is>
       </c>
       <c r="T9" s="2" t="inlineStr"/>
-      <c r="U9" s="2" t="inlineStr"/>
+      <c r="U9" s="2" t="inlineStr">
+        <is>
+          <t>&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;01 —&lt;/span&gt;Situación&lt;/h2&gt;
+&lt;p&gt;MERAKI es una iniciativa de voluntariado que nació de un programa de liderazgo en transformación. Reúne a profesionales de la educación, la terapia, el diseño, el marketing y la recaudación de fondos para traducir la neurociencia y la compasión en herramientas prácticas para el desarrollo de la primera infancia. Su aliado ancla, la &lt;em&gt;Fundación Antioquia Infantil (FAIN)&lt;/em&gt;, está inaugurando una nueva sede en Caldas, Antioquia, para atender a niños y familias en contextos de alta vulnerabilidad.&lt;/p&gt;
+&lt;p&gt;El objetivo: dotar este sitio de ambientes inclusivos y con enfoque sensorial —aulas participativas, una sala multisensorial estructurada y espacios adaptativos que apoyen la regulación, la comunicación, el juego y la participación de los cuidadores—. La ambición más amplia es crear un modelo replicable que integre el diseño basado en evidencia, la intervención temprana y la participación comunitaria para niños de 0 a 6 años, incluidos aquellos con retrasos en el desarrollo, condiciones del espectro autista o desafíos de procesamiento sensorial.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;02 —&lt;/span&gt;Tarea&lt;/h2&gt;
+&lt;p&gt;Inicié y lideré la conceptualización de MERAKI como un movimiento: un sistema vivo de aulas sensoriales, prácticas y comunidades arraigado en la neurociencia, la compasión y la equidad. Luego conformé y movilicé a un equipo multidisciplinario de voluntarios —diseñadores, terapeutas, educadores, líderes operativos y recaudadores de fondos— para darle vida. Como líder del proyecto, impulso la visión y la estrategia, estructuro las líneas de trabajo y conecto a los stakeholders de FAIN, los proveedores, los donantes y el equipo de MERAKI. También me aseguro de la alineación con los principios de la primera infancia, lidero la movilización de recursos y defino los playbooks e indicadores que guiarán las futuras replicaciones.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;03 —&lt;/span&gt;Acción&lt;/h2&gt;
+&lt;p&gt;&lt;strong&gt;Conceptualización y encuadre del movimiento.&lt;/strong&gt; MERAKI empezó como una visión personal para tender un puente entre la neurociencia y la equidad a través del diseño. La encuadré no como una intervención aislada, sino como la semilla de un sistema más grande: una red de aulas sensoriales adaptables a distintos territorios y realidades. Esto llevó a la creación de un modelo modular que combina espacios físicos, protocolos de formación y activación comunitaria. La columna vertebral conceptual posicionó a MERAKI como un movimiento por la justicia sensorial en la primera infancia.&lt;/p&gt;
+&lt;p&gt;&lt;strong&gt;Gobernanza e integración de la hoja de ruta.&lt;/strong&gt; Para operacionalizar la visión, creamos una estructura de proyecto con cuatro frentes sincronizados —Infraestructura y Dotación, Protocolos Educativos, Comunicaciones y Recaudación, y Administración—, coordinados mediante hitos compartidos y un ritual semanal de integración. Establecí una hoja de ruta por fases, matrices de decisión y un tablero liviano para monitorear el avance, los riesgos y el impacto.&lt;/p&gt;
+&lt;p&gt;&lt;strong&gt;Infraestructura y dotación.&lt;/strong&gt; En colaboración con los terapeutas y educadores de FAIN, diseñamos programas espaciales alineados con los objetivos sensoriales: zonificación, iluminación, acústica y circulación. Se seleccionó un equipamiento que apoyara la estimulación vestibular, táctil, propioceptiva y auditiva.&lt;/p&gt;
+&lt;p&gt;&lt;strong&gt;Componente educativo y formación.&lt;/strong&gt; Arrancamos con un taller de neuroeducación para el personal de FAIN, que fundamentó la integración sensorial en la práctica cotidiana. A partir de ahí, codiseñamos módulos de formación sobre cómo observar las respuestas del niño, dosificar los estímulos sensoriales y diseñar rutinas adaptativas.&lt;/p&gt;
+&lt;p&gt;&lt;strong&gt;Comunicaciones y recaudación de fondos.&lt;/strong&gt; Para movilizar apoyos, creamos una estrategia de recaudación impulsada por lo social que combina narrativas digitales, pequeños aportes individuales y apoyo corporativo en especie. Dos eventos insignia —una formación en neuroeducación y un evento musical de recaudación en Medellín— ayudaron a ampliar el alcance y a generar visibilidad. Un tablero basado en el embudo hace seguimiento al alcance, el engagement y el cumplimiento de las donaciones, y orienta optimizaciones semanales.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;04 —&lt;/span&gt;Resultado&lt;/h2&gt;
+&lt;p&gt;A comienzos de 2026, la sede de FAIN en Caldas abrirá con un ecosistema de aprendizaje sensorial totalmente dotado, que se proyecta beneficiará a más de 200 niños al año, además de a sus cuidadores. El espacio traduce la neurociencia en interacciones cotidianas, apoyando la atención, la comunicación, la regulación emocional y la coordinación motriz mediante un diseño inclusivo.&lt;/p&gt;
+&lt;p&gt;Los educadores y las familias obtienen estrategias simples y repetibles que se extienden del aula al hogar. El piloto de Caldas establece el primer nodo de una visión más grande: una red MERAKI de espacios sensoriales, arraigada en la equidad, la ciencia y el cuidado, posicionada para escalar a nuevas comunidades en los próximos años.&lt;/p&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -1382,7 +1510,26 @@
       </c>
       <c r="S10" s="2" t="inlineStr"/>
       <c r="T10" s="2" t="inlineStr"/>
-      <c r="U10" s="2" t="inlineStr"/>
+      <c r="U10" s="2" t="inlineStr">
+        <is>
+          <t>&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;01 —&lt;/span&gt;Contexto&lt;/h2&gt;
+&lt;p&gt;Ecopetrol, una destacada compañía de energía de América Latina, buscaba optimizar la gestión de su flujo de caja en medio de un mercado energético global volátil y de la transición hacia prácticas sostenibles. Una gestión eficaz del flujo de caja es crucial para que Ecopetrol navegue las fluctuaciones de precios y los cambios en la demanda, y respalde su crecimiento y sostenibilidad. La Vicepresidencia de Finanzas y el Hub de EBA se propusieron mejorar los procesos y resultados financieros mediante la iniciativa 360° Cash Flow, aprovechando analítica avanzada y tecnología.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;02 —&lt;/span&gt;Desafío&lt;/h2&gt;
+&lt;p&gt;El principal desafío era pasar de un análisis de flujo de caja tradicional, centrado en la producción, a un modelo proactivo orientado al valor. Ecopetrol necesitaba un sistema robusto que ofreciera insights en tiempo real, agilizara la captura de datos y mejorara la precisión de las proyecciones financieras. Esta transformación exigía superar las ineficiencias operativas existentes e integrar soluciones tecnológicas innovadoras.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;03 —&lt;/span&gt;El proceso&lt;/h2&gt;
+&lt;p&gt;El proyecto comenzó con una fase de planeación enfocada en la que definimos los objetivos estratégicos y conformamos un equipo multidisciplinario. Se entrevistó a los stakeholders clave para capturar puntos de dolor y aspiraciones, sentando las bases para un proceso de diseño colaborativo e informado.&lt;/p&gt;
+&lt;p&gt;Con esta base, pasamos a la fase de exploración y alineación. Juntos, construimos una base de conocimiento compartida que permitió a los participantes mapear el desafío y aclarar los objetivos de largo plazo. Esto creó las condiciones para un entendimiento colectivo y una visión unificada.&lt;/p&gt;
+&lt;p&gt;A partir de ahí, entramos en una etapa de ideación altamente creativa. Mediante sesiones estructuradas de cocreación, el equipo generó una amplia variedad de ideas y exploró diversas formas de mejorar la gestión del flujo de caja. Estas ideas se fueron refinando progresivamente con bocetos y discusiones hasta que surgió un concepto cohesivo.&lt;/p&gt;
+&lt;p&gt;Siguió la toma de decisiones, en la que priorizamos las ideas más viables y empezamos a dar forma a la experiencia de usuario. Se creó un flujo de prototipo de alto nivel, apoyado en diseños detallados de pantallas que ilustraban cómo funcionaría la plataforma.&lt;/p&gt;
+&lt;p&gt;Luego llegó la etapa de prototipado. Desarrollamos un prototipo realista e interactivo y diseñamos un guion narrativo para demostrar el potencial de la solución. Este prototipo mostró funcionalidades clave como el seguimiento de la posición de liquidez, herramientas de proyección y capacidades de simulación.&lt;/p&gt;
+&lt;p&gt;Finalmente, el prototipo se probó con expertos financieros y stakeholders. Sus comentarios fueron fundamentales para identificar oportunidades de mejora y asegurar que la solución respondiera de manera efectiva a necesidades reales.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;04 —&lt;/span&gt;Resultados&lt;/h2&gt;
+&lt;p&gt;El prototipo de &lt;em&gt;360° Cash Flow&lt;/em&gt; introdujo una nueva forma de gestionar las finanzas en Ecopetrol. Ofreció herramientas intuitivas para la simulación de escenarios, la visualización del flujo de caja y la planeación estratégica, lo que permite a los equipos pasar del análisis reactivo a un insight proactivo. El Design Sprint dio lugar a varios avances clave:&lt;/p&gt;
+&lt;ol&gt;&lt;li&gt;&lt;strong&gt;Desarrollo del prototipo:&lt;/strong&gt; Creamos un prototipo funcional de una plataforma 360° Cash Flow, con herramientas intuitivas para explorar, filtrar y analizar datos financieros. Entre las funcionalidades clave estaban la posición de liquidez, la proyección de caja, la simulación del flujo de caja, el seguimiento del desempeño y la optimización.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Soluciones centradas en el usuario:&lt;/strong&gt; Validamos el prototipo con stakeholders, asegurando que respondiera a las necesidades de los usuarios y a los principales puntos de dolor. Las herramientas facilitaron una toma de decisiones más eficiente y basada en datos, reduciendo las tareas manuales y mejorando la claridad de los datos.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Alineación estratégica:&lt;/strong&gt; Alineamos las nuevas herramientas con los objetivos estratégicos de Ecopetrol, apoyando un enfoque más estructurado y sistemático del análisis de flujo de caja y del pronóstico macroeconómico. Esta alineación permitió una mejor integración del conocimiento experto, los modelos analíticos y las fuentes de datos externas.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Colaboración fortalecida:&lt;/strong&gt; Fomentamos una cultura colaborativa entre los miembros del equipo, combinando diversas perspectivas para innovar y resolver problemas complejos. La participación de los stakeholders fue crucial para lograr la aceptación y el respaldo de las nuevas iniciativas.&lt;/li&gt;&lt;/ol&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;05 —&lt;/span&gt;Impacto&lt;/h2&gt;
+&lt;p&gt;Esta iniciativa transformó la gestión del flujo de caja en Ecopetrol. La plataforma permitió obtener insights en tiempo real, redujo el manejo manual de datos y mejoró la precisión de los pronósticos. También respaldó la toma de decisiones estratégicas con herramientas de simulación y optimización. Más allá de los beneficios técnicos, el proyecto impulsó un cambio cultural hacia la agilidad, el pensamiento centrado en el usuario y la innovación, sentando las bases de un futuro financiero más inteligente y resiliente.&lt;/p&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -1465,7 +1612,21 @@
       </c>
       <c r="S11" s="2" t="inlineStr"/>
       <c r="T11" s="2" t="inlineStr"/>
-      <c r="U11" s="2" t="inlineStr"/>
+      <c r="U11" s="2" t="inlineStr">
+        <is>
+          <t>&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;01 —&lt;/span&gt;Punto de partida&lt;/h2&gt;
+&lt;p&gt;En octubre de 2024, Ecopetrol, en alianza con &lt;strong&gt;The Cocktail&lt;/strong&gt;, CCCS y XM, realizó un &lt;strong&gt;taller de cocreación&lt;/strong&gt; en Bogotá. El objetivo era explorar oportunidades para reutilizar subproductos de la industria de petróleo y gas en la construcción sostenible, siguiendo los principios de la &lt;strong&gt;Economía Circular&lt;/strong&gt;. Ecopetrol enfrentaba desafíos para que estos materiales (por ejemplo, catalizadores gastados, sólidos de clarificación y residuos de construcción y demolición) fueran comercialmente viables y sostenibles para los sectores de la construcción y la infraestructura.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;02 —&lt;/span&gt;El desafío&lt;/h2&gt;
+&lt;p&gt;El desafío era crear un &lt;strong&gt;modelo de negocio sostenible y circular&lt;/strong&gt; que permitiera la certificación y comercialización de los subproductos generados en las operaciones de Ecopetrol. La dificultad radicaba en reunir a distintos actores del ecosistema —entes reguladores, constructoras y aliados estratégicos— asegurando al mismo tiempo la factibilidad técnica, la aceptación del mercado y el cumplimiento normativo.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;03 —&lt;/span&gt;Qué hicimos&lt;/h2&gt;
+&lt;ul&gt;&lt;li&gt;Facilitamos un &lt;strong&gt;taller de cocreación&lt;/strong&gt; con metodologías ágiles en The Cocktail Bogotá.&lt;/li&gt;&lt;li&gt;Involucramos a equipos de &lt;strong&gt;CCCS y XM&lt;/strong&gt;, junto con expertos en ciencia, tecnología e innovación de Ecopetrol.&lt;/li&gt;&lt;li&gt;Identificamos y priorizamos subproductos clave para la exploración circular: &lt;strong&gt;sólidos de clarificación, catalizadores FCC gastados, residuos de construcción y asfalto modificado&lt;/strong&gt;.&lt;/li&gt;&lt;li&gt;Desarrollamos &lt;strong&gt;prototipos de modelos de negocio&lt;/strong&gt; centrados en la reutilización de estos subproductos.&lt;/li&gt;&lt;li&gt;Exploramos &lt;strong&gt;áreas de aplicación&lt;/strong&gt;, entre ellas infraestructura pública, vivienda social y proyectos de construcción comercial.&lt;/li&gt;&lt;li&gt;Establecimos &lt;strong&gt;sinergias y alianzas&lt;/strong&gt; para habilitar proyectos piloto.&lt;/li&gt;&lt;li&gt;Documentamos los resultados y delineamos los próximos pasos para &lt;strong&gt;escalar&lt;/strong&gt; el modelo.&lt;/li&gt;&lt;/ul&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;04 —&lt;/span&gt;El impacto&lt;/h2&gt;
+&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Identificamos 5 áreas clave de aplicación&lt;/strong&gt; de los subproductos en infraestructura y construcción.&lt;/li&gt;&lt;li&gt;Desarrollamos &lt;strong&gt;prototipos de modelos de negocio&lt;/strong&gt; enfocados en reutilizar sólidos de clarificación y catalizadores FCC.&lt;/li&gt;&lt;li&gt;Exploramos &lt;strong&gt;alianzas estratégicas&lt;/strong&gt; entre sectores para apoyar la certificación y comercialización de los subproductos.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Inspiración y alineación&lt;/strong&gt; entre los participantes, que fomentan futuras colaboraciones para operaciones sostenibles.&lt;/li&gt;&lt;/ul&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;05 —&lt;/span&gt;Después de este proyecto&lt;/h2&gt;
+&lt;p&gt;En VML desarrollamos un proyecto de venture building con Ecopetrol para lanzar una nueva unidad de negocio enfocada en encontrar soluciones circulares para los subproductos de sus procesos productivos.&lt;/p&gt;
+&lt;p&gt;En las refinerías de Ecopetrol, el agua del río Magdalena debe clarificarse antes de entrar al ciclo productivo, lo que deja un material sólido que antes se trataba como desecho. En Neture Impact (parte de VML), ayudamos a Ecopetrol a transformar este subproducto en ladrillos sostenibles, convirtiendo lo que antes era un material desechado en una solución comercial valiosa para la industria de la construcción.&lt;/p&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -1541,7 +1702,18 @@
       </c>
       <c r="S12" s="2" t="inlineStr"/>
       <c r="T12" s="2" t="inlineStr"/>
-      <c r="U12" s="2" t="inlineStr"/>
+      <c r="U12" s="2" t="inlineStr">
+        <is>
+          <t>&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;01 —&lt;/span&gt;Contexto&lt;/h2&gt;
+&lt;p&gt;Este proyecto consistió en diseñar una metodología para caracterizar los 11 retos de Ecopetrol en Ciencia, Tecnología e Innovación (CT+i) hacia 2040. Colaboramos con el equipo de la Gerencia de Estrategia CT+i de Ecopetrol y con expertos técnicos del ICPET (Centro de Investigación). Inicialmente, no existía un proceso estandarizado para analizar estos retos complejos y multidimensionales, lo que dificultaba la toma de decisiones estratégicas y la asignación de recursos. El proyecto buscaba crear un enfoque estructurado y participativo para comprender estos retos, identificar las palancas tecnológicas clave y habilitar una planeación estratégica informada, alineada con la visión 2040 de Ecopetrol.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;02 —&lt;/span&gt;Desafío&lt;/h2&gt;
+&lt;p&gt;El principal desafío era la falta de una metodología clara y consistente para analizar los megaretos. Esta ausencia dificultaba la resolución eficaz de problemas, la priorización de recursos y la alineación de esfuerzos entre las distintas áreas y filiales de Ecopetrol. Los enfoques existentes ofrecían perspectivas limitadas y aisladas, que no lograban capturar la naturaleza interconectada de los retos ni el entorno dinámico en el que existen. Esta falta de un entendimiento y un marco compartidos dificultaba identificar soluciones efectivas y medir el avance hacia las metas estratégicas 2040.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;03 —&lt;/span&gt;Acciones realizadas&lt;/h2&gt;
+&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Planeación inicial y alineación:&lt;/strong&gt; El equipo de The-Cocktail sostuvo reuniones con la Gerencia de Estrategia CT+i de Ecopetrol para comprender su visión, recopilar información y alinear las expectativas del proyecto.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Diseño colaborativo del taller:&lt;/strong&gt; Se diseñó un taller virtual de cocreación con ejercicios interactivos y dinámicas colaborativas para facilitar un entendimiento compartido del reto y de los resultados deseados.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Taller virtual de cocreación:&lt;/strong&gt; Se realizó un taller virtual de cuatro horas con personal de Ecopetrol y expertos técnicos del ICPET. Los participantes realizaron actividades para definir el propósito, el alcance y los resultados deseados del proceso de caracterización.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Desarrollo de la metodología:&lt;/strong&gt; Con base en los resultados del taller, se desarrolló una metodología de cinco etapas que incorpora principios de pensamiento sistémico y diseño participativo.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Ejemplos ilustrativos y herramientas:&lt;/strong&gt; Se desarrollaron ejemplos ilustrativos, métodos y herramientas para guiar la aplicación de la metodología.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Documentación y reporte:&lt;/strong&gt; Se elaboró un informe integral que documenta el proceso del taller, la metodología resultante y las recomendaciones para los siguientes pasos.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Recomendación de un proyecto piloto:&lt;/strong&gt; Se recomendó un proyecto piloto para probar y refinar la metodología con uno de los megaretos.&lt;/li&gt;&lt;/ul&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;04 —&lt;/span&gt;Impacto&lt;/h2&gt;
+&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Metodología estructurada:&lt;/strong&gt; Se creó una metodología clara de cinco etapas para caracterizar los megaretos, que ofrece un enfoque estructurado para el análisis y la toma de decisiones.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Entendimiento compartido:&lt;/strong&gt; El taller y el informe posterior fomentaron un entendimiento compartido de los retos y de la importancia de un enfoque multidisciplinario.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Colaboración fortalecida:&lt;/strong&gt; El proceso participativo impulsó la colaboración y el intercambio de conocimiento entre las distintas áreas y filiales de Ecopetrol.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Alineación estratégica:&lt;/strong&gt; La metodología aseguró la alineación con la visión y los objetivos estratégicos 2040 de Ecopetrol.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Marco accionable:&lt;/strong&gt; La metodología definida y la recomendación del proyecto piloto ofrecieron un marco accionable para avanzar en el proceso de caracterización.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Desarrollo de capacidades:&lt;/strong&gt; El taller y los materiales de apoyo contribuyeron al desarrollo de capacidades en Ecopetrol en pensamiento sistémico y métodos participativos.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Mayor eficiencia:&lt;/strong&gt; Se espera que el enfoque estructurado aumente la eficiencia en la asignación de recursos y la priorización de proyectos.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -1630,7 +1802,27 @@
       </c>
       <c r="S13" s="2" t="inlineStr"/>
       <c r="T13" s="2" t="inlineStr"/>
-      <c r="U13" s="2" t="inlineStr"/>
+      <c r="U13" s="2" t="inlineStr">
+        <is>
+          <t>&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;01 —&lt;/span&gt;Contexto&lt;/h2&gt;
+&lt;p&gt;Ecopetrol, una de las principales compañías de energía de América Latina, enfrentaba desafíos para analizar y visualizar de manera eficiente los pronósticos de precios y las variables macroeconómicas. El departamento de Análisis Económico e Industria dependía en gran medida de una hoja de cálculo integral conocida como la "Hoja de Precios", ampliamente utilizada en diversas áreas gerenciales y operativas. Sin embargo, se hizo evidente la necesidad de una solución tecnológica más robusta, interactiva y escalable para respaldar mejor las decisiones estratégicas y operativas.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;02 —&lt;/span&gt;Desafío&lt;/h2&gt;
+&lt;p&gt;El principal desafío era mejorar las metodologías de análisis de precios y variables macroeconómicas, y perfeccionar el despliegue y la visualización de esta información crítica. Las herramientas existentes no eran lo suficientemente interactivas ni amigables, lo que generaba ineficiencias y dificultades en la interpretación de los datos y en la toma de decisiones. Para abordarlo, se inició un Design Sprint con el fin de desarrollar soluciones ágiles y colaborativas que transformaran las prácticas actuales.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;03 —&lt;/span&gt;Qué hicimos&lt;/h2&gt;
+&lt;p&gt;&lt;strong&gt;Planeación y preparación.&lt;/strong&gt; Definimos el desafío y los objetivos del sprint. Seleccionamos un equipo central multidisciplinario y planeamos las actividades del sprint. Recopilamos información relevante y realizamos entrevistas con stakeholders para comprender el contexto.&lt;/p&gt;
+&lt;p&gt;&lt;strong&gt;Comprensión y definición.&lt;/strong&gt; Creamos una base de conocimiento compartida entre los participantes mediante conversaciones estructuradas. Mapeamos el desafío y definimos metas de largo plazo y preguntas clave por resolver.&lt;/p&gt;
+&lt;p&gt;&lt;strong&gt;Ideación y bocetos.&lt;/strong&gt; Realizamos ejercicios para generar y refinar una amplia variedad de ideas. Desarrollamos bocetos detallados de posibles soluciones.&lt;/p&gt;
+&lt;p&gt;&lt;strong&gt;Toma de decisiones.&lt;/strong&gt; Evaluamos y seleccionamos las ideas más prometedoras por consenso del equipo. Creamos un flujo de prototipo de alto nivel y diseños detallados de pantallas.&lt;/p&gt;
+&lt;p&gt;&lt;strong&gt;Prototipado.&lt;/strong&gt; Desarrollamos un prototipo realista de la solución elegida. Diseñamos y definimos un guion para presentar el concepto y las funcionalidades.&lt;/p&gt;
+&lt;p&gt;&lt;strong&gt;Validación.&lt;/strong&gt; Probamos el prototipo con stakeholders clave. Recopilamos comentarios para identificar fortalezas y oportunidades de mejora.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;04 —&lt;/span&gt;Resultados&lt;/h2&gt;
+&lt;p&gt;El Design Sprint produjo avances significativos en los procesos de análisis de precios de Ecopetrol:&lt;/p&gt;
+&lt;ol&gt;&lt;li&gt;&lt;strong&gt;Desarrollo del prototipo:&lt;/strong&gt; Creamos un prototipo funcional de un portal de análisis de precios, con herramientas intuitivas para explorar, consumir, filtrar y analizar la información relevante. El portal incluía funcionalidades como la búsqueda de variables, visualizaciones en formato de gráfico o tabla, el guardado de escenarios y la comparación entre distintos conjuntos de precios.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Soluciones centradas en el usuario:&lt;/strong&gt; El prototipo se validó con stakeholders, asegurando que respondiera a las necesidades de los usuarios y a los principales puntos de dolor. Las nuevas herramientas facilitaron una toma de decisiones más eficiente y basada en datos, reduciendo la dependencia de métodos manuales y mejorando la claridad de la información.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Alineación estratégica:&lt;/strong&gt; Las nuevas herramientas se alinearon con los objetivos estratégicos de largo plazo de Ecopetrol, apoyando un enfoque más estructurado y sistemático del análisis de precios y del pronóstico macroeconómico. Esta alineación permitió una mejor integración del conocimiento experto, los modelos analíticos y las fuentes de datos externas.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Colaboración fortalecida:&lt;/strong&gt; El sprint fomentó una cultura colaborativa entre los miembros del equipo, combinando diversas perspectivas para innovar y resolver problemas complejos. La participación activa de los stakeholders en el proceso del sprint ayudó a lograr la aceptación y el respaldo de las nuevas iniciativas.&lt;/li&gt;&lt;/ol&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;05 —&lt;/span&gt;Impacto&lt;/h2&gt;
+&lt;p&gt;El Design Sprint no solo transformó el enfoque de Ecopetrol frente al análisis de precios, sino que también sentó un precedente para futuros proyectos de innovación. La iniciativa puso de relieve el valor de las metodologías ágiles y del diseño centrado en el usuario para impulsar el cambio organizacional y mejorar la eficiencia. Se espera que la implementación exitosa de las nuevas herramientas y metodologías fortalezca de manera significativa la capacidad de Ecopetrol para tomar decisiones estratégicas informadas con base en datos precisos y oportunos.&lt;/p&gt;
+&lt;p&gt;Al abordar las brechas tecnológicas y metodológicas, la iniciativa del Design Sprint abrió el camino hacia soluciones más robustas y escalables, contribuyendo en última instancia a la misión de Ecopetrol de generar valor sostenible para sus grupos de interés.&lt;/p&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
@@ -1708,7 +1900,16 @@
       </c>
       <c r="S14" s="2" t="inlineStr"/>
       <c r="T14" s="2" t="inlineStr"/>
-      <c r="U14" s="2" t="inlineStr"/>
+      <c r="U14" s="2" t="inlineStr">
+        <is>
+          <t>&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;01 —&lt;/span&gt;Contexto&lt;/h2&gt;
+&lt;p&gt;En julio de 2024, Ecopetrol, en colaboración con The-Cocktail, realizó un Bootcamp de Diseño Ágil para fortalecer sus procesos de innovación y la conceptualización de iniciativas. Este programa intensivo estuvo dirigido al equipo del Analytics Hub de Ecopetrol, un grupo cuya misión es maximizar el valor del grupo empresarial mediante la analítica, identificando oportunidades y desarrollando soluciones que mejoren la toma de decisiones y optimicen las operaciones de la compañía.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;02 —&lt;/span&gt;El desafío&lt;/h2&gt;
+&lt;p&gt;El principal desafío del Analytics Hub de Ecopetrol era demostrar su valor a través del impacto tangible de sus iniciativas. Adoptar metodologías de diseño ágil era esencial para acelerar la identificación y solución de problemas, promover la colaboración interdisciplinaria y permitir una iteración rápida de las ideas. Este enfoque buscaba mejorar la capacidad del equipo para responder con rapidez a las necesidades del mercado, impulsar su cultura de innovación y generar valor sostenible para la compañía.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;03 —&lt;/span&gt;Qué hicimos&lt;/h2&gt;
+&lt;ul&gt;&lt;li&gt;Realizamos un bootcamp intensivo de un día en el que se presentó el marco de diseño ágil y su relevancia en contextos empresariales.&lt;/li&gt;&lt;li&gt;Definimos las expectativas y metas de largo plazo del equipo del Analytics Hub.&lt;/li&gt;&lt;li&gt;Identificamos los problemas clave con el Mapa de Desafíos y preguntas HMW.&lt;/li&gt;&lt;li&gt;Generamos soluciones creativas con técnicas como Crazy 8.&lt;/li&gt;&lt;li&gt;Construimos prototipos rápidos de las mejores ideas seleccionadas.&lt;/li&gt;&lt;li&gt;Probamos los prototipos con usuarios reales para recopilar comentarios.&lt;/li&gt;&lt;li&gt;Resumimos los hallazgos y planeamos los siguientes pasos para implementar las soluciones desarrolladas.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
@@ -1796,7 +1997,18 @@
         </is>
       </c>
       <c r="T15" s="2" t="inlineStr"/>
-      <c r="U15" s="2" t="inlineStr"/>
+      <c r="U15" s="2" t="inlineStr">
+        <is>
+          <t>&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;01 —&lt;/span&gt;Contexto&lt;/h2&gt;
+&lt;p&gt;En julio de 2024, Ecopetrol, en colaboración con The-Cocktail, realizó un Design Sprint para mejorar sus procesos de comercialización de crudo mediante analítica avanzada. Este sprint intensivo de tres días buscaba identificar y abordar los desafíos críticos del equipo de trading, como optimizar la toma de decisiones, mejorar la eficiencia operativa y maximizar los márgenes comerciales. Participaron diversas áreas de la compañía para asegurar la integración fluida de las nuevas estrategias en los flujos de trabajo diarios.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;02 —&lt;/span&gt;Desafío&lt;/h2&gt;
+&lt;p&gt;El equipo de comercialización de crudo de Ecopetrol enfrentaba múltiples desafíos en un mercado altamente volátil y competitivo. La necesidad de acceder a información crítica dispersa y gestionarla, evaluar y mitigar riesgos de manera eficiente y optimizar procesos manuales limitaba su capacidad de maximizar los márgenes comerciales. Además, la falta de coordinación entre departamentos y la complejidad de mantener relaciones sólidas con los clientes dificultaban la toma de decisiones informadas. El desafío general era transformar el proceso de comercialización desarrollando soluciones innovadoras que alinearan a todas las áreas involucradas y aprovecharan la analítica avanzada para una gestión más ágil y efectiva.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;03 —&lt;/span&gt;Acciones realizadas&lt;/h2&gt;
+&lt;ul&gt;&lt;li&gt;Realizamos un Design Sprint de tres días con metodologías ágiles y creativas, enfocado en optimizar la comercialización de crudo mediante analítica avanzada.&lt;/li&gt;&lt;li&gt;Involucramos a más de 18 participantes de Ecopetrol para asegurar perspectivas diversas y soluciones integrales.&lt;/li&gt;&lt;li&gt;Desarrollamos 13 conceptos de solución e identificamos 22 funcionalidades clave para el backlog.&lt;/li&gt;&lt;li&gt;Creamos un prototipo validado para la comercialización en el mercado asiático.&lt;/li&gt;&lt;li&gt;Mapeamos el proceso de comercialización y facilitamos la coordinación entre departamentos.&lt;/li&gt;&lt;li&gt;Realizamos ejercicios para priorizar las iniciativas de mayor valor y detallamos los conceptos para un prototipo de alta fidelidad.&lt;/li&gt;&lt;li&gt;Validamos el prototipo con stakeholders clave e incorporamos sus comentarios en la solución final.&lt;/li&gt;&lt;/ul&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;04 —&lt;/span&gt;Impacto esperado&lt;/h2&gt;
+&lt;ul&gt;&lt;li&gt;Procesos de toma de decisiones fortalecidos, que permiten respuestas más rápidas e informadas ante las fluctuaciones del mercado.&lt;/li&gt;&lt;li&gt;Mayor eficiencia operativa gracias a procesos manuales optimizados y a una mejor coordinación entre departamentos.&lt;/li&gt;&lt;li&gt;Mayores márgenes comerciales al alinear las estrategias de comercialización con los insights de la analítica avanzada.&lt;/li&gt;&lt;li&gt;Mayor satisfacción de los clientes gracias a más transparencia, personalización y tiempos de transacción más rápidos.&lt;/li&gt;&lt;li&gt;Adopción facilitada de nuevas metodologías y herramientas de comercialización entre el personal de Ecopetrol, asegurando una transición fluida hacia prácticas de trading más avanzadas.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
@@ -1894,7 +2106,24 @@
         </is>
       </c>
       <c r="T16" s="2" t="inlineStr"/>
-      <c r="U16" s="2" t="inlineStr"/>
+      <c r="U16" s="2" t="inlineStr">
+        <is>
+          <t>&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;01 —&lt;/span&gt;Contexto&lt;/h2&gt;
+&lt;p&gt;Parque Explora, un reconocido museo de ciencias de Medellín, Colombia, emprendió un camino de transformación estratégica para aumentar su impacto en la comunidad y asegurar su sostenibilidad a largo plazo. La organización buscaba integrar sus diversas ofertas, entre ellas exposiciones interactivas, programas educativos y esfuerzos de conservación, en un marco estratégico cohesivo. Esta iniciativa respondía a la necesidad de alinear los procesos internos, fomentar una cultura organizacional unificada y aprovechar los avances tecnológicos para lograr una mayor eficiencia operativa.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;02 —&lt;/span&gt;El desafío&lt;/h2&gt;
+&lt;p&gt;Parque Explora había llegado a un punto de inflexión: el crecimiento rápido y la diversificación generaron un fuerte impulso, pero también revelaron la oportunidad de &lt;strong&gt;clarificar la dirección estratégica&lt;/strong&gt; y fortalecer las &lt;strong&gt;prácticas organizacionales compartidas&lt;/strong&gt;. Con el tiempo, las operaciones se habían vuelto más complejas y fragmentadas, lo que llevó a prioridades desalineadas, ineficiencias en los procesos y momentos en que el foco en la misión central del museo se diluía. En paralelo, avanzar hacia un &lt;strong&gt;modelo financiero sostenible&lt;/strong&gt; y profundizar la &lt;strong&gt;relación con los grupos de interés&lt;/strong&gt; se volvió crítico para asegurar la viabilidad a largo plazo.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;03 —&lt;/span&gt;Mi rol&lt;/h2&gt;
+&lt;p&gt;Lideré el desarrollo integral de la propuesta comercial, desde la construcción de una propuesta de valor ganadora hasta las presentaciones al cliente y la negociación del alcance del proyecto. Una vez iniciado el proyecto, guié al equipo consultor aportando dirección estratégica, insights de contexto sobre Parque Explora y profundidad de análisis. También le di forma a la narrativa de impacto alineada con las tendencias globales de futuro y refiné el modelo operativo para asegurar la coherencia entre la visión y la ejecución.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;04 —&lt;/span&gt;El proceso&lt;/h2&gt;
+&lt;p&gt;Comenzamos con un diagnóstico integral para comprender el estado actual de la organización. Este incluyó más de 50 documentos internos, 20 entrevistas con el liderazgo y dos grupos focales con equipos de primera línea y miembros de la comunidad. Una visita física al sitio nos dio una idea de las realidades espaciales y operativas del museo. Esta fase reveló una profunda desalineación entre los equipos, iniciativas desconectadas y la falta de un lenguaje estratégico compartido.&lt;/p&gt;
+&lt;p&gt;A través de talleres colaborativos, sacamos a la luz las tensiones y aspiraciones centrales. Identificamos cuatro fuerzas globales que están dando forma al futuro —la salud planetaria, la aceleración tecnológica, la justicia social y la globalización—, que se convirtieron en la base del sensemaking estratégico. Facilitamos la alineación del liderazgo en torno a un propósito audaz pero aterrizado: catalizar la transformación social y ambiental a través del conocimiento, la curiosidad y la participación.&lt;/p&gt;
+&lt;p&gt;Cocreamos con el liderazgo una nueva arquitectura estratégica: un propósito compartido, un objetivo organizacional y cuatro pilares de impacto —Curiosidad Aumentada, Ciudadanía Activa, Escuelas Relevantes y Conservación Consciente—. Estos pilares conectaron los diversos programas de Explora con los futuros globales y las realidades locales. También articulamos un modelo de operación dual —museo y centro de desarrollo de proyectos— e introdujimos la metáfora de un "ecotono cultural" para describir la sinergia entre ambos mundos.&lt;/p&gt;
+&lt;p&gt;Tradujimos la estrategia en una hoja de ruta de transformación construida en torno a cuatro frentes estratégicos: Despliegue Estratégico, Armonía Cultural, Sinfonía Operativa y Camino al Futuro. Cada frente incluyó un conjunto de iniciativas de alto apalancamiento —como la transformación cultural, la arquitectura de interoperabilidad y un nuevo modelo de sostenibilidad—, diseñadas para cerrar la brecha entre la visión y la ejecución.&lt;/p&gt;
+&lt;p&gt;Estas definiciones estratégicas ofrecen a Parque Explora un marco integral para afrontar los desafíos futuros, asegurando la alineación de sus operaciones con su misión y sus metas, al tiempo que fomentan una cultura de aprendizaje, colaboración y sostenibilidad.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;05 —&lt;/span&gt;Resultado&lt;/h2&gt;
+&lt;p&gt;El proyecto entregó la primera estrategia corporativa formal de Parque Explora, totalmente cocreada y aprobada por su equipo directivo. Estableció un sistema operativo estratégico que alinea sus dos identidades —museo y aliado de innovación— y lo posiciona como catalizador del aprendizaje colectivo y la transformación. En lo personal, el proyecto profundizó mi práctica en prospectiva estratégica, diseño de sistemas culturales e innovación pública, reafirmando el diseño como motor del cambio sistémico.&lt;/p&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
@@ -1979,7 +2208,19 @@
       </c>
       <c r="S17" s="2" t="inlineStr"/>
       <c r="T17" s="2" t="inlineStr"/>
-      <c r="U17" s="2" t="inlineStr"/>
+      <c r="U17" s="2" t="inlineStr">
+        <is>
+          <t>&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;01 —&lt;/span&gt;Contexto&lt;/h2&gt;
+&lt;p&gt;Coppel, una importante cadena minorista de México, emprendió una iniciativa estratégica para mejorar la experiencia del cliente en sus tiendas. La iniciativa, facilitada por The Cocktail, buscaba abordar desafíos sistémicos, explorar oportunidades y establecer una hoja de ruta clara para mejorar la experiencia en tienda, en línea con el compromiso de Coppel con la satisfacción del cliente y la excelencia operativa.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;02 —&lt;/span&gt;Desafío&lt;/h2&gt;
+&lt;p&gt;Coppel enfrentaba varios desafíos significativos:&lt;/p&gt;
+&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Experiencia del cliente:&lt;/strong&gt; Garantizar una experiencia de compra fluida, satisfactoria y personalizada para cada cliente.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Accesibilidad:&lt;/strong&gt; Mejorar la accesibilidad de las tiendas para todos los clientes, incluidos aquellos con discapacidad.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Eficiencia operativa:&lt;/strong&gt; Optimizar las operaciones de las tiendas para mejorar el servicio y la satisfacción del cliente.&lt;/li&gt;&lt;/ul&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;03 —&lt;/span&gt;Metodología&lt;/h2&gt;
+&lt;p&gt;&lt;strong&gt;Comprensión y contextualización del desafío.&lt;/strong&gt; Realizamos un análisis a profundidad de la experiencia actual en tienda mediante observaciones y comentarios de los clientes. Identificamos las principales fortalezas y debilidades del recorrido actual del cliente.&lt;/p&gt;
+&lt;p&gt;&lt;strong&gt;Definición estratégica e identificación de oportunidades.&lt;/strong&gt; Definimos intenciones estratégicas claras para mejorar la experiencia en tienda. Identificamos tres áreas clave de oportunidad: personalización, accesibilidad y convivialidad.&lt;/p&gt;
+&lt;p&gt;&lt;strong&gt;Ideación y desarrollo de soluciones.&lt;/strong&gt; Realizamos talleres colaborativos para generar y priorizar posibles soluciones. Desarrollamos propuestas detalladas para las iniciativas con mayor potencial de impacto.&lt;/p&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
@@ -2079,7 +2320,26 @@
         </is>
       </c>
       <c r="T18" s="2" t="inlineStr"/>
-      <c r="U18" s="2" t="inlineStr"/>
+      <c r="U18" s="2" t="inlineStr">
+        <is>
+          <t>&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;01 —&lt;/span&gt;Contexto&lt;/h2&gt;
+&lt;p&gt;En Tu Hogar es una iniciativa estratégica liderada por KOF - TCCC para establecer una visión renovada y una hoja de ruta estratégica para el canal D2C (Direct-to-Consumer) de Coca-Cola en México. El proyecto busca consolidar un plan estratégico que dé foco y dirección a las acciones futuras, aprovechando las mayores áreas de oportunidad y abordando los desafíos clave para convertirse en un referente del canal digital D2C. El objetivo inicial es transformar la forma en que Coca-Cola interactúa con sus clientes mediante un ecosistema digital robusto y escalable.&lt;/p&gt;
+&lt;p&gt;Coca-Cola En tu Hogar ocupa un lugar muy querido en la cultura mexicana, que evoca nostalgia y momentos familiares compartidos. Su amplio rango de productos, su asequibilidad y su accesibilidad han consolidado su estatus icónico a lo largo de generaciones.&lt;/p&gt;
+&lt;p&gt;Sin embargo, en un mercado saturado y dominado por jugadores de entrega rápida y puramente digitales, este legado por sí solo no es suficiente. El canal enfrenta un bajo nivel de recordación y carece de una propuesta de valor distintiva, lo que limita su capacidad de competir eficazmente y retener clientes.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;02 —&lt;/span&gt;El desafío&lt;/h2&gt;
+&lt;p&gt;Coca-Cola FEMSA y The Coca-Cola Company se propusieron redefinir la dirección estratégica de su canal direct-to-consumer (D2C) en México, conocido como Coca-Cola en Tu Hogar (CCETH). A pesar de un aumento de 19 % en los ingresos frente al año anterior y de una base creciente de clientes digitales, el canal enfrentaba desafíos importantes: una propuesta de valor fragmentada, poca diferenciación y brechas internas que limitaban la escalabilidad. El objetivo era alinear a ambas organizaciones en torno a una visión audaz y accionable, y construir las bases estratégicas para que CCETH se convirtiera en un negocio de USD 1.500 millones para 2028.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;03 —&lt;/span&gt;El proceso&lt;/h2&gt;
+&lt;p&gt;&lt;strong&gt;Inmersión: comprender el ecosistema e identificar puntos ciegos.&lt;/strong&gt; Comenzamos con una fase de inmersión rápida pero rigurosa, en la que analizamos más de 24 documentos internos de KOF y KO, revisamos iniciativas pasadas y realizamos sesiones de seguimiento con stakeholders ejecutivos. Esto nos permitió mapear el ecosistema de manera integral y sacar a la luz inconsistencias entre la estrategia formal y la experiencia real de los usuarios y los equipos. A través de este "chequeo de realidad", descubrimos brechas críticas en la segmentación de clientes, la consistencia del servicio y la preparación digital.&lt;/p&gt;
+&lt;p&gt;&lt;strong&gt;Exploración: diálogo con stakeholders e investigación de usuarios.&lt;/strong&gt; La fase de exploración combinó más de 25 entrevistas con stakeholders con entrevistas individuales a usuarios y actividades de cocreación. Involucramos a quienes toman decisiones en marketing, tecnología y operaciones para entender sus ambiciones estratégicas, e incorporamos la voz directa de los clientes para validar las percepciones de valor. Luego facilitamos un taller de pensamiento estratégico en Ciudad de México con líderes de KO y KOF, en el que usamos marcos visuales para conectar la intención del negocio con las expectativas de los usuarios.&lt;/p&gt;
+&lt;p&gt;&lt;strong&gt;Diagnóstico: seis dimensiones estratégicas.&lt;/strong&gt; Sintetizamos nuestros hallazgos en seis dimensiones —cliente, competencia, finanzas, plataforma, estructura organizacional y alineación corporativa— para formar un diagnóstico del estado actual. Este análisis reveló un modelo D2C que luchaba por ofrecer consistencia y conexión emocional en su experiencia digital. Mapeamos protopersonas (por ejemplo, madres solteras, planificadores digitales, familias modernas) y las vinculamos con necesidades insatisfechas a lo largo del recorrido de la experiencia: desde la entrega hasta la lealtad y la variedad de productos.&lt;/p&gt;
+&lt;p&gt;&lt;strong&gt;Definición de capacidades y ventaja competitiva.&lt;/strong&gt; Luego, enmarcamos seis habilitadores de crecimiento para hacer tangible la propuesta de valor: Atracción del Hogar, Experiencia del Cliente, Desarrollo de Portafolio, Estrategia de Datos, Route-to-Market y Transformación Organizacional. Mapeamos las brechas de capacidades y sacamos a la luz dónde estaban alineados KOF y KO, y dónde no. Este insight nos ayudó a diseñar un modelo de transformación en dos fases: "Fix the Basics" para estabilizar la operación y "Value to Home" para escalar y diferenciarse.&lt;/p&gt;
+&lt;p&gt;&lt;strong&gt;Encuadre estratégico y priorización.&lt;/strong&gt; En la etapa final de definición, tradujimos la visión en una hoja de ruta clara y por fases. Cada capacidad se desglosó en iniciativas estratégicas que atendían las necesidades más urgentes del negocio —mejorar la confiabilidad de la entrega, ampliar el portafolio de productos y diseñar un modelo de lealtad basado en valor emocional y financiero—. Desarrollamos una narrativa ejecutiva y un modelo visual para comunicar cómo CCETH podía evolucionar de un servicio transaccional a una plataforma de relación distintiva y escalable.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;04 —&lt;/span&gt;Tarea&lt;/h2&gt;
+&lt;p&gt;Como Strategic Design Lead, guié la exploración desde una perspectiva centrada en el cliente y de pensamiento sistémico. Facilité los espacios clave con stakeholders, sinteticé insights de múltiples fuentes de datos y traduje los hallazgos en marcos estratégicos y áreas de oportunidad. También lideré la articulación de la narrativa estratégica que dio forma a nuestra definición final de capacidades, motores de crecimiento y prioridades de la hoja de ruta.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;05 —&lt;/span&gt;Resultado&lt;/h2&gt;
+&lt;p&gt;El proyecto entregó una visión estratégica compartida, una hoja de ruta priorizada y un conjunto de motores de crecimiento accionables que tanto KOF como KO adoptaron como base para la siguiente evolución del canal D2C. Estas definiciones han orientado decisiones de inversión posteriores y sirvieron como norte para la transformación digital, de portafolio y organizacional. Para mí, este proyecto afinó mi capacidad de diseñar en la complejidad —equilibrando el insight del usuario, la lógica de negocio y el cambio sistémico— mientras facilitaba la alineación entre audiencias ejecutivas diversas.&lt;/p&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
@@ -2172,7 +2432,27 @@
         </is>
       </c>
       <c r="T19" s="2" t="inlineStr"/>
-      <c r="U19" s="2" t="inlineStr"/>
+      <c r="U19" s="2" t="inlineStr">
+        <is>
+          <t>&lt;blockquote class="c-quote"&gt;Este proyecto fue un ejercicio académico del curso "Introduction to Futures Design" en CENTRO.&lt;/blockquote&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;01 —&lt;/span&gt;Contexto&lt;/h2&gt;
+&lt;p&gt;Ciudad de México (CDMX) enfrenta una amenaza creciente por el cambio climático, que se manifiesta en sequías, inundaciones y temperaturas extremas. La desigualdad socioeconómica y la falta de acceso a servicios básicos agravan la situación. En este contexto, se realizó un taller de prospectiva para diseñar futuros posibles y resilientes para la CDMX en 2050, con el fin de anticipar y mitigar los efectos adversos del cambio climático y de la gentrificación climática.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;02 —&lt;/span&gt;El desafío&lt;/h2&gt;
+&lt;p&gt;El principal desafío era abordar los múltiples problemas que enfrenta la CDMX debido al cambio climático y a la creciente desigualdad. Entre ellos están la escasez de agua, la migración climática, la contaminación del aire y la exclusión social causada por la gentrificación climática. Era crucial encontrar soluciones inclusivas y sostenibles que le permitieran a la ciudad adaptarse a un futuro incierto y adverso.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;03 —&lt;/span&gt;El método&lt;/h2&gt;
+&lt;p&gt;El proyecto utilizó una metodología de prospectiva integral que incluyó horizon scanning para identificar tendencias emergentes y señales de cambio, mapeo de tendencias para comprender las influencias clave sobre el futuro de la ciudad, y la aplicación de los Arquetipos de Futuros de Dator para explorar escenarios diversos como continuación, colapso, disciplina y transformación. Se crearon escenarios detallados, entre ellos el del "Oasis Amurallado", para visualizar posibles resultados. El estado futuro deseado se definió con un enfoque en la resiliencia, la inclusión y la sostenibilidad.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;04 —&lt;/span&gt;Escenario "Oasis Amurallado"&lt;/h2&gt;
+&lt;p&gt;El escenario del "Oasis Amurallado" presenta una visión provocadora y distópica de la Ciudad de México (CDMX) en 2050, que destaca la compleja interacción entre la resiliencia climática y la desigualdad social. Este escenario sirve como una narrativa poderosa para explorar las posibles consecuencias de un cambio climático sin control y de las dinámicas socioeconómicas que podría agravar.&lt;/p&gt;
+&lt;p&gt;En este futuro imaginado, ciertas zonas de la CDMX han evolucionado hasta convertirse en zonas "oasis", caracterizadas por una infraestructura altamente adaptable y resiliente. Estas zonas se han beneficiado de inversiones públicas y privadas significativas que las transformaron en refugios urbanos capaces de resistir eventos climáticos extremos. Sin embargo, esta prosperidad tiene un alto costo: &lt;strong&gt;la intensificación de la exclusión social a través de la gentrificación climática.&lt;/strong&gt; Estas son algunas implicaciones:&lt;/p&gt;
+&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Exclusión social:&lt;/strong&gt; El escenario ilustra con crudeza cómo los esfuerzos de adaptación al cambio climático pueden llevar, sin quererlo, a una mayor exclusión social si no se gestionan de manera inclusiva. Los oasis fortificados se convierten en enclaves de privilegio, y dejan a los menos favorecidos lidiando con condiciones ambientales cada vez peores.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Fragmentación urbana:&lt;/strong&gt; Las barreras físicas y sociales creadas por el muro refuerzan la segregación, lo que da lugar a un paisaje urbano fragmentado en el que las oportunidades y los recursos están distribuidos de forma desigual.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Tensiones y conflictos:&lt;/strong&gt; El escenario sugiere el potencial de mayores tensiones y conflictos sociales a medida que las disparidades se hacen más marcadas, con las zonas fortificadas como símbolo del fracaso en lograr una resiliencia equitativa.&lt;/li&gt;&lt;/ul&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;05 —&lt;/span&gt;El concepto: Centro de Resiliencia Climática&lt;/h2&gt;
+&lt;p&gt;El Centro de Resiliencia Climática (CRC) representa un enfoque visionario e incluyente para enfrentar los múltiples desafíos que plantea el cambio climático en la Ciudad de México (CDMX). Concebido como un faro de esperanza y un centro de innovación, el CRC busca fomentar un entorno urbano más resiliente y equitativo promoviendo la colaboración, la investigación y la acción frente al cambio climático y sus impactos socioeconómicos.&lt;/p&gt;
+&lt;h3 class="c-h3"&gt;Visión y misión&lt;/h3&gt;
+&lt;p&gt;El CRC aspira a un futuro en el que la CDMX prospere en un contexto de resiliencia climática participativa. Imagina una sociedad en la que la academia, las instituciones públicas, el sector privado y las comunidades trabajen juntos para forjar soluciones equitativas a los desafíos climáticos. La misión del centro hace énfasis en la accesibilidad, la inclusión y la democratización del conocimiento climático, procurando que todos los ciudadanos se beneficien de sus iniciativas.&lt;/p&gt;
+&lt;h3 class="c-h3"&gt;Características clave&lt;/h3&gt;
+&lt;ol&gt;&lt;li&gt;&lt;strong&gt;Investigación colaborativa:&lt;/strong&gt; El CRC facilita investigación de punta en ciencia climática, con foco en soluciones prácticas que puedan implementarse en entornos urbanos. Fomenta la colaboración entre científicos, formuladores de política y líderes comunitarios para abordar eficazmente los problemas climáticos locales.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Educación y formación:&lt;/strong&gt; El centro ofrece amplios programas de formación y talleres orientados a desarrollar capacidades entre residentes, profesionales y formuladores de política. Estas iniciativas se enfocan en la alfabetización climática, las prácticas sostenibles y las estrategias innovadoras de adaptación.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Incidencia en políticas públicas:&lt;/strong&gt; Mediante la incidencia política, el CRC busca influir en las políticas públicas y promover regulaciones que apoyen la resiliencia climática y la equidad social. Actúa como voz de las comunidades vulnerables, asegurando que sus necesidades y perspectivas se tengan en cuenta en los procesos de toma de decisiones.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Sensibilización pública y divulgación:&lt;/strong&gt; El CRC se dedica a generar conciencia pública sobre los impactos del cambio climático y la importancia de la resiliencia. A través de campañas, seminarios y eventos comunitarios, busca fomentar una cultura de adaptación proactiva y de cuidado del medio ambiente.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Centro de innovación:&lt;/strong&gt; El centro funciona como incubadora de innovaciones relacionadas con el clima e iniciativas emprendedoras. Apoya startups y proyectos que ofrecen soluciones sostenibles a los desafíos urbanos, brindando recursos y mentoría para convertir las ideas en acciones de impacto.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Refugio temporal para migrantes climáticos:&lt;/strong&gt; Reconociendo el problema creciente de la migración inducida por el clima, el CRC ofrece alojamiento temporal y servicios de apoyo para migrantes climáticos. Esta iniciativa garantiza que los migrantes tengan acceso a recursos esenciales y programas de integración.&lt;/li&gt;&lt;/ol&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
@@ -2257,7 +2537,19 @@
       </c>
       <c r="S20" s="2" t="inlineStr"/>
       <c r="T20" s="2" t="inlineStr"/>
-      <c r="U20" s="2" t="inlineStr"/>
+      <c r="U20" s="2" t="inlineStr">
+        <is>
+          <t>&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;01 —&lt;/span&gt;El contexto&lt;/h2&gt;
+&lt;p&gt;La Fundación Botánica y Zoológica de Barranquilla (ZooBaq), una institución de ciencia y conservación de larga trayectoria en la región Caribe de Colombia, enfrentaba desafíos urgentes de relevancia pública, deterioro de la infraestructura y obsolescencia digital. En medio de las cambiantes expectativas globales en torno al bienestar animal, la conservación y la experiencia de los visitantes, ZooBaq buscaba definir una visión convincente de su futuro. El objetivo: trazar una hoja de ruta estratégica que le permitiera a la organización prosperar como centro regional de ciencia y epicentro de la biodiversidad.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;02 —&lt;/span&gt;La tarea&lt;/h2&gt;
+&lt;p&gt;Como Strategic Design Lead en The Cocktail LATAM, lideré el diseño y la facilitación de un WorkShot (taller de estrategia) enfocado en alinear al liderazgo en torno a una visión compartida y en definir las prioridades clave para la transformación organizacional. Mi rol consistió en orquestar el análisis sistémico, sintetizar las aspiraciones colectivas y traducir la complejidad en direcciones de diseño accionables y oportunidades estratégicas.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;03 —&lt;/span&gt;El proceso&lt;/h2&gt;
+&lt;p&gt;Reunimos al equipo ejecutivo de ZooBaq en un WorkShot estratégico de dos días para cocrear su trayectoria futura. Usando los marcos propios de The Cocktail, mapeamos las dimensiones estratégicas actuales de la organización —propósito, propuesta de valor, comunidades, capacidades y recursos— y las contrastamos con sus aspiraciones futuras.&lt;/p&gt;
+&lt;p&gt;A través de métodos participativos, sacamos a la luz seis desafíos sistémicos (por ejemplo, incertidumbre en la infraestructura, pérdida de relevancia pública y una experiencia digital fragmentada) y desarrollamos las prioridades de transformación correspondientes.&lt;/p&gt;
+&lt;p&gt;El resultado incluyó una hoja de ruta con cinco frentes estratégicos: posicionamiento público, renovación de la infraestructura, sostenibilidad financiera mediante la activación de servicios, transformación digital y claridad operativa. Cada línea se detalló con objetivos, habilitadores, barreras e iniciativas clave, lo que le permitió a la institución alinear la acción con su misión.&lt;/p&gt;
+&lt;p&gt;Un componente central del proceso fue un ejercicio de prospectiva en el que los participantes imaginaron el rol de largo plazo de ZooBaq en la conservación de la región Caribe. Esto incluyó la codefinición de una visión "Estrella del Norte" y la exploración de escenarios futuros plausibles en torno a la infraestructura, la participación de la comunidad y la sostenibilidad. Estas exploraciones de escenarios ayudaron a identificar tensiones estratégicas y a crear una hoja de ruta por fases, receptiva tanto a las restricciones actuales como a las posibilidades futuras.&lt;/p&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
@@ -2344,7 +2636,21 @@
       </c>
       <c r="S21" s="2" t="inlineStr"/>
       <c r="T21" s="2" t="inlineStr"/>
-      <c r="U21" s="2" t="inlineStr"/>
+      <c r="U21" s="2" t="inlineStr">
+        <is>
+          <t>&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;01 —&lt;/span&gt;Contexto&lt;/h2&gt;
+&lt;p&gt;AFORE Coppel, una destacada administradora de fondos de pensiones de México, desempeña un papel crítico en la gestión de los recursos de retiro de millones de trabajadores. A pesar de los avances del sistema pensional, muchos afiliados enfrentan dificultades para reunir fondos suficientes para una pensión completa al momento del retiro. Esta iniciativa estratégica buscaba identificar oportunidades para aumentar la participación y las aportaciones de los afiliados y, en última instancia, mejorar los resultados pensionales.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;02 —&lt;/span&gt;Desafío&lt;/h2&gt;
+&lt;p&gt;AFORE Coppel enfrentaba desafíos significativos:&lt;/p&gt;
+&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Demografía y patrones de aportación:&lt;/strong&gt; Casi el 50 % de los afiliados tiene menos de 35 años y gana entre 1 y 3 salarios mínimos, con aportaciones esporádicas debido a empleos inestables o informales.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Afiliados inactivos:&lt;/strong&gt; Aproximadamente el 70 % de los afiliados está inactivo y no hace aportaciones regulares, lo que los pone en riesgo de no asegurar una pensión completa.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Educación financiera:&lt;/strong&gt; La falta de educación y conciencia financiera entre los afiliados limita su participación y su comprensión de los beneficios de aportar de manera constante.&lt;/li&gt;&lt;/ul&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;03 —&lt;/span&gt;Metodología&lt;/h2&gt;
+&lt;p&gt;&lt;strong&gt;Inmersión sistémica.&lt;/strong&gt; Realizamos un análisis a profundidad de todo el ciclo de vida de un afiliado de AFORE Coppel, desde la conciencia inicial hasta la recepción de su pensión. Identificamos los principales habilitadores e inhibidores que afectan la participación de los afiliados y sus comportamientos de aportación.&lt;/p&gt;
+&lt;p&gt;&lt;strong&gt;Definición estratégica e identificación de oportunidades.&lt;/strong&gt; Definimos intenciones claras para acompañar a los afiliados desde su primera aportación hasta su último pago de pensión, con transparencia, información y educación. Identificamos ocho áreas clave de oportunidad para intervenir, entre ellas activación, formación, estructura interna, aprendizaje del cliente, aprovechamiento del ecosistema de Coppel, programas de lealtad, mejoras en el presente y comunicación.&lt;/p&gt;
+&lt;p&gt;&lt;strong&gt;Ideación y desarrollo de soluciones.&lt;/strong&gt; Generamos y priorizamos una variedad de iniciativas para abordar los desafíos identificados, con foco tanto en los procesos internos como en la participación externa de los afiliados. Desarrollamos propuestas detalladas para las iniciativas con mayor potencial de impacto.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;04 —&lt;/span&gt;Áreas centrales de impacto&lt;/h2&gt;
+&lt;ol&gt;&lt;li&gt;&lt;strong&gt;Mayor participación de los afiliados:&lt;/strong&gt; Impulsar las aportaciones regulares mejorando el conocimiento de los beneficios del empleo formal y del ahorro constante.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Educación financiera fortalecida:&lt;/strong&gt; Ofrecer una educación financiera integral que empodere a los afiliados con mejores hábitos de ahorro y una toma de decisiones informada.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Eficiencia operativa:&lt;/strong&gt; Optimizar procesos e integrar datos para mejorar los flujos de trabajo internos y la eficiencia del servicio al cliente.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Prácticas de ahorro sostenibles:&lt;/strong&gt; Promover el ahorro voluntario y premiar los buenos comportamientos financieros mediante programas e incentivos innovadores.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Inclusión social y empleo formal:&lt;/strong&gt; Apoyar a los trabajadores inactivos e informales en su tránsito hacia el empleo formal, aumentando sus posibilidades de asegurar una pensión completa.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Mejor experiencia del cliente:&lt;/strong&gt; Mejorar la experiencia general del afiliado con acompañamiento personalizado, información clara y un servicio receptivo a lo largo de su recorrido de ahorro.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Mayor confianza de la comunidad:&lt;/strong&gt; Fomentar un sentido de pertenencia y confianza de los afiliados hacia AFORE Coppel, fortaleciendo la lealtad y la participación a largo plazo.&lt;/li&gt;&lt;/ol&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
@@ -2426,7 +2732,20 @@
       </c>
       <c r="S22" s="2" t="inlineStr"/>
       <c r="T22" s="2" t="inlineStr"/>
-      <c r="U22" s="2" t="inlineStr"/>
+      <c r="U22" s="2" t="inlineStr">
+        <is>
+          <t>&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;01 —&lt;/span&gt;El contexto&lt;/h2&gt;
+&lt;p&gt;Ecopetrol, una compañía líder de energía en América Latina, emprendió una iniciativa estratégica para mejorar sus procesos de gestión de activos financieros. La estrategia de largo plazo de la compañía, "Energía que Transforma", busca abordar desafíos ambientales, sociales y de gobernanza, creando valor sostenible para sus grupos de interés. La Vicepresidencia de Finanzas y el Hub de EBA buscaron desarrollar modelos analíticos apoyados en soluciones tecnológicas para mejorar la planeación y gestión de activos, en línea con los objetivos estratégicos de la compañía.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;02 —&lt;/span&gt;El desafío&lt;/h2&gt;
+&lt;p&gt;El principal desafío de Ecopetrol era transformar sus conversaciones sobre la gestión de activos financieros. Tradicionalmente centradas en el desempeño pasado y la rendición de cuentas, la meta era pasar a maximizar el valor futuro y a una perspectiva de 360 grados. Esto exigía superar prácticas y supuestos arraigados, y adoptar nuevas metodologías ágiles que pudieran fomentar la innovación y las soluciones centradas en el usuario.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;03 —&lt;/span&gt;El proceso&lt;/h2&gt;
+&lt;ol&gt;&lt;li&gt;&lt;strong&gt;Planeación y preparación:&lt;/strong&gt; Definimos el desafío y los objetivos del sprint. Seleccionamos un equipo central multidisciplinario y planeamos las actividades de la semana del sprint. Recopilamos información relevante y realizamos entrevistas con stakeholders para comprender el contexto.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Comprensión y definición:&lt;/strong&gt; Realizamos conversaciones estructuradas para crear una base de conocimiento compartida entre los participantes. Mapeamos el desafío y definimos las metas de largo plazo y las preguntas clave por resolver.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Ideación y bocetos:&lt;/strong&gt; Facilitamos ejercicios para generar y refinar una amplia variedad de ideas. Desarrollamos bocetos detallados de posibles soluciones.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Toma de decisiones:&lt;/strong&gt; Evaluamos y seleccionamos las ideas más prometedoras por consenso del equipo. Creamos un flujo de prototipo de alto nivel y diseños detallados de pantallas.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Prototipado:&lt;/strong&gt; Desarrollamos un prototipo realista de la solución elegida. Diseñamos y definimos un guion para presentar el concepto y las funcionalidades.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Validación:&lt;/strong&gt; Probamos el prototipo con cinco stakeholders clave. Recopilamos comentarios para identificar fortalezas y oportunidades de mejora.&lt;/li&gt;&lt;/ol&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;04 —&lt;/span&gt;Impacto&lt;/h2&gt;
+&lt;p&gt;El Design Sprint produjo avances significativos en el enfoque de gestión de activos de Ecopetrol:&lt;/p&gt;
+&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Desarrollo del prototipo:&lt;/strong&gt; Creamos un prototipo funcional que facilitó la visualización en tiempo real de los datos financieros, permitiendo a los gerentes tomar decisiones informadas con base en métricas de desempeño actuales y proyectadas.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Soluciones centradas en el usuario:&lt;/strong&gt; Validamos el prototipo con stakeholders, asegurando que la solución respondiera a las necesidades de los usuarios y a los principales puntos de dolor, como reducir los procesos manuales y fortalecer la toma de decisiones basada en datos.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Alineación estratégica:&lt;/strong&gt; Alineamos la nueva herramienta con la estrategia de largo plazo de Ecopetrol, habilitando un enfoque más proactivo y predictivo de la gestión de activos.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Colaboración fortalecida:&lt;/strong&gt; Fomentamos una cultura colaborativa entre los miembros del equipo, combinando diversas perspectivas para innovar y resolver problemas complejos.&lt;/li&gt;&lt;/ul&gt;
+&lt;p&gt;Este Design Sprint no solo transformó los procesos de gestión de activos financieros en Ecopetrol, sino que también sentó un precedente para futuros proyectos de innovación, destacando el valor de las metodologías ágiles y del diseño centrado en el usuario para impulsar el cambio organizacional.&lt;/p&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
@@ -2509,7 +2828,21 @@
         </is>
       </c>
       <c r="T23" s="2" t="inlineStr"/>
-      <c r="U23" s="2" t="inlineStr"/>
+      <c r="U23" s="2" t="inlineStr">
+        <is>
+          <t>&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;01 —&lt;/span&gt;Situación — El desafío&lt;/h2&gt;
+&lt;p&gt;Como parte del programa &lt;em&gt;Juntos Aprendemos&lt;/em&gt;, y en colaboración con Parque Explora, nos propusimos apoyar a docentes y directivos escolares de Antioquia a afrontar los desafíos posteriores a la pandemia. Muchas aulas habían permanecido estáticas pese a los crecientes cambios tecnológicos, sociales y educativos. Los educadores buscaban maneras de reconectar a los estudiantes y reinventar las experiencias de aprendizaje. Nuestro taller buscaba encender esta transformación mediante intervenciones pequeñas pero poderosas —"hacks"— para reimaginar el aula como un espacio dinámico y participativo de aprendizaje para el siglo XXI.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;02 —&lt;/span&gt;Tarea — Mi rol&lt;/h2&gt;
+&lt;p&gt;Lideré la iniciativa como Head of Innovation, codiseñando y facilitando el taller virtual en alianza con el equipo de Parque Explora. Desarrollé la estructura del taller, la nutrí con metodologías creativas y conduje la sesión con más de 300 educadores. Mi enfoque fue guiar a los participantes a través de un proceso de reflexión, ideación y prototipado, creando un espacio de conexión, creatividad y aprendizaje compartido entre regiones.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;03 —&lt;/span&gt;Acción — El proceso&lt;/h2&gt;
+&lt;p&gt;&lt;strong&gt;Descubrimiento y definición de intenciones.&lt;/strong&gt; Abrimos la sesión sacando a la luz intenciones compartidas: ¿qué hace memorable una experiencia de aprendizaje? Con herramientas colaborativas como Mentimeter, los participantes definieron su propia "EMA" (experiencia memorable de aprendizaje), que sentó la base de sus retos de diseño.&lt;/p&gt;
+&lt;p&gt;&lt;strong&gt;Empatía e inmersión.&lt;/strong&gt; Luego, invitamos a los educadores a ponerse en los zapatos de sus estudiantes. A través de un ejercicio de imaginación guiada, mapearon las experiencias del aula desde la perspectiva del aprendiz, observando comportamientos, emociones e interacciones para identificar necesidades insatisfechas y oportunidades.&lt;/p&gt;
+&lt;p&gt;&lt;strong&gt;Ideación y diseño de hacks.&lt;/strong&gt; Inspirados por preguntas detonantes (por ejemplo, "¿Cómo podríamos reconfigurar el aula para distintos estilos de aprendizaje?"), los participantes propusieron hacks tangibles, desde el aprendizaje basado en proyectos hasta la reorganización del espacio y el intercambio intercultural. Usando Padlet, compartieron, comentaron e iteraron ideas en tiempo real, construyendo un repositorio colectivo de prototipos e inspiración.&lt;/p&gt;
+&lt;p&gt;&lt;strong&gt;Narración y reflexión.&lt;/strong&gt; Para cerrar, los participantes escribieron breves piezas narrativas —"cartas de amor" a sus futuras aulas— que conectaban sus intenciones con las intervenciones propuestas. La sesión terminó con una reflexión compartida sobre cómo las pequeñas acciones pueden generar un cambio sistémico en la educación.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;04 —&lt;/span&gt;Resultado — El impacto&lt;/h2&gt;
+&lt;p&gt;El taller llegó a más de 300 educadores de Antioquia, fomentando un diálogo creativo y nuevas conexiones dentro de una comunidad que aún se estaba recuperando de la pandemia. Aunque se diseñó como un ejercicio de sensibilización, activó una mentalidad de experimentación y empoderó a los docentes para verse a sí mismos como agentes de transformación. Un aprendizaje clave: el cambio sistémico puede comenzar con pequeños hacks intencionales, especialmente cuando se fundamentan en la empatía y en un propósito compartido.&lt;/p&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
@@ -2600,7 +2933,21 @@
         </is>
       </c>
       <c r="T24" s="2" t="inlineStr"/>
-      <c r="U24" s="2" t="inlineStr"/>
+      <c r="U24" s="2" t="inlineStr">
+        <is>
+          <t>&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;01 —&lt;/span&gt;Situación&lt;/h2&gt;
+&lt;p&gt;Después de una década de operación, el Planetario de Medellín necesitaba una renovación profunda para mantenerse vigente en un panorama cultural y educativo cambiante. Su oferta museográfica original, centrada principalmente en la astronomía, ya no resonaba con audiencias cada vez más diversas y críticas. El desafío no era solo modernizar la infraestructura y los contenidos, sino replantear el planetario como un espacio para la reflexión existencial, el diálogo interdisciplinario y la participación pública inclusiva, posicionando la ciencia como herramienta de asombro y, a la vez, como catalizador de la responsabilidad planetaria.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;02 —&lt;/span&gt;Tarea&lt;/h2&gt;
+&lt;p&gt;Me desempeñé como Head of Innovation y lideré al equipo de museografía a lo largo del proceso de conceptualización y diseño de la experiencia. Mi rol incluyó guiar la visión creativa y estratégica, facilitar talleres interdisciplinarios y asegurar la coherencia entre las dimensiones científica, cultural y espacial de la experiencia del visitante. Trabajé de cerca con educadores, científicos, diseñadores y actores de la comunidad para crear una exposición que invita al pensamiento crítico y a la conexión emocional.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;03 —&lt;/span&gt;Acción&lt;/h2&gt;
+&lt;p&gt;&lt;strong&gt;Descubrimiento y encuadre estratégico.&lt;/strong&gt; Comenzamos con una extensa fase de investigación participativa: encuestas a más de 200 visitantes y no visitantes, entrevistas con stakeholders, grupos focales con educadores y líderes comunitarios, y sesiones internas de ideación. Esto nos ayudó a sacar a la luz insights profundos de los usuarios, en especial la necesidad de ir más allá de la ciencia dura hacia un territorio más humano, emocional y filosófico.&lt;/p&gt;
+&lt;p&gt;&lt;strong&gt;Desarrollo del concepto.&lt;/strong&gt; A partir de la investigación, desarrollamos la narrativa central: &lt;em&gt;“Nuestro lugar en el universo”&lt;/em&gt;, no solo como una pregunta científica, sino también humana y existencial. Definimos dos horizontes guía: &lt;strong&gt;Orígenes&lt;/strong&gt; (de dónde venimos) y &lt;strong&gt;Bordes&lt;/strong&gt; (qué hay más allá), para anclar el contenido y la narración espacial. Esta narrativa se construyó para provocar asombro, descentralizar las perspectivas occidentales y reintroducir a los visitantes ante sí mismos como ciudadanos cósmicos.&lt;/p&gt;
+&lt;p&gt;&lt;strong&gt;Codiseño de la experiencia.&lt;/strong&gt; Lideramos múltiples talleres de cocreación con el equipo de Explora, astrónomos, artistas, defensores de la accesibilidad y docentes para definir experiencias multisensoriales e inclusivas. Este proceso puso el énfasis en una interacción que va más allá de lo visual —a través del sonido, la tactilidad, la postura y la narrativa— para que la ciencia sea accesible y significativa para todos los públicos, incluidos niños, adultos mayores y personas con discapacidad.&lt;/p&gt;
+&lt;p&gt;&lt;strong&gt;Integración espacial y narrativa.&lt;/strong&gt; Mi equipo trabajó en traducir conceptos abstractos en experiencias espaciales inmersivas. Desarrollamos una secuencia a lo largo de tres pisos —desde la biodiversidad de la Tierra hasta la escala cósmica— usando herramientas de diseño como constelaciones interactivas, marcadores de distancias planetarias y un mural de gran formato sobre la historia cósmica. Cada zona equilibraba la profundidad científica con la narración artística y la resonancia emocional.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;04 —&lt;/span&gt;Resultado&lt;/h2&gt;
+&lt;p&gt;La propuesta resultante redefinió el Planetario no solo como un recinto de ciencia, sino como un espacio cultural para la reflexión crítica y la imaginación colectiva. Introdujo nuevas formas de accesibilidad, de participación multisensorial y de profundidad narrativa que antes no existían. Un aprendizaje clave: al diseñar para la ciencia, anclar la complejidad en la emoción humana y en el contexto local puede crear experiencias públicas más profundas y transformadoras.&lt;/p&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
@@ -2690,7 +3037,24 @@
       </c>
       <c r="S25" s="2" t="inlineStr"/>
       <c r="T25" s="2" t="inlineStr"/>
-      <c r="U25" s="2" t="inlineStr"/>
+      <c r="U25" s="2" t="inlineStr">
+        <is>
+          <t>&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;01 —&lt;/span&gt;Contexto&lt;/h2&gt;
+&lt;p&gt;El proyecto se centra en la renovación y revitalización del Museo Estación de la Memoria en Puerto Colombia, un lugar con una rica historia de migración y desarrollo cultural. Puerto Colombia, conocido por su histórico muelle y su estación de ferrocarril, ha sido desde el siglo XIX una puerta de entrada fundamental al país y un centro de intercambios culturales y económicos.&lt;/p&gt;
+&lt;p&gt;En 2022, Parque Explora fue seleccionado para diseñar el próximo capítulo del museo mediante un esfuerzo integral de Plan Maestro, con el fin de consolidar un museo para la apropiación pública de la historia del puerto —sus migrantes y colonos, el muelle y su vida cotidiana, la estación y el ferrocarril— y de la huella que este hito dejó en la cultura de Puerto Colombia y en la transformación de Colombia.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;02 —&lt;/span&gt;El desafío&lt;/h2&gt;
+&lt;p&gt;El principal desafío era comprender y documentar las necesidades y percepciones de la comunidad local y de los visitantes frente a la revitalización del museo. El objetivo era identificar los elementos históricos y culturales más relevantes, así como las oportunidades para mejorar la infraestructura y la oferta cultural del museo, asegurando su sostenibilidad y pertinencia en el contexto actual.&lt;/p&gt;
+&lt;blockquote class="c-quote"&gt;A través de historias y memorias vivas, presentes en objetos, documentos de archivo, álbumes familiares, restos de infraestructura y elementos actuales de la mezcla de culturas, los visitantes se sumergirán en el pasado y el presente de un lugar que fue la puerta de entrada a la transformación del país y que hoy se proyecta como símbolo de un desarrollo consciente, sostenible y humano.&lt;/blockquote&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;03 —&lt;/span&gt;Qué hicimos&lt;/h2&gt;
+&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Revisión documental:&lt;/strong&gt; Un análisis extenso de la historia y el patrimonio de Puerto Colombia, así como de los planes de desarrollo locales y nacionales.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Visitas al sitio:&lt;/strong&gt; Visitas al lugar para comprender mejor su estado actual y su potencial.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Entrevistas y talleres:&lt;/strong&gt; Organizamos entrevistas con stakeholders clave y talleres de cocreación con miembros de la comunidad y expertos para recoger perspectivas diversas y construir una visión compartida del proyecto.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Análisis contextual:&lt;/strong&gt; Se desarrollaron diagnósticos sobre el estado normativo y las necesidades de la población local, considerando factores sociales, económicos y culturales.&lt;/li&gt;&lt;/ul&gt;
+&lt;p&gt;Los resultados de esta fase de diagnóstico permitieron:&lt;/p&gt;
+&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Identificación de desafíos y oportunidades:&lt;/strong&gt; Se destacaron aspectos clave, como la importancia de incluir a comunidades diversas y de potenciar el patrimonio vivo de Puerto Colombia.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Base para el diseño del proyecto:&lt;/strong&gt; Se consolidaron ideas y propuestas de intervención museográfica y urbana, alineadas con las necesidades y expectativas de la comunidad.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Participación de la comunidad:&lt;/strong&gt; La participación activa de los habitantes de Puerto Colombia generó un sentido de apropiación y respaldo al proyecto, fundamental para su éxito y sostenibilidad futuros.&lt;/li&gt;&lt;/ul&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;04 —&lt;/span&gt;La propuesta&lt;/h2&gt;
+&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Diseño de experiencias interactivas:&lt;/strong&gt; Propusimos nuevas narrativas y formatos interactivos que integran medios digitales y físicos para enriquecer la experiencia del visitante.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Intervención arquitectónica:&lt;/strong&gt; Planeamos la renovación de la estación y la construcción de nuevos espacios, como un pabellón multipropósito y una pérgola de conexión, para unificar los distintos elementos del sitio.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Museografía ampliada:&lt;/strong&gt; Propusimos extender la experiencia del museo más allá de sus muros con instalaciones y señalización en la plaza y el muelle, creando una ruta cultural accesible y atractiva.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Sostenibilidad y gestión:&lt;/strong&gt; Diseñamos estrategias para asegurar la viabilidad económica y operativa del museo a largo plazo, incluida la búsqueda de alianzas y financiación.&lt;/li&gt;&lt;/ul&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;05 —&lt;/span&gt;Impacto esperado&lt;/h2&gt;
+&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Revitalización del patrimonio:&lt;/strong&gt; La intervención propuesta busca valorar y preservar el patrimonio cultural de Puerto Colombia, convirtiendo el museo en un referente de la historia y la identidad locales.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Inclusión y participación comunitaria:&lt;/strong&gt; Involucrar voces diversas en el diseño y la planeación del proyecto fortalece el sentido de apropiación y la colaboración entre la comunidad y el museo.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Turismo y atractivo cultural:&lt;/strong&gt; La renovación y ampliación del museo posicionan a Puerto Colombia como un destino turístico y cultural destacado, impulsando la economía local y fomentando el desarrollo sostenible.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Innovación educativa:&lt;/strong&gt; Crear experiencias educativas y participativas enriquece la oferta cultural y educativa del museo, en beneficio de estudiantes y visitantes de todas las edades.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
@@ -2770,7 +3134,22 @@
       </c>
       <c r="S26" s="2" t="inlineStr"/>
       <c r="T26" s="2" t="inlineStr"/>
-      <c r="U26" s="2" t="inlineStr"/>
+      <c r="U26" s="2" t="inlineStr">
+        <is>
+          <t>&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;01 —&lt;/span&gt;Contexto&lt;/h2&gt;
+&lt;p&gt;Los rápidos avances en movilidad sostenible y transición energética están transformando el panorama de la industria de estaciones de servicio de combustible (EDS) a nivel global, incluida Colombia. Este estudio de caso se centra en el estado actual y las perspectivas futuras de las estaciones de servicio en Colombia mientras atraviesan esta transición significativa. El contexto inicial incluye una red de aproximadamente 6.000 estaciones de servicio, operadas principalmente por distribuidores pequeños y medianos, con grandes jugadores como Terpel, Primax, Biomax y Chevron dominando el mercado. El objetivo es explorar cómo pueden evolucionar estas estaciones para responder a las demandas de un futuro más verde.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;02 —&lt;/span&gt;El desafío&lt;/h2&gt;
+&lt;p&gt;El principal desafío de la industria de EDS en Colombia es el giro hacia la movilidad sostenible en un entorno que aún depende en gran medida de los combustibles fósiles. Con apenas un 0,2 % de las estaciones ofreciendo carga rápida para vehículos eléctricos, la industria está rezagada en la infraestructura necesaria para la adopción de vehículos eléctricos (VE). Entre los obstáculos clave están convencer a numerosos propietarios de estaciones pequeñas de invertir en nuevas tecnologías, desarrollar una red de carga robusta y atender la baja demanda actual de VE. Además, la industria debe alinearse con las tendencias globales de descarbonización y prepararse para un mercado en el que se espera que predominen los vehículos eléctricos e híbridos.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;03 —&lt;/span&gt;Metodología&lt;/h2&gt;
+&lt;p&gt;Seguí un proceso estructurado compuesto por cuatro etapas clave:&lt;/p&gt;
+&lt;ol&gt;&lt;li&gt;&lt;strong&gt;Plan — Configuración y organización:&lt;/strong&gt; Esta etapa inicial consiste en establecer el marco del proyecto, organizar el cronograma de trabajo y fijar los objetivos de la semana. Asegura una hoja de ruta clara y una gestión eficiente del tiempo para la exploración que sigue.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Explore — Investigación documental, análisis de tendencias y entrevistas con expertos:&lt;/strong&gt; Se realiza una revisión extensa de documentos relevantes y se exploran las tendencias actuales. Se entrevista a dos expertos para obtener insights y reunir perspectivas diversas.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Define — Desarrollo de la estrategia:&lt;/strong&gt; Con base en la información reunida, se define un enfoque estratégico y se identifican las áreas clave de oportunidad. Esta etapa se centra en fijar metas claras y delinear el impacto potencial de las soluciones propuestas.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Imagine — Proyección de conceptos de diseño:&lt;/strong&gt; Se desarrollan y proyectan diversos conceptos de diseño que responden a las oportunidades identificadas. Esta etapa creativa incluye lluvia de ideas, bocetos y refinamiento de ideas para proponer soluciones innovadoras y prácticas.&lt;/li&gt;&lt;/ol&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;04 —&lt;/span&gt;Resultados: reimaginar las estaciones de servicio&lt;/h2&gt;
+&lt;p&gt;Se desarrollaron diversos conceptos de diseño para transformar las estaciones de servicio tradicionales en centros multifuncionales adaptados a la movilidad sostenible. Estos conceptos incluyen torres de carga vehicular que optimizan el espacio, centros de entrega de última milla para zonas urbanas, centros de energía y experiencia que convierten las estaciones en destinos recreativos, y servicios de carga a domicilio para mayor comodidad. Además, se propusieron módulos de estaciones de carga para lugares de alto tráfico, complejos multienergía en carreteras, espacios de trabajo conocidos como "terceros lugares" y estaciones en rutas turísticas verdes. Estos diseños buscan diversificar la oferta de servicios y de energía, mejorar la experiencia del usuario y apoyar la transición hacia un futuro más sostenible.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;05 —&lt;/span&gt;Impacto esperado&lt;/h2&gt;
+&lt;p&gt;Reimaginar las estaciones de servicio genera beneficios significativos en múltiples dimensiones:&lt;/p&gt;
+&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Impacto ambiental:&lt;/strong&gt; El giro hacia la energía eléctrica y renovable reduce la huella de carbono; la integración de paneles solares y turbinas eólicas apoya la sostenibilidad.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Experiencia del cliente:&lt;/strong&gt; Introducción de carga para VE, servicios de alquiler y centros de experiencia; los elementos interactivos y de entretenimiento mejoran las visitas de los clientes.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Beneficios económicos:&lt;/strong&gt; Servicios como el alquiler de VE y la carga a domicilio generan ingresos adicionales; los nuevos servicios y tecnologías crean oportunidades de empleo.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Movilidad sostenible:&lt;/strong&gt; Una red ampliada de cargadores para VE apoya la adopción de vehículos eléctricos; los servicios de carga a domicilio y la infraestructura pública alivian las preocupaciones sobre la autonomía de los VE.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Avances tecnológicos:&lt;/strong&gt; Las apps móviles para servicios e interacción con el cliente mejoran la integración tecnológica; uso eficiente de fuentes de energía renovable.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Alianzas estratégicas:&lt;/strong&gt; Las alianzas público-privadas fomentan soluciones de movilidad sostenible; la colaboración con startups y empresas de tecnología impulsa la innovación.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Preferencias del consumidor:&lt;/strong&gt; La analítica de datos permite ofrecer servicios personalizados y mejora la satisfacción; las opciones de energía verde responden a las expectativas de los consumidores conscientes del medio ambiente.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Viabilidad del negocio:&lt;/strong&gt; La diversificación asegura la viabilidad del negocio a largo plazo; las múltiples opciones de energía y servicios hacen que las estaciones sean más resilientes a los cambios del mercado.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
@@ -2860,7 +3239,20 @@
         </is>
       </c>
       <c r="T27" s="2" t="inlineStr"/>
-      <c r="U27" s="2" t="inlineStr"/>
+      <c r="U27" s="2" t="inlineStr">
+        <is>
+          <t>&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;01 —&lt;/span&gt;El contexto&lt;/h2&gt;
+&lt;p&gt;El edificio &lt;em&gt;Future Seeds&lt;/em&gt; (Semillas del Futuro), parte del Centro Internacional de Agricultura Tropical (CIAT) en Palmira, Colombia, es un sitio de importancia mundial para la conservación de la biodiversidad agrícola. Tradicionalmente un espacio dedicado exclusivamente a la investigación científica, tenía un potencial sin explotar para convertirse en un puente entre la ciencia y la sociedad. En alianza con Parque Explora, el CIAT imaginó transformar este espacio emblemático en un lugar vibrante donde el público pudiera comprender y conectar con el valor de la biodiversidad y la conservación del germoplasma.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;02 —&lt;/span&gt;El desafío&lt;/h2&gt;
+&lt;p&gt;El principal desafío era transformar las áreas subutilizadas del edificio &lt;em&gt;Semillas del Futuro&lt;/em&gt; en espacios educativos y atractivos sin interrumpir sus funciones científicas centrales. El objetivo era abrir las instalaciones a públicos diversos preservando su integridad como centro de investigación, convirtiéndolo en un entorno de doble propósito que apoyara tanto la ciencia rigurosa como una comunicación científica cautivadora.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;03 —&lt;/span&gt;El proceso&lt;/h2&gt;
+&lt;p&gt;Para iniciar la transformación, primero establecimos una colaboración cercana con el equipo científico del CIAT para identificar las narrativas centrales que resonarían tanto con especialistas como con visitantes generales. Entre ellas estaban la importancia de preservar la biodiversidad agrícola, el papel del germoplasma en la seguridad alimentaria y la relevancia global de las instalaciones &lt;em&gt;Future Seeds&lt;/em&gt;. Este diálogo nos permitió fundamentar el proceso de diseño en la precisión científica y, a la vez, traducir temas complejos en historias accesibles y significativas.&lt;/p&gt;
+&lt;p&gt;Con estas narrativas definidas, desarrollamos una estrategia de diseño basada en la idea de una "ciencia que da la bienvenida". Esto significó repensar la manera en que los visitantes se mueven por el edificio y experimentan la información. Identificamos zonas subutilizadas dentro de las instalaciones que podían reconvertirse en espacios interactivos sin interrumpir su flujo operativo. Estas zonas se convirtieron en puntos de encuentro: áreas donde el público podía interactuar con los contenidos a través de experiencias inmersivas y sensoriales.&lt;/p&gt;
+&lt;p&gt;Diseñamos e instalamos tres exhibiciones interactivas que combinaban elementos análogos y digitales. Estas exhibiciones invitaban a los visitantes a explorar la diversidad de las semillas, las técnicas de conservación y el intercambio global de conocimiento agrícola. Cada instalación se elaboró con cuidado para ser intuitiva, atractiva y visualmente convincente, con gráficos, texturas y componentes participativos que cautivaran tanto a públicos no especializados como a visitantes académicos.&lt;/p&gt;
+&lt;p&gt;Las intervenciones gráficas y espaciales se diseñaron para armonizar con el contexto arquitectónico y científico del edificio. En lugar de imponer una capa museográfica tradicional, trabajamos con la materialidad y la circulación existentes del espacio, incorporando elementos interpretativos que se sintieran naturales y respetuosos de la identidad investigativa del edificio.&lt;/p&gt;
+&lt;p&gt;Finalmente, apoyamos la integración de estas nuevas funciones públicas capacitando a los científicos del CIAT como comunicadores de ciencia y mediadores del espacio. Su presencia y participación activa enriquecieron la experiencia del visitante, permitiendo la interpretación, el diálogo y la conexión en tiempo real. Este enfoque centrado en las personas ayudó a tender un puente entre la investigación rigurosa y la comprensión de la sociedad, haciendo que la ciencia cobrara vida para todos.&lt;/p&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
@@ -2953,7 +3345,31 @@
       </c>
       <c r="S28" s="2" t="inlineStr"/>
       <c r="T28" s="2" t="inlineStr"/>
-      <c r="U28" s="2" t="inlineStr"/>
+      <c r="U28" s="2" t="inlineStr">
+        <is>
+          <t>&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;01 —&lt;/span&gt;El contexto&lt;/h2&gt;
+&lt;p&gt;En 2022, el Ministerio de Cultura de Colombia lanzó una iniciativa nacional para crear una red de espacios del Museo de Historia Natural y Cultural de Colombia. El objetivo era fortalecer la apropiación pública de la ciencia y la tecnología y encender una conversación nacional centrada en la vida, la regeneración y la biodiversidad. Mediante una convocatoria pública, se invitó a instituciones culturales, científicas y educativas a presentar propuestas de proyecto viables en solo cuatro semanas. Parque Explora, en colaboración con diversos aliados, aceptó el reto de diseñar y conceptualizar la red nacional.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;02 —&lt;/span&gt;El desafío&lt;/h2&gt;
+&lt;p&gt;El principal desafío era desarrollar, en solo cuatro semanas, una propuesta integral y factible para 12 espacios museales físicos y 6 virtuales en toda Colombia. Esto exigió coordinar a múltiples actores, elaborar una narrativa unificada que resonara en todo el país y crear contenidos y formatos adaptables que respetaran los diversos contextos físicos y sociales de cada lugar.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;03 —&lt;/span&gt;La idea&lt;/h2&gt;
+&lt;p&gt;En su esencia, la Red de espacios del Museo de Historia Natural y Cultural de Colombia (MHNCC) es un llamado a reconocer y celebrar las interconexiones entre las formas de vida, los ecosistemas y las culturas de Colombia. La red se concibió no solo como una serie de exposiciones de museo, sino como una plataforma nacional para regenerar nuestra comprensión y nuestra relación con la naturaleza a través del conocimiento, la emoción y la acción.&lt;/p&gt;
+&lt;p&gt;&lt;strong&gt;Propósito.&lt;/strong&gt; El proyecto busca inspirar un giro colectivo hacia un pensamiento centrado en la vida, animando a los colombianos a explorar la biodiversidad de su territorio y a participar en su cuidado. A través de la ciencia, la narración y el diseño, &lt;em&gt;Biofilia&lt;/em&gt; aspira a despertar la conciencia ecológica y las prácticas regenerativas, arraigadas en las realidades locales y los saberes ancestrales.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;04 —&lt;/span&gt;Enfoque de contenidos&lt;/h2&gt;
+&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Anclarnos a una historia común:&lt;/strong&gt; Historias de origen. Hitos geológicos y culturales que han creado un territorio cambiante y biodiverso.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Regenerar las relaciones y la vida:&lt;/strong&gt; A partir de un llamado a la acción urgente, propone la regeneración del suelo, los bosques y las relaciones socioecológicas.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Nuestro paisaje presente:&lt;/strong&gt; Quiénes somos y cómo vivimos hoy en este territorio compartido. Historias de un presente lleno de relatos naturales y culturales, en torno a la biodiversidad y los desafíos de la resiliencia.&lt;/li&gt;&lt;/ul&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;05 —&lt;/span&gt;Museografía&lt;/h2&gt;
+&lt;p&gt;Entendimos los espacios de la red como un gran sistema compuesto por un conjunto de &lt;strong&gt;elementos museográficos interrelacionados&lt;/strong&gt; que ocurren en un contexto físico y social específico. Esos elementos pueden agruparse temáticamente, con base en un único principio, una gran idea o una serie de conexiones que los hacen coherentes desde una perspectiva informativa.&lt;/p&gt;
+&lt;p&gt;Cada exposición está compuesta por una mezcla de formatos museográficos, resultado tanto de los recursos disponibles para el proyecto como de los propósitos comunicativos y educativos del MHNCC.&lt;/p&gt;
+&lt;h3 class="c-h3"&gt;La modularidad de los formatos&lt;/h3&gt;
+&lt;p&gt;Cada espacio de la red tendrá una mezcla de formatos, con proporciones adaptadas a las oportunidades conceptuales, las fortalezas institucionales, las restricciones operativas y las experiencias del público. Así, un espacio podrá tener una vocación más contemplativa, con una visita rápida y autogestionada, mientras que otro podrá favorecer la participación ciudadana y la construcción colectiva del conocimiento.&lt;/p&gt;
+&lt;h3 class="c-h3"&gt;Tipologías de espacio&lt;/h3&gt;
+&lt;p&gt;Para lograr un sistema museal flexible que pueda adaptarse a las distintas condiciones de los espacios de la red, consideramos dos variables fundamentales: el tamaño del espacio y su permanencia en el tiempo. El cruce de las variables nos permitió establecer tres tipos de espacios:&lt;/p&gt;
+&lt;ul&gt;&lt;li&gt;Espacio S (entre 20 y 50 m²)&lt;/li&gt;&lt;li&gt;Espacio M (entre 50 y 100 m²)&lt;/li&gt;&lt;li&gt;Espacio L (entre 100 y 250 m²)&lt;/li&gt;&lt;/ul&gt;
+&lt;h3 class="c-h3"&gt;Espacios virtuales&lt;/h3&gt;
+&lt;p&gt;Se desarrollará una plataforma digital que servirá como portal para difundir contenidos. También será el lugar donde el público podrá encontrar recursos de la estrategia de e-Learning.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;06 —&lt;/span&gt;De la estrategia al impacto&lt;/h2&gt;
+&lt;ul&gt;&lt;li&gt;La red de espacios es hoy una realidad conocida como &lt;em&gt;Alianza Biofilia&lt;/em&gt;.&lt;/li&gt;&lt;li&gt;Se implementó con éxito un sistema museográfico flexible que celebra la diversidad biológica y cultural de Colombia.&lt;/li&gt;&lt;li&gt;Se fortalecieron las alianzas estratégicas y las capacidades locales en comunicación de la ciencia.&lt;/li&gt;&lt;li&gt;Se logró una participación pública significativa con la ciencia en regiones históricamente desatendidas.&lt;/li&gt;&lt;li&gt;Se alcanzó una integración fluida entre los formatos museales físicos y digitales.&lt;/li&gt;&lt;li&gt;Se estableció el proyecto como un referente de innovación museal y diseño estratégico en América Latina.&lt;/li&gt;&lt;li&gt;Se demostró el poder del diseño colaborativo para abordar desafíos complejos con impacto nacional.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
@@ -3050,7 +3466,27 @@
         </is>
       </c>
       <c r="T29" s="2" t="inlineStr"/>
-      <c r="U29" s="2" t="inlineStr"/>
+      <c r="U29" s="2" t="inlineStr">
+        <is>
+          <t>&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;01 —&lt;/span&gt;Contexto&lt;/h2&gt;
+&lt;p&gt;El proyecto Parque de Aves y Agricultura Regenerativa se ubica en la Hacienda Piedechinche, en El Cerrito, Valle del Cauca. Este parque busca fusionar la conservación de la biodiversidad, en particular de las aves, con prácticas agrícolas regenerativas, creando un espacio para el aprendizaje y el turismo sostenibles. La iniciativa es una colaboración entre el Ingenio Providencia y Audubon Américas, con el objetivo de promover la sostenibilidad ambiental, la educación y la integración comunitaria.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;02 —&lt;/span&gt;El desafío&lt;/h2&gt;
+&lt;p&gt;El principal desafío del proyecto era armonizar la producción agrícola tradicional con la conservación de la biodiversidad, especialmente de las aves. El proyecto debía adaptar prácticas agrícolas regenerativas asegurando al mismo tiempo la protección y promoción de las especies de aves locales. Hubo dificultades específicas para conseguir financiación, garantizar la seguridad del público y crear experiencias atractivas para audiencias diversas. Además, integrar estas prácticas dentro del contexto cultural e histórico existente de la Hacienda añadió otra capa de complejidad.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;03 —&lt;/span&gt;Qué hicimos&lt;/h2&gt;
+&lt;ul&gt;&lt;li&gt;Realizamos visitas al sitio y talleres estratégicos.&lt;/li&gt;&lt;li&gt;Sostuvimos entrevistas con stakeholders clave, entre ellos líderes comunitarios, grupos ambientalistas y expertos en turismo.&lt;/li&gt;&lt;li&gt;Desarrollamos un taller de cocreación y pensamiento estratégico para comprender y proyectar la visión del parque.&lt;/li&gt;&lt;li&gt;Mapeamos el territorio para identificar oportunidades y desafíos.&lt;/li&gt;&lt;li&gt;Colaboramos con universidades y organizaciones locales para diseñar e implementar parcelas agrícolas regenerativas.&lt;/li&gt;&lt;li&gt;Integramos la infraestructura existente con nuevas intervenciones arquitectónicas sostenibles.&lt;/li&gt;&lt;li&gt;Desarrollamos experiencias interactivas e inmersivas para los visitantes.&lt;/li&gt;&lt;li&gt;Diseñamos estrategias digitales para mantener la conexión con audiencias diversas.&lt;/li&gt;&lt;/ul&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;04 —&lt;/span&gt;El plan maestro&lt;/h2&gt;
+&lt;p&gt;El plan maestro del proyecto Parque de Aves y Agricultura Regenerativa integró con éxito diversos componentes estratégicos y creó un marco integral que hace énfasis en la sostenibilidad ambiental, la educación y la participación comunitaria. Delineó el desarrollo de múltiples áreas temáticas, entre ellas espacios contemplativos, escenarios regenerativos, ambientaciones museográficas y entornos experimentales. El plan también incorporó la infraestructura existente, asegurando la conectividad ecológica y principios de diseño modulares y sistémicos. Entre los resultados clave están el establecimiento de experiencias inmersivas e interactivas para los visitantes, la creación de parcelas demostrativas de agricultura regenerativa y la construcción de espacios arquitectónicos innovadores como pasarelas elevadas, observatorios de aves y pabellones multipropósito. El plan busca que el parque sea un líder regional en conservación, investigación, educación y turismo de naturaleza, fomentando al mismo tiempo las prácticas sostenibles y la inclusión de la comunidad.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;05 —&lt;/span&gt;Impacto esperado&lt;/h2&gt;
+&lt;h3 class="c-h3"&gt;Ambiental&lt;/h3&gt;
+&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Conservación de la biodiversidad:&lt;/strong&gt; Proteger y mejorar los hábitats de especies de aves residentes y migratorias mediante prácticas agrícolas sostenibles.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Restauración ecológica:&lt;/strong&gt; Implementar agricultura regenerativa para restaurar ecosistemas, mejorar la salud del suelo y promover el equilibrio ecológico.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Prácticas sostenibles:&lt;/strong&gt; Demostrar la viabilidad de combinar la agricultura con la conservación, sirviendo como modelo para iniciativas similares.&lt;/li&gt;&lt;/ul&gt;
+&lt;h3 class="c-h3"&gt;Educativo&lt;/h3&gt;
+&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Oportunidades de aprendizaje:&lt;/strong&gt; Ofrecer programas educativos y experiencias interactivas para visitantes, colegios y universidades, promoviendo la conciencia sobre la biodiversidad y la agricultura sostenible.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Participación de la comunidad:&lt;/strong&gt; Fomentar una comprensión y valoración más profundas de los problemas ambientales locales y globales mediante talleres y actividades de ciencia participativa.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Investigación e innovación:&lt;/strong&gt; Crear un laboratorio vivo para la investigación en agricultura regenerativa y conservación de la biodiversidad, impulsando alianzas académicas e innovación.&lt;/li&gt;&lt;/ul&gt;
+&lt;h3 class="c-h3"&gt;Económico&lt;/h3&gt;
+&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Desarrollo turístico:&lt;/strong&gt; Posicionar el parque como un destino de primer nivel para el ecoturismo y el avistamiento de aves, atrayendo visitantes nacionales e internacionales.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Generación de empleo:&lt;/strong&gt; Generar oportunidades de empleo en los sectores de conservación, agricultura, turismo y educación, apoyando el crecimiento económico local.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Valor agregado:&lt;/strong&gt; Aumentar el valor económico de los productos agrícolas mediante prácticas sostenibles y ecocertificaciones.&lt;/li&gt;&lt;/ul&gt;
+&lt;h3 class="c-h3"&gt;Social&lt;/h3&gt;
+&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Empoderamiento comunitario:&lt;/strong&gt; Empoderar a las comunidades locales involucrándolas en la gestión y las actividades del parque, promoviendo la cohesión social y el sentido de apropiación.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Preservación cultural:&lt;/strong&gt; Integrar el rico patrimonio cultural e histórico de la región en la narrativa del parque, preservando y celebrando las tradiciones y saberes locales.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Salud y bienestar:&lt;/strong&gt; Ofrecer un entorno sereno y educativo para los visitantes, que contribuya al bienestar mental y físico mediante actividades basadas en la naturaleza.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
@@ -3145,7 +3581,21 @@
         </is>
       </c>
       <c r="T30" s="2" t="inlineStr"/>
-      <c r="U30" s="2" t="inlineStr"/>
+      <c r="U30" s="2" t="inlineStr">
+        <is>
+          <t>&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;01 —&lt;/span&gt;La situación&lt;/h2&gt;
+&lt;p&gt;Artista de Archivo fue originalmente una instalación interactiva alojada en el Museo Cámara de Maravillas, parte de la Biblioteca Pública Piloto de Medellín. Diseñada para acercar a los visitantes a contenidos de archivo mediante herramientas de composición creativa, la exposición invitaba a los usuarios a remezclar fragmentos visuales de la memoria cultural de Colombia. Con la llegada de la pandemia de COVID-19, el proyecto enfrentó un desafío crítico: cómo traducir esta experiencia de museo, basada en el hacer, en una interacción digital significativa y accesible, en un momento en que las instituciones culturales buscaban con urgencia nuevas estrategias para seguir conectadas con sus audiencias.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;02 —&lt;/span&gt;La tarea&lt;/h2&gt;
+&lt;p&gt;Lideré la adaptación estratégica y de diseño de la experiencia, guiando su transición de una interfaz de museo físico a una plataforma web intuitiva y atractiva. Mis responsabilidades incluyeron el mapeo de la experiencia, la definición de UX/UI, la validación de usabilidad y la articulación de una estrategia de comunicación para asegurar la participación de la audiencia en el espacio digital.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;03 —&lt;/span&gt;El proceso&lt;/h2&gt;
+&lt;p&gt;El proceso de transformación comenzó con un taller de cocreación para identificar qué aspectos de la experiencia original debían reinterpretarse para los entornos digitales. Establecimos tres pilares de adaptación: simplificación de los contenidos, rediseño de la interfaz para un uso responsivo y optimización de la usabilidad con base en heurísticas web. Todos los recursos gráficos se reconstruyeron para un buen desempeño digital, y el flujo del usuario se rediseñó como una experiencia guiada paso a paso, optimizada para móvil.&lt;/p&gt;
+&lt;p&gt;Desarrollamos un prototipo funcional con Elementor dentro de WordPress y realizamos una prueba de Escala de Usabilidad del Sistema (SUS) con 17 participantes. Los insights de estas sesiones llevaron a refinamientos clave de la interfaz y a mejoras de accesibilidad.&lt;/p&gt;
+&lt;h3 class="c-h3"&gt;Pruebas de usabilidad e iteración&lt;/h3&gt;
+&lt;p&gt;La experiencia final permitía a los usuarios crear composiciones personalizadas —cartas, portadas de libros, sellos ex libris— e integraba animaciones lúdicas y funciones para compartir en redes sociales. Paralelamente, desarrollamos una hoja de ruta de comunicaciones con campañas y eventos digitales para promover la participación del público y la participación creativa.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;04 —&lt;/span&gt;El resultado&lt;/h2&gt;
+&lt;p&gt;El relanzamiento digital de Artista de Archivo amplió con éxito el alcance del museo durante un periodo de cierre físico, preservando al mismo tiempo su esencia interactiva y educativa. El proyecto fortaleció la presencia digital de la institución y sentó un precedente para las experiencias culturales híbridas. Para mí, fue una clara demostración de cómo el diseño puede movilizar la memoria, la creatividad y la participación ciudadana, incluso en tiempos de disrupción.&lt;/p&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
@@ -3236,7 +3686,21 @@
         </is>
       </c>
       <c r="T31" s="2" t="inlineStr"/>
-      <c r="U31" s="2" t="inlineStr"/>
+      <c r="U31" s="2" t="inlineStr">
+        <is>
+          <t>&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;01 —&lt;/span&gt;Contexto&lt;/h2&gt;
+&lt;p&gt;El Centro de Ciencia EUREKA es un proyecto propuesto que busca establecer un centro de cultura, ciencia, tecnología e innovación en Cúcuta, Colombia, y en la región fronteriza colombo-venezolana. El proyecto busca fortalecer la alfabetización científica, el enriquecimiento cultural y el desarrollo comunitario, transformando así el panorama socioeconómico local.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;02 —&lt;/span&gt;El desafío&lt;/h2&gt;
+&lt;p&gt;El principal desafío era diseñar un plan maestro que respondiera a las complejidades socioculturales y logísticas de la región fronteriza. El proyecto debía:&lt;/p&gt;
+&lt;ul&gt;&lt;li&gt;Comprender e integrar las necesidades y aspiraciones de la comunidad.&lt;/li&gt;&lt;li&gt;Asegurar que el diseño y las actividades del centro sean relevantes y atractivos.&lt;/li&gt;&lt;li&gt;Alinearse con los planes de desarrollo urbano y regional existentes.&lt;/li&gt;&lt;li&gt;Fomentar la colaboración y la integración transfronterizas.&lt;/li&gt;&lt;/ul&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;03 —&lt;/span&gt;Qué hicimos&lt;/h2&gt;
+&lt;p&gt;Realizamos un proceso integral de planificación maestra para el Centro de Ciencia EUREKA, que incluyó un taller de pensamiento estratégico con líderes locales y miembros de la comunidad, encuestas detalladas y entrevistas a profundidad con usuarios para recoger insights sobre las expectativas y necesidades de la comunidad. Analizamos más de 24 documentos existentes para extraer datos relevantes, realizamos más de 25 entrevistas con stakeholders para identificar oportunidades y produjimos entregables estratégicos clave, entre ellos un Diagnóstico y un Informe final de Definición. Además, realizamos un análisis contextual y espacial para asegurar que el diseño del centro se alinee con los marcos regionales y las necesidades de la comunidad.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;04 —&lt;/span&gt;Los resultados&lt;/h2&gt;
+&lt;p&gt;El proyecto definió estrategias arquitectónicas y de diseño para crear un espacio atractivo, funcional y educativo. También delineó el programa ASCTI de modelos operativos, con énfasis en la sostenibilidad y la gestión autónoma. El centro busca promover la diversidad cultural, la inclusión social y la participación de la comunidad. Conceptualmente, EUREKA abraza la idea de una "frontera difusa" como zona de transición, un "contexto ampliado" para conectar perspectivas locales y globales, una "identidad ambiental" que reconoce a los seres humanos como parte del ecosistema y un "conocimiento abierto" que fusiona las ciencias tradicionales con el arte y la cultura. Temáticamente, abarca la vida inteligente, la cultura, la ecología, el medio ambiente, la ciencia y la tecnología. Espacialmente, EUREKA está diseñado para ser permeable, adaptable, ampliado, progresivo y afectivo, integrándose con el entorno y fomentando la participación de la comunidad.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;05 —&lt;/span&gt;Impacto esperado&lt;/h2&gt;
+&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Enriquecimiento educativo y cultural:&lt;/strong&gt; Estimular la curiosidad científica, mejorar los resultados educativos y promover el enriquecimiento cultural para fomentar una comunidad científicamente alfabetizada y culturalmente consciente.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Desarrollo comunitario:&lt;/strong&gt; Contribuir al desarrollo social y económico de la región fronteriza creando oportunidades de interacción social, construcción de comunidad y crecimiento económico mediante actividades educativas y culturales.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Integración transfronteriza:&lt;/strong&gt; Fomentar la colaboración y la integración entre Colombia y Venezuela para fortalecer las relaciones transfronterizas, promover el entendimiento mutuo y crear un sentido compartido de identidad regional.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Conciencia ambiental:&lt;/strong&gt; Promover la conciencia ambiental y la sostenibilidad impulsando prácticas sostenibles, generando conciencia sobre los problemas ambientales e integrando la educación ecológica en la comunidad.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Visión estratégica y participación de stakeholders:&lt;/strong&gt; Desarrollar una visión clara y compartida del Centro de Ciencia EUREKA, alineada con los planes de desarrollo regional y las aspiraciones de la comunidad, asegurando que el centro responda a las necesidades y expectativas de esta.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Diseño centrado en la comunidad:&lt;/strong&gt; Asegurar que el diseño y la planeación del centro se fundamenten en las necesidades y expectativas de la comunidad, creando un espacio acogedor, atractivo y relevante que mejore la experiencia general del usuario y fomente una participación de largo plazo.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
@@ -3312,7 +3776,18 @@
       </c>
       <c r="S32" s="2" t="inlineStr"/>
       <c r="T32" s="2" t="inlineStr"/>
-      <c r="U32" s="2" t="inlineStr"/>
+      <c r="U32" s="2" t="inlineStr">
+        <is>
+          <t>&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;01 —&lt;/span&gt;El contexto&lt;/h2&gt;
+&lt;p&gt;Ante los desafíos sin precedentes que planteó la pandemia de COVID-19, Parque Explora inició en 2020 un proceso de transformación estratégica llamado "Compás Estratégico". Esta iniciativa buscaba &lt;strong&gt;reimaginar el rol y las operaciones de la organización en un momento de crisis, con foco en abordar los desafíos de la sociedad, adaptarse a nuevas realidades y asegurar la sostenibilidad a largo plazo.&lt;/strong&gt; A través de sesiones colaborativas, la organización buscó redefinir su propósito, identificar prioridades críticas y prepararse para distintos escenarios futuros, sin perder su misión de promover la educación, la cultura y la ciencia.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;02 —&lt;/span&gt;El desafío&lt;/h2&gt;
+&lt;p&gt;La pandemia trajo consigo disrupciones significativas, entre ellas la reducción del turismo cultural, la inestabilidad financiera y el aumento de las desigualdades sociales. Parque Explora enfrentó la caída de los ingresos por venta de entradas y alianzas, un contacto físico limitado con sus audiencias y la necesidad de adaptarse rápidamente a las plataformas digitales. Además, la organización tuvo que atender desafíos internos como derribar los silos, fomentar la colaboración y construir resiliencia para navegar con eficacia un futuro incierto.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;03 —&lt;/span&gt;El proceso&lt;/h2&gt;
+&lt;p&gt;El proceso de transformación se estructuró en tres sesiones de pensamiento estratégico: definir una narrativa de propósito, imaginar un futuro reimaginado e identificar estrategias accionables. Mediante ciclos iterativos de aprendizaje y adaptación, el equipo exploró escenarios posibles —desde una contracción económica prolongada hasta una recuperación rápida— y sus implicaciones para la organización. Entre las actividades clave estuvieron el mapeo de las capacidades organizacionales, la alineación de los recursos con las oportunidades emergentes y el desarrollo de una hoja de ruta para la agilidad y la resiliencia. Las sesiones hicieron énfasis en la colaboración, la creatividad y el pensamiento sistémico para asegurar la alineación con la misión de Parque Explora y su adaptabilidad a condiciones cambiantes.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;04 —&lt;/span&gt;El impacto&lt;/h2&gt;
+&lt;p&gt;La iniciativa "Compás Estratégico" dio como resultado un marco claro de cinco prioridades estratégicas: potenciar el impacto en la comunidad, consolidar un ecosistema transmedia, fortalecer las alianzas para la sostenibilidad, identificar los recursos y capacidades críticos, y convertirse en una organización más ágil y resiliente. Estas prioridades se respaldaron con metas accionables, como ampliar la oferta digital, fomentar la inclusión y mejorar la flexibilidad operativa. El proceso también puso de relieve la importancia de aprovechar la tecnología, formar nuevas alianzas y abordar barreras como la resistencia al cambio. Al prepararse para múltiples escenarios, Parque Explora se posicionó para navegar la incertidumbre y, a la vez, reafirmar su rol como líder en educación, cultura y ciencia.&lt;/p&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
@@ -3397,7 +3872,23 @@
       </c>
       <c r="S33" s="2" t="inlineStr"/>
       <c r="T33" s="2" t="inlineStr"/>
-      <c r="U33" s="2" t="inlineStr"/>
+      <c r="U33" s="2" t="inlineStr">
+        <is>
+          <t>&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;01 —&lt;/span&gt;El contexto&lt;/h2&gt;
+&lt;p&gt;La pandemia de COVID-19 ha planteado desafíos sin precedentes para los museos de todo el mundo, incluido Parque Explora. Dependientes tradicionalmente de la venta de entradas, de la financiación estatal de proyectos y del apoyo del sector privado, los museos enfrentaron una presión financiera inmediata al cancelarse las agendas, congelarse los recursos del Estado y sobrevolar el riesgo de cierre.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;02 —&lt;/span&gt;El desafío&lt;/h2&gt;
+&lt;p&gt;El principal desafío era adaptarse a un entorno que cambiaba rápidamente y con altos niveles de incertidumbre, garantizando la seguridad y la confianza de los visitantes y manteniendo al mismo tiempo la viabilidad operativa y financiera del museo. Esto exigió replantear por completo cómo relacionarse con el público, gestionar los espacios y sostener las actividades del museo durante la pandemia y después de ella.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;03 —&lt;/span&gt;El proceso&lt;/h2&gt;
+&lt;p&gt;Para abordar estos desafíos, Parque Explora implementó una estrategia multifacética:&lt;/p&gt;
+&lt;p&gt;&lt;strong&gt;Establecer una estructura de respuesta a la crisis.&lt;/strong&gt; Conformó un equipo multidisciplinario para asegurar respuestas ágiles, flexibles y creativas ante la crisis, incorporando liderazgo y capacidades organizacionales para anticipar eventos y construir visiones compartidas.&lt;/p&gt;
+&lt;p&gt;&lt;strong&gt;Crear un modelo operativo flexible.&lt;/strong&gt; Diseñó un modelo adaptativo que podía expandirse y contraerse según las dinámicas locales y nacionales, con protocolos, comunicaciones, estrategias comerciales y ajustes de infraestructura.&lt;/p&gt;
+&lt;p&gt;&lt;strong&gt;Implementar protocolos de seguridad.&lt;/strong&gt; Desarrolló protocolos de seguridad integrales para visitantes y personal, que incluían medidas de higiene, distanciamiento social y lineamientos operativos para garantizar un entorno seguro.&lt;/p&gt;
+&lt;p&gt;&lt;strong&gt;Plan de reapertura por fases.&lt;/strong&gt; Estructuró una estrategia de reapertura por fases, priorizando las áreas y actividades con menor riesgo de contagio y aumentando gradualmente la capacidad operativa, a la vez que adaptaba los espacios a los nuevos requisitos de salud y seguridad.&lt;/p&gt;
+&lt;p&gt;&lt;strong&gt;Pruebas piloto.&lt;/strong&gt; Realizó pruebas piloto con el personal interno y con grupos específicos de público para evaluar y refinar el modelo operativo antes de su implementación a gran escala.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;04 —&lt;/span&gt;Impacto esperado&lt;/h2&gt;
+&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Seguridad y confianza de los visitantes:&lt;/strong&gt; Al garantizar el estricto cumplimiento de los protocolos de salud y seguridad, el museo busca reconstruir la confianza de los visitantes y crear un entorno seguro para la participación del público.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Resiliencia operativa:&lt;/strong&gt; El modelo operativo flexible está diseñado para resistir futuras disrupciones, permitiendo que el museo se adapte rápidamente a circunstancias cambiantes y mantenga su continuidad.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Participación sostenible:&lt;/strong&gt; Los contenidos digitales mejorados y los planes de reapertura por fases buscan sostener el interés y la participación del público, asegurando que el museo siga siendo relevante y accesible.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Apoyo e inclusión de la comunidad:&lt;/strong&gt; La participación activa de las comunidades locales y los stakeholders en la planeación y ejecución fomenta un sentido de apropiación y respaldo a las iniciativas del museo.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Viabilidad a largo plazo:&lt;/strong&gt; La estrategia integral, que incluye la planeación financiera y la creación de nuevas fuentes de ingresos, busca asegurar la salud financiera y la sostenibilidad del museo a largo plazo.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
@@ -3478,7 +3969,19 @@
       </c>
       <c r="S34" s="2" t="inlineStr"/>
       <c r="T34" s="2" t="inlineStr"/>
-      <c r="U34" s="2" t="inlineStr"/>
+      <c r="U34" s="2" t="inlineStr">
+        <is>
+          <t>&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;01 —&lt;/span&gt;El contexto&lt;/h2&gt;
+&lt;p&gt;El Ministerio de Educación Nacional (MEN), la Organización de Estados Iberoamericanos (OEI) y Parque Explora de Medellín colaboraron en una iniciativa estratégica orientada a crear un marco integral de educación STEM+ para Colombia. Esta iniciativa se diseñó para fomentar la innovación y dotar a los estudiantes de las habilidades del siglo XXI necesarias para prosperar en un mundo que cambia con rapidez. El proyecto, titulado "Supernova, Aprendizaje Expandido", se concibió para atender los desafíos educativos que plantearon la pandemia de COVID-19 y la Cuarta Revolución Industrial, asegurando que los estudiantes colombianos estén bien preparados para el futuro.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;02 —&lt;/span&gt;El desafío&lt;/h2&gt;
+&lt;p&gt;Colombia enfrentaba varios desafíos para integrar la educación STEM en su diverso panorama educativo. Entre ellos:&lt;/p&gt;
+&lt;ol&gt;&lt;li&gt;&lt;strong&gt;Disparidades en el acceso:&lt;/strong&gt; Garantizar que estudiantes de distintos contextos socioeconómicos tengan igual acceso a la educación STEM y a sus recursos.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Integración curricular:&lt;/strong&gt; Desarrollar un currículo cohesivo y flexible que integre las disciplinas STEM con otras asignaturas.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Formación docente:&lt;/strong&gt; Ofrecer desarrollo profesional continuo a los docentes para que impartan la educación STEM de manera efectiva.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Participación de la comunidad:&lt;/strong&gt; Involucrar a las familias y a las comunidades locales en el proceso educativo para apoyar y potenciar el aprendizaje.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Inclusión de género:&lt;/strong&gt; Promover la equidad de género en los campos STEM fomentando la participación de niñas y mujeres jóvenes.&lt;/li&gt;&lt;/ol&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;03 —&lt;/span&gt;Impacto esperado&lt;/h2&gt;
+&lt;ol&gt;&lt;li&gt;&lt;strong&gt;Mayor claridad estratégica:&lt;/strong&gt; Establecer una visión y una misión unificadas que lleven a acciones más coherentes e impactantes. Mejorar la alineación de los proyectos con los objetivos organizacionales.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Inclusión de género:&lt;/strong&gt; Promover la equidad de género en los campos STEM mediante programas dirigidos a niñas y mujeres jóvenes. Fomentar la participación y el liderazgo femeninos en las disciplinas STEM.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Participación de la comunidad:&lt;/strong&gt; Involucrar a las familias y a las comunidades locales en el proceso educativo para crear un entorno de aprendizaje de apoyo. Fortalecer el tejido social fomentando la colaboración y las metas compartidas.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Aprendizaje a lo largo de la vida:&lt;/strong&gt; Fomentar el aprendizaje permanente y el desarrollo profesional continuo entre educadores y estudiantes.&lt;/li&gt;&lt;/ol&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;04 —&lt;/span&gt;Conclusión&lt;/h2&gt;
+&lt;p&gt;Esta iniciativa estratégica, liderada por el MEN, la OEI y Parque Explora, representa un paso significativo hacia la transformación de la educación STEM en Colombia. Al abordar los desafíos y aprovechar las fortalezas de diversos actores, el proyecto busca crear un marco STEM+ robusto e inclusivo que prepare a los estudiantes para el futuro, fomente la innovación y promueva el desarrollo sostenible. Este esfuerzo colaborativo no solo mejora la calidad de la educación, sino que también contribuye al crecimiento socioeconómico general del país.&lt;/p&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
@@ -3570,7 +4073,22 @@
         </is>
       </c>
       <c r="T35" s="2" t="inlineStr"/>
-      <c r="U35" s="2" t="inlineStr"/>
+      <c r="U35" s="2" t="inlineStr">
+        <is>
+          <t>&lt;blockquote class="c-quote"&gt;Fortalecimiento de la infraestructura pública de ciencia en el Valle del Cauca, Colombia&lt;/blockquote&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;01 —&lt;/span&gt;Situación — El desafío&lt;/h2&gt;
+&lt;p&gt;Después de más de una década de operación, dos grandes centros de ciencia del Valle del Cauca —el Museo de Historia Natural y Cultural del Valle del Cauca (operado por el INCIVA) y el Museo Interactivo Abracadabra (operado por la Biblioteca Departamental)— enfrentaban una relevancia en declive. Su museografía se había quedado obsoleta, la infraestructura técnica estaba desactualizada y los contenidos educativos ya no reflejaban las narrativas científicas contemporáneas. Aunque ambas instituciones compartían el mismo complejo público, &lt;em&gt;La Manzana del Saber&lt;/em&gt;, sus experiencias estaban fragmentadas a nivel arquitectónico, operativo y organizacional. Esta fragmentación debilitaba la colaboración, la gobernanza y la experiencia general del visitante, en un momento en que Colciencias (hoy MinCiencias) priorizaba el fortalecimiento de los centros de ciencia en todo el país.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;02 —&lt;/span&gt;Tarea — Mi rol&lt;/h2&gt;
+&lt;p&gt;Formé parte del liderazgo de diseño estratégico del proyecto, y ayudé a articular una visión compartida entre ambas instituciones y a alinear a diversos stakeholders en torno a un modelo de experiencia unificado. Trabajé de cerca con directores institucionales, equipos curatoriales, educadores, arquitectos y aliados del sector público para enmarcar el desafío de manera integral. Mi responsabilidad abarcó el encuadre estratégico, la visualización de la experiencia y el liderazgo metodológico en educación, infraestructura, gobernanza y contenidos. También tuve un papel clave en la orquestación de líneas de trabajo paralelas de gran escala para asegurar la coherencia entre disciplinas.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;03 —&lt;/span&gt;Acción — El proceso&lt;/h2&gt;
+&lt;p&gt;&lt;strong&gt;Diagnóstico y definición de la línea base.&lt;/strong&gt; Comenzamos con una fase integral de diagnóstico de 360° para establecer un entendimiento compartido del estado actual. Esto incluyó la evaluación de la museografía, los modelos educativos, la infraestructura física y técnica, la colaboración organizacional y las estructuras de gobernanza. Esta línea base, sustentada en evidencia, se convirtió en el fundamento de todas las decisiones posteriores.&lt;/p&gt;
+&lt;p&gt;&lt;strong&gt;Experiencia unificada y alineación estratégica.&lt;/strong&gt; A través de talleres y sesiones de cocreación, alineamos a ambas instituciones en torno a la idea de una única experiencia integrada de centro de ciencia, que más adelante se llamó &lt;strong&gt;MALVA&lt;/strong&gt;. Esto exigió replantear el proyecto más allá del diseño de exposiciones, para incluir modelos de aprendizaje, colaboración operativa y gobernanza de largo plazo.&lt;/p&gt;
+&lt;p&gt;&lt;strong&gt;Diseño concurrente y desarrollo de contenidos.&lt;/strong&gt; Con un equipo multidisciplinario de más de 30 profesionales trabajando en paralelo, desarrollamos formatos museográficos, conceptos arquitectónicos, estrategias de mediación y narrativas científicas. Las nuevas áreas de contenido incluyeron las ciencias de la Tierra y del espacio, la biodiversidad, zonas de experimentación y laboratorios creativos públicos, todas diseñadas para fomentar la participación y el aprendizaje intergeneracional.&lt;/p&gt;
+&lt;p&gt;&lt;strong&gt;Modelo de gobernanza y sostenibilidad.&lt;/strong&gt; En paralelo, definimos un nuevo modelo de colaboración y gobernanza que permitiera una coordinación sostenida entre las instituciones. Esto aseguró que la experiencia unificada estuviera respaldada no solo por el diseño, sino por estructuras organizacionales y estratégicas capaces de mantenerla en el tiempo.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;04 —&lt;/span&gt;Resultado — El impacto&lt;/h2&gt;
+&lt;p&gt;MALVA se convirtió en un centro de ciencia integrado, completamente diseñado y en buena parte implementado, que unificó con éxito dos instituciones antes fragmentadas en una experiencia pública coherente. El proyecto renovó las narrativas científicas, modernizó la infraestructura e introdujo formas más participativas, familiares e inclusivas de relacionarse con la ciencia. Más allá de la transformación física, MALVA propició una colaboración institucional más sólida y posicionó a &lt;em&gt;La Manzana del Saber&lt;/em&gt; como un ecosistema contemporáneo de ciencia y aprendizaje, orientado al futuro, lo que demuestra cómo el diseño estratégico puede generar valor público de largo plazo.&lt;/p&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
@@ -3664,7 +4182,24 @@
         </is>
       </c>
       <c r="T36" s="2" t="inlineStr"/>
-      <c r="U36" s="2" t="inlineStr"/>
+      <c r="U36" s="2" t="inlineStr">
+        <is>
+          <t>&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;01 —&lt;/span&gt;Situación&lt;/h2&gt;
+&lt;p&gt;La Autoridad del Canal de Panamá buscaba profundizar el entendimiento nacional sobre la importancia histórica, ecológica y geopolítica del Canal, en particular entre las comunidades del interior del país, históricamente desconectadas de él. Para lograrlo, lanzó un concurso para conceptualizar un nuevo centro de visitantes interactivo en Santiago de Veraguas, una región elegida estratégicamente por su ubicación en el centro del país. El desafío: hacer tangibles, participativas y significativas para todos los panameños la relevancia global del Canal y su impacto local.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;02 —&lt;/span&gt;Tarea&lt;/h2&gt;
+&lt;p&gt;Como Senior Exhibit Designer dentro del equipo de Parque Explora, tuve un papel clave en dar forma a la visión conceptual y a la estrategia de narración interactiva de la propuesta. Me enfoqué en alinear las narrativas espaciales con los objetivos de participación de la comunidad, asegurando que las decisiones de diseño resonaran con audiencias diversas y comunicaran el valor del Canal más allá de su función económica. Mis aportes abarcaron desde la ideación temprana hasta el desarrollo del concepto, integrando en todo momento la investigación participativa y la planeación interpretativa.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;03 —&lt;/span&gt;Acción&lt;/h2&gt;
+&lt;p&gt;Abordamos el proyecto como un puente tanto espacial como cultural, creando un recorrido para el visitante que invita a las personas a sentirse dentro del Canal. El concepto incluía seis galerías temáticas y 18 experiencias interactivas, que combinaban medios análogos, digitales e híbridos.&lt;/p&gt;
+&lt;p&gt;Los visitantes podían explorar los orígenes geológicos del istmo, la biodiversidad de sus ecosistemas y los hitos de ingeniería de la construcción y ampliación del Canal. Para desarrollar contenidos con arraigo local, realizamos investigación de campo participativa en la región y usamos metodologías de cocreación para sacar a la luz las perspectivas de la comunidad.&lt;/p&gt;
+&lt;p&gt;Esto orientó el tono del centro, los formatos de medios y los modos de interacción. A través de una narración inmersiva, tradujimos temas complejos —como la geopolítica, la gestión del agua y el comercio global— en formatos atractivos y accesibles para todas las edades.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;04 —&lt;/span&gt;Resultado&lt;/h2&gt;
+&lt;p&gt;Nuestra propuesta ganó el concurso nacional, dando inicio a la fase de diseño detallado del Centro de Experiencia del Canal de Panamá. El proyecto logró replantear el Canal no solo como infraestructura, sino como un símbolo vivo de la identidad nacional y de la responsabilidad compartida. Este caso reafirmó el poder de las prácticas de diseño inclusivo para fomentar la participación pública y generar un sentido de apropiación sobre narrativas patrimoniales de gran escala.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;05 —&lt;/span&gt;Del diseño a la realidad&lt;/h2&gt;
+&lt;figure class="c-img"&gt;&lt;img src="https://portafolio.parqueexplora.org/_next/image?url=https%3A%2F%2Fimgix.cosmicjs.com%2Fdf9138f0-87de-11ee-a141-bf415eaf0a74-img-test-2.webp%3Ffit%3Dcrop%26h%3D683%26w%3D1105%26upscale%3Dtrue%26auto%3Dformat%2Ccompress&amp;w=3840&amp;q=75" alt="Panama Canal Experience Center" loading="lazy" onerror="this.parentNode.remove()"&gt;&lt;/figure&gt;
+&lt;p&gt;&lt;em&gt;Usamos diversos formatos digitales, análogos y mixtos. Asimismo, nuestra metodología de investigación en campo nos permitió abordar el conocimiento de manera participativa. En este lugar, los visitantes reconocen esta gran obra de la humanidad.&lt;/em&gt;&lt;/p&gt;
+&lt;figure class="c-img"&gt;&lt;img src="https://portafolio.parqueexplora.org/_next/image?url=https%3A%2F%2Fimgix.cosmicjs.com%2F89adfbb0-87c2-11ee-a141-bf415eaf0a74-img-test-1.webp%3Ffit%3Dcrop%26h%3D683%26w%3D1105%26upscale%3Dtrue%26auto%3Dformat%2Ccompress&amp;w=3840&amp;q=75" alt="Panama Canal Experience Center" loading="lazy" onerror="this.parentNode.remove()"&gt;&lt;/figure&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
@@ -3750,7 +4285,20 @@
         </is>
       </c>
       <c r="T37" s="2" t="inlineStr"/>
-      <c r="U37" s="2" t="inlineStr"/>
+      <c r="U37" s="2" t="inlineStr">
+        <is>
+          <t>&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;01 —&lt;/span&gt;Contexto&lt;/h2&gt;
+&lt;p&gt;Como parte de mi maestría en Ingeniería en la Universidad EAFIT, lideré un proyecto de investigación enfocado en fortalecer las capacidades de diseño de experiencias interactivas en museos y centros de ciencia. A partir de mi experiencia profesional en Parque Explora, la iniciativa buscaba abordar la fragmentación teórica y práctica en el diseño de exhibiciones mediante el desarrollo de un marco integrado que pudiera guiar a los profesionales de museos en la creación de experiencias significativas para los visitantes.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;02 —&lt;/span&gt;El desafío&lt;/h2&gt;
+&lt;p&gt;El diseño de exhibiciones interactivas en los centros de ciencia suele verse obstaculizado por la falta de un lenguaje compartido, la dependencia de la intuición y la escasez de marcos de evaluación. Esto lleva a implementaciones costosas con un impacto limitado. El desafío era cerrar la brecha entre el conocimiento teórico y la aplicación práctica, ofreciendo a los equipos de museos una forma estructurada de conceptualizar, diseñar y evaluar experiencias con base en la participación de los usuarios y en los resultados de aprendizaje.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;03 —&lt;/span&gt;El proceso&lt;/h2&gt;
+&lt;ul&gt;&lt;li&gt;Desarrollé el marco DEX como una herramienta metodológica para diseñar y evaluar exposiciones interactivas.&lt;/li&gt;&lt;li&gt;Realicé investigación empírica con análisis temático y card sorting para identificar las cualidades experienciales críticas para la participación de los visitantes.&lt;/li&gt;&lt;li&gt;Facilité talleres de cocreación con equipos multidisciplinarios para aplicar la herramienta DEX en escenarios reales de diseño.&lt;/li&gt;&lt;li&gt;Me asocié con expertos nacionales e internacionales para validar y refinar la herramienta.&lt;/li&gt;&lt;li&gt;Implementé proyectos piloto en colaboración con aliados tecnológicos.&lt;/li&gt;&lt;li&gt;Impartí sesiones de formación y presentaciones en conferencias globales como ASTC y ECSITE.&lt;/li&gt;&lt;li&gt;Publiqué y difundí los hallazgos para contribuir a las comunidades más amplias de museos y diseño.&lt;/li&gt;&lt;/ul&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;04 —&lt;/span&gt;Impacto y logros&lt;/h2&gt;
+&lt;ul&gt;&lt;li&gt;Introduje un marco validado que apoya el proceso de toma de decisiones estratégicas y creativas en el diseño de exhibiciones.&lt;/li&gt;&lt;li&gt;Fortalecí la cultura interna de diseño en Parque Explora y en las instituciones aliadas.&lt;/li&gt;&lt;li&gt;Mejoré la experiencia del visitante al hacer las exposiciones más inmersivas, accesibles y emocionalmente resonantes.&lt;/li&gt;&lt;li&gt;Obtuve reconocimiento internacional a través de conferencias y publicaciones, lo que aumentó la visibilidad y la credibilidad.&lt;/li&gt;&lt;li&gt;Inspiré una nueva ola de desarrollo de exhibiciones basada en la experiencia de usuario y el diseño participativo.&lt;/li&gt;&lt;li&gt;Contribuí al desarrollo profesional del personal de museos mediante formación práctica y herramientas aplicables.&lt;/li&gt;&lt;li&gt;Posicioné a Parque Explora como líder en diseño centrado en la experiencia para la comunicación de la ciencia.&lt;/li&gt;&lt;/ul&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;05 —&lt;/span&gt;Publicaciones y presentaciones de DEX&lt;/h2&gt;
+&lt;ul&gt;&lt;li&gt;Ocampo-Agudelo J., Maya J. (2021) Core Concepts Linking Exhibit Design and the Visitor Experience in Science Centers: An Early Framework. En: Rauterberg M. (eds) Culture and Computing. Design Thinking and Cultural Computing. HCII 2021. Lecture Notes in Computer Science, vol 12795. Springer, Cham. &lt;a href="https://doi.org/10.1007/978-3-030-77431-8_7" target="_blank" rel="noopener"&gt;doi.org/10.1007/978-3-030-77431-8_7&lt;/a&gt;&lt;/li&gt;&lt;li&gt;&lt;a href="https://www.researchgate.net/publication/328223899_The_Design_of_Experience-centered_Exhibits_in_Science_Museums" target="_blank" rel="noopener"&gt;The Design of Experience-centered Exhibits in Science Centers&lt;/a&gt; (2018). Conferencia ASTC. Hartford, Estados Unidos.&lt;/li&gt;&lt;li&gt;Ocampo-Agudelo, Jose; Maya, Jorge; Roldán, Andrés (2017). &lt;a href="https://www.researchgate.net/publication/321135314_A_Tool_for_the_Design_of_Experience-Centered_Exhibits_in_Science_Centers" target="_blank" rel="noopener"&gt;“A Tool for the Design of Experience-Centered Exhibits in Science Centers”&lt;/a&gt;. Presentación de póster en Science Centre World Summit. Tokio, Japón.&lt;/li&gt;&lt;li&gt;Ocampo-Agudelo, J., &amp;amp; Maya, J. (2017). &lt;a href="https://www.researchgate.net/publication/319402257_Experiential_qualities_of_science_museum_exhibits_a_thematic_analysis" target="_blank" rel="noopener"&gt;Experiential qualities of science museum exhibits: a thematic analysis.&lt;/a&gt; En DS 87-8 Proceedings of the 21st International Conference on Engineering Design (ICED 17) Vol 8: Human Behaviour in Design, Vancouver, Canadá (pp. 439-448).&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
@@ -3840,7 +4388,20 @@
         </is>
       </c>
       <c r="T38" s="2" t="inlineStr"/>
-      <c r="U38" s="2" t="inlineStr"/>
+      <c r="U38" s="2" t="inlineStr">
+        <is>
+          <t>&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;01 —&lt;/span&gt;El contexto&lt;/h2&gt;
+&lt;p&gt;En 2017, como parte de una iniciativa estratégica liderada por la Secretaría Distrital de Cultura, Recreación y Deporte de Bogotá, al equipo de Parque Explora, en el que participé como estratega de experiencia, se le encargó diseñar una guía conceptual y estratégica para implementar "Espacios Creativos" en cinco bibliotecas públicas de la red BibloRed. Esta iniciativa buscaba reposicionar las bibliotecas como centros de innovación comunitaria, creatividad y apropiación social del conocimiento, desplazando su rol tradicional hacia espacios más dinámicos, inclusivos y participativos.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;02 —&lt;/span&gt;El desafío&lt;/h2&gt;
+&lt;p&gt;El principal desafío era redefinir el rol de las bibliotecas públicas en los contextos urbanos contemporáneos, haciendo de ellas no solo repositorios de información, sino motores de transformación social. Las bibliotecas carecían de marcos para integrar de manera sistemática la ciencia, el arte, la tecnología y el conocimiento comunitario de formas accesibles y atractivas. Era esencial diseñar un modelo que pudiera escalarse, adaptarse a las condiciones locales y ser acogido por comunidades de usuarios diversas.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;03 —&lt;/span&gt;El proceso&lt;/h2&gt;
+&lt;ul&gt;&lt;li&gt;Realizamos una extensa investigación documental y un benchmarking internacional sobre espacios creativos y maker.&lt;/li&gt;&lt;li&gt;Facilitamos talleres con comunidades locales, personal de las bibliotecas y stakeholders para comprender necesidades, barreras y aspiraciones.&lt;/li&gt;&lt;li&gt;Estructuramos el proyecto con el proceso de diseño Doble Diamante: Descubrir, Definir, Diseñar y Desarrollar.&lt;/li&gt;&lt;li&gt;Creamos una guía conceptual que incluía tipologías de espacios creativos, actividades clave y recomendaciones espaciales.&lt;/li&gt;&lt;li&gt;Propusimos principios de diseño flexibles que promueven la experimentación, la colaboración y la producción de conocimiento local.&lt;/li&gt;&lt;li&gt;Integramos los lineamientos educativos del marco ASCTI (Apropiación Social de la Ciencia, la Tecnología y la Innovación).&lt;/li&gt;&lt;li&gt;Desarrollamos estrategias de implementación a la medida de cinco bibliotecas piloto en Bogotá.&lt;/li&gt;&lt;/ul&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;04 —&lt;/span&gt;El impacto&lt;/h2&gt;
+&lt;ul&gt;&lt;li&gt;Desarrollamos el "Guion General de Espacios Creativos", hoy un documento de referencia para la innovación en bibliotecas en Colombia.&lt;/li&gt;&lt;li&gt;Ayudamos a posicionar las bibliotecas como centros activos de creatividad y desarrollo comunitario.&lt;/li&gt;&lt;li&gt;Hicimos posible la implementación de transformaciones físicas y programáticas en cinco grandes bibliotecas, creando entornos adaptables e inclusivos.&lt;/li&gt;&lt;li&gt;Fomentamos una nueva cultura de aprendizaje y participación mediante tecnologías creativas y conocimiento abierto.&lt;/li&gt;&lt;li&gt;Aportamos insumos para futuras políticas y estrategias en infraestructura cultural, con un fuerte enfoque centrado en el usuario y sistémico.&lt;/li&gt;&lt;li&gt;Recibimos comentarios positivos de instituciones culturales y educativas, que validaron la relevancia y la aplicabilidad del marco.&lt;/li&gt;&lt;li&gt;Inspiramos a otras instituciones de América Latina a explorar transformaciones similares en espacios públicos y culturales.&lt;/li&gt;&lt;/ul&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;05 —&lt;/span&gt;Resultados&lt;/h2&gt;
+&lt;p&gt;Tras el proceso de diseño estratégico, Biblored decidió implementar un piloto en una de las principales bibliotecas públicas de Bogotá.&lt;/p&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
@@ -3925,7 +4486,23 @@
       </c>
       <c r="S39" s="2" t="inlineStr"/>
       <c r="T39" s="2" t="inlineStr"/>
-      <c r="U39" s="2" t="inlineStr"/>
+      <c r="U39" s="2" t="inlineStr">
+        <is>
+          <t>&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;01 —&lt;/span&gt;Situación&lt;/h2&gt;
+&lt;p&gt;Los fenómenos climáticos de El Niño y La Niña suelen explicarse desde lentes científicos o técnicos, con foco en la complejidad meteorológica y el impacto global. Sin embargo, este proyecto buscó sacar a la luz las dimensiones socioculturales que a menudo se pasan por alto: cómo las comunidades viven, narran y dan sentido a estos cambios. En colaboración con Parque Explora (Colombia), la Cité de l’espace y el Museo de Toulouse (Francia), cocreamos una exposición que replantea estos fenómenos a través de las experiencias vividas de las personas. El objetivo era provocar reflexión, empatía y diálogo al llevar el arte y la ciencia a un espacio sensorial compartido.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;02 —&lt;/span&gt;Tarea&lt;/h2&gt;
+&lt;p&gt;Lideré la conceptualización y el diseño de la experiencia de la exposición, guiando la dirección curatorial junto con instituciones científicas y culturales de Colombia y Francia. Colaboré de cerca con expertos en contenidos, museógrafos y productores de exposiciones para dar forma a una narrativa convincente y participativa. Mi rol abarcó desde el encuadre inicial y el diseño narrativo hasta la supervisión creativa de la experiencia final del visitante en múltiples geografías. Este proyecto me permitió ampliar los límites de cómo pueden comunicarse los fenómenos climáticos a través de la narración sociocultural.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;03 —&lt;/span&gt;Acción&lt;/h2&gt;
+&lt;p&gt;&lt;strong&gt;Desarrollo del concepto.&lt;/strong&gt; Comenzamos definiendo una metáfora unificadora para la exposición: historias superpuestas. Inspirados en la dualidad de El Niño y La Niña, exploramos las tensiones entre las épocas seca y húmeda, la abundancia y la escasez, la memoria personal y la colectiva. Estas polaridades dieron forma a la estructura temática y espacial de la exposición. Desarrollamos una estrategia narrativa multisensorial que usó &lt;em&gt;filtros de color&lt;/em&gt; como dispositivo interpretativo, permitiendo a los visitantes cambiar de perspectiva de forma física y metafórica.&lt;/p&gt;
+&lt;p&gt;&lt;strong&gt;Codiseño y curaduría de contenidos.&lt;/strong&gt; En colaboración con científicos, educadores y representantes de la comunidad, reunimos historias y materiales que reflejaban los diversos impactos socioculturales de los fenómenos. Esto incluyó testimonios, artefactos locales, paisajes sonoros y medios visuales. Trabajar con aliados internacionales enriqueció el alcance de las narrativas y ayudó a validar los contenidos en distintos contextos.&lt;/p&gt;
+&lt;p&gt;&lt;strong&gt;Diseño y producción de la exposición.&lt;/strong&gt; Diseñamos tres espacios temáticos capaces de evocar una conexión emocional e intelectual. Cada espacio invitaba a los visitantes a recorrer líneas de tiempo, geografías y experiencias personales superpuestas. La exposición difuminó la frontera entre el arte y la ciencia mediante visuales inmersivos, componentes interactivos y atmósferas contrastantes. A pesar de los recursos limitados, prototipamos varios formatos de instalación para probar la respuesta de la audiencia antes de la producción a gran escala.&lt;/p&gt;
+&lt;p&gt;&lt;strong&gt;Lanzamiento internacional y adaptación.&lt;/strong&gt; Tras su primera temporada en Medellín, la exposición se adaptó y se instaló en Francia y México. Cada iteración mantuvo el concepto central, pero se contextualizó localmente para reflejar historias y referentes culturales relevantes. El carácter itinerante de la exposición permitió el intercambio intercultural y aumentó su alcance y resonancia.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;04 —&lt;/span&gt;Resultado&lt;/h2&gt;
+&lt;p&gt;La exposición logró cambiar la comprensión del público sobre El Niño y La Niña: de eventos climáticos abstractos a experiencias profundamente humanas y ricas en contexto. Despertó una participación significativa entre distintos grupos de edad y trasfondos culturales, aumentando la conciencia sobre la vulnerabilidad y la resiliencia ambientales.&lt;/p&gt;
+&lt;p&gt;Un aprendizaje clave fue el poder de la metáfora y del diseño multisensorial para crear un acceso emocional y cognitivo a fenómenos complejos. Aunque modesto en escala, el proyecto nos posicionó como líderes experimentales en la narración museográfica internacional y fortaleció los vínculos institucionales entre América Latina y Europa.&lt;/p&gt;
+&lt;p&gt;&lt;strong&gt;Aliados:&lt;/strong&gt; Cité de l'espace, Embajada de Francia en Colombia, Instituto Francés.&lt;/p&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
@@ -4008,7 +4585,21 @@
       </c>
       <c r="S40" s="2" t="inlineStr"/>
       <c r="T40" s="2" t="inlineStr"/>
-      <c r="U40" s="2" t="inlineStr"/>
+      <c r="U40" s="2" t="inlineStr">
+        <is>
+          <t>&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;01 —&lt;/span&gt;Contexto&lt;/h2&gt;
+&lt;p&gt;Parque Explora, un centro interactivo para la apropiación y divulgación de la ciencia y la tecnología, se creó en 2007 como símbolo de transformación social a través de la educación. Su misión es "Inspirar, comunicar y transformar mediante escenarios interactivos que contribuyan a la apropiación pública del conocimiento científico, tecnológico y social necesario para la construcción de una mejor sociedad". Una de las exhibiciones clave, la sala "Física Viva", abrió al público en diciembre de 2007 y ha sido exitosa en atraer públicos diversos, especialmente niños y jóvenes.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;02 —&lt;/span&gt;El desafío&lt;/h2&gt;
+&lt;p&gt;El principal desafío era desarrollar una nueva exhibición que pudiera reemplazar la exitosísima sala "Física Viva". El objetivo era crear un nuevo escenario que siguiera brindando experiencias memorables de aprendizaje (EMA) a los visitantes, incorporando las tendencias museográficas modernas y atendiendo las necesidades y expectativas de las audiencias contemporáneas. Esto exigía un cuidadoso equilibrio entre preservar el carácter educativo e interactivo de las exhibiciones y, a la vez, introducir elementos nuevos e innovadores.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;03 —&lt;/span&gt;Qué hicimos&lt;/h2&gt;
+&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Fase de diseño estratégico:&lt;/strong&gt; Empezamos con una fase abierta y exploratoria para reunir ideas y definir la dirección temática y estratégica de la nueva exhibición. Esto implicó analizar tendencias, intereses de las audiencias y posibles aliados.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Talleres participativos:&lt;/strong&gt; Realizamos talleres con diversos stakeholders, entre ellos miembros de la comunidad, educadores y expertos, para recoger aportes y asegurar que la nueva exhibición fuera relevante y atractiva.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Proceso de diseño iterativo:&lt;/strong&gt; Empleamos una metodología altamente iterativa, con etapas continuas de creación y evaluación. Esto aseguró que el diseño se mantuviera flexible y receptivo a los comentarios a lo largo de todo el proyecto.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Prototipado y pruebas:&lt;/strong&gt; Desarrollamos prototipos de los componentes de la nueva exhibición y los probamos con los públicos objetivo para refinar y optimizar la experiencia del visitante.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Colaboración interdisciplinaria:&lt;/strong&gt; Involucramos a un equipo multidisciplinario de distintas áreas de Parque Explora, asegurando que todos los aspectos del proyecto, desde el contenido educativo hasta la implementación técnica, estuvieran alineados.&lt;/li&gt;&lt;/ul&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;04 —&lt;/span&gt;Impacto esperado&lt;/h2&gt;
+&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Mayor participación de los visitantes:&lt;/strong&gt; Al incorporar elementos interactivos modernos y experiencias sensoriales diversas, la nueva exhibición busca cautivar y educar a los visitantes de manera más eficaz.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Entorno de aprendizaje sostenible:&lt;/strong&gt; Concebida como un espacio dinámico y en evolución, la nueva exhibición ofrecerá contenidos frescos y relevantes con el tiempo, incentivando las visitas repetidas y el interés sostenido.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Participación de la comunidad:&lt;/strong&gt; El enfoque participativo asegura que la exhibición resuene con la comunidad local, fomentando un sentido de apropiación y orgullo.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Mayor alcance educativo:&lt;/strong&gt; A través de elementos interdisciplinarios y transmedia, la exhibición conectará con una audiencia más amplia, que incluye colegios, familias y grupos de interés especial, promoviendo el aprendizaje a lo largo de la vida y la curiosidad.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Uso innovador del espacio:&lt;/strong&gt; La exhibición contará con espacios flexibles y multifuncionales que pueden adaptarse a distintas actividades y eventos, maximizando la utilidad y el impacto del entorno museal.&lt;/li&gt;&lt;/ul&gt;
+&lt;p&gt;&lt;a href="https://www.parqueexplora.org/sala-m-sica" target="_blank" rel="noopener"&gt;parqueexplora.org/sala-m-sica&lt;/a&gt;&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;05 —&lt;/span&gt;Premios&lt;/h2&gt;
+&lt;ul&gt;&lt;li&gt;"MÚSICA: Tú eres la orquesta" (MUSIC: You are the Orchestra) fue ganadora de bronce en la categoría Onsite Digital Experience de los Muse Awards 2019 de la American Alliance of Museums.&lt;/li&gt;&lt;li&gt;“Paisajes Musicales” (Musical Landscapes), una experiencia de la sala de música, fue ganadora de plata en la categoría Video, Film, Animation, and Live Media or Digital Performances de los Muse Awards 2019 de la American Alliance of Museums.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
@@ -4103,7 +4694,25 @@
         </is>
       </c>
       <c r="T41" s="2" t="inlineStr"/>
-      <c r="U41" s="2" t="inlineStr"/>
+      <c r="U41" s="2" t="inlineStr">
+        <is>
+          <t>&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;01 —&lt;/span&gt;Situación&lt;/h2&gt;
+&lt;p&gt;Desde 2003, Comfama, una empresa social colombiana, ha operado el histórico Claustro San Ignacio en Medellín principalmente como centro de servicios y espacio educativo. Al reconocer su subutilización y su inmenso potencial cultural, Comfama se asoció con Parque Explora para reimaginar el edificio como un centro cultural y creativo de referencia. Este proyecto buscaba honrar el patrimonio arquitectónico del sitio y, al mismo tiempo, transformarlo en un espacio que fomente el desarrollo humano, la ciudadanía y la expresión cultural inclusiva.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;02 —&lt;/span&gt;El desafío&lt;/h2&gt;
+&lt;p&gt;El uso del edificio era predominantemente transaccional, centrado en un modelo de atención al cliente que desincentivaba la participación del público. Elementos arquitectónicos clave como los patios, la capilla (auditorio) y la biblioteca eran inaccesibles o no estaban adecuadamente equipados para sostener experiencias culturales y educativas significativas. Las desconexiones espaciales y la accesibilidad limitada evidenciaron aún más la necesidad de una transformación radical, alineada con las dinámicas urbanas y culturales contemporáneas.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;03 —&lt;/span&gt;Tarea&lt;/h2&gt;
+&lt;p&gt;Fui parte del equipo central que apoyó a Comfama y a Parque Explora en la definición de la visión fundacional y la dirección estratégica de la transformación del Claustro. Mi rol abarcó la investigación de diseño, la síntesis, la facilitación creativa y el desarrollo conceptual, ayudando a cocrear el manifiesto, la estrategia espacial y el posicionamiento cultural del proyecto. Colaboré de cerca con líderes internos de Comfama, equipos de servicio, arquitectos y educadores para dar forma a una visión compartida, fundamentada en las necesidades de los usuarios y en el propósito institucional.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;04 —&lt;/span&gt;Acción&lt;/h2&gt;
+&lt;p&gt;&lt;strong&gt;Descubrimiento y alineación.&lt;/strong&gt; Realizamos visitas al sitio, entrevistas con stakeholders y talleres participativos con más de una docena de líderes de Comfama de las áreas de servicio, educación, infraestructura y estrategia. Este trabajo de base sacó a la luz tensiones críticas: el desajuste entre el potencial del edificio y su uso actual, y la necesidad de un espacio cívico más acogedor, inspirador e inclusivo.&lt;/p&gt;
+&lt;p&gt;&lt;strong&gt;Encuadre estratégico y definición de intenciones.&lt;/strong&gt; Aplicando la metodología VEA (Visión de la Experiencia de Aprendizaje) de Parque Explora, cocreamos un &lt;em&gt;Manifiesto de Intención&lt;/em&gt; que articula una visión compartida: convertir el Claustro en un centro creativo para el desarrollo del talento y la activación cultural. Definimos principios fundacionales —participación, pensamiento crítico, inspiración y expresión— y mapeamos sus implicaciones para el contenido, la experiencia y el espacio.&lt;/p&gt;
+&lt;p&gt;&lt;strong&gt;Diseño conceptual y estrategia espacial.&lt;/strong&gt; Propusimos un nuevo esquema arquitectónico y programático que transformó el Claustro de un edificio cerrado y con una fuerte carga de servicios en un entorno público por capas. El plan introdujo laboratorios de aprendizaje flexibles, zonas de exhibición, escenarios culturales y una terraza pública en la azotea. Las tipologías de espacios incluyeron un laboratorio transmedia, un estudio de gastronomía, talleres de ideación y un renovado centro Comfama Interactivo.&lt;/p&gt;
+&lt;p&gt;&lt;strong&gt;Hoja de ruta y factibilidad.&lt;/strong&gt; Finalmente, detallamos un plan de transformación por fases que incluía programas arquitectónicos, etapas de intervención, proyecciones presupuestales y una estrategia operativa para permitir un aprendizaje y una adaptación continuos durante la ejecución.&lt;/p&gt;
+&lt;h3 class="c-h3"&gt;Aspectos destacados del proceso&lt;/h3&gt;
+&lt;ul&gt;&lt;li&gt;Realizamos visitas al sitio, entrevistas con stakeholders y talleres de cocreación para recoger insights y aspiraciones.&lt;/li&gt;&lt;li&gt;Aplicamos la metodología VEA (Visión de la Experiencia de Aprendizaje) para un diseño sistémico y centrado en el usuario.&lt;/li&gt;&lt;li&gt;Definimos una visión estratégica y un programa arquitectónico alineados con la misión de Comfama y las necesidades de la comunidad.&lt;/li&gt;&lt;li&gt;Propusimos una distribución multifuncional que incluye plazas públicas, laboratorios creativos, áreas de coworking y espacios de aprendizaje reimaginados.&lt;/li&gt;&lt;li&gt;Diseñamos ambientes flexibles como el Laboratorio Transmedia, el Laboratorio de Gastronomía y el Auditorio Público para sostener una programación cultural diversa.&lt;/li&gt;&lt;li&gt;Creamos mejoras de accesibilidad e integramos sistemas de circulación vertical para unificar la experiencia del edificio.&lt;/li&gt;&lt;li&gt;Desarrollamos un plan de ejecución por fases que permitiera la operación continua durante la renovación.&lt;/li&gt;&lt;/ul&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;05 —&lt;/span&gt;Resultado&lt;/h2&gt;
+&lt;p&gt;Este trabajo estableció la base estratégica y experiencial de una de las transformaciones cívicas más ambiciosas de Medellín. Desde entonces, el Claustro se ha convertido en un punto de referencia de la vida cultural de la ciudad, con más de 2,1 millones de visitantes y más de 6.000 eventos públicos realizados entre 2023 y 2025. El proyecto demostró cómo los espacios patrimoniales pueden reactivarse mediante un diseño orientado por el propósito, y dio forma a mi enfoque actual de alinear la transformación física con la visión institucional y el sentido para los usuarios.&lt;/p&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
@@ -4199,7 +4808,22 @@
         </is>
       </c>
       <c r="T42" s="2" t="inlineStr"/>
-      <c r="U42" s="2" t="inlineStr"/>
+      <c r="U42" s="2" t="inlineStr">
+        <is>
+          <t>&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;01 —&lt;/span&gt;Situación&lt;/h2&gt;
+&lt;p&gt;La exposición temporal &lt;em&gt;Molas: capas de sabiduría&lt;/em&gt; en el Museo del Oro de Bogotá buscaba revelar las cosmovisiones y los saberes ancestrales del pueblo Guna de Colombia y Panamá. Central en esta expresión cultural son las &lt;em&gt;molas&lt;/em&gt;: textiles de múltiples capas que visten las mujeres guna, cargados de significado simbólico y protector. El desafío curatorial era transformar estas intrincadas telas en una experiencia sensorial inmersiva capaz de comunicar el viaje espiritual de los &lt;em&gt;Neles&lt;/em&gt; (líderes y visionarios guna), honrando sus cosmogonías en capas y su conexión con las fuerzas creadoras del mundo.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;02 —&lt;/span&gt;Tarea&lt;/h2&gt;
+&lt;p&gt;Fui responsable de liderar la conceptualización y el diseño audiovisual de la pieza inmersiva &lt;em&gt;Los Galus&lt;/em&gt;. Mi tarea era traducir la cosmología guna en una narrativa espacial que evocara los viajes oníricos de los Neles a través de las dimensiones en capas de las molas. El objetivo no era representar literalmente sus historias, sino crear un espacio respetuoso y afectivo de contemplación y asombro.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;03 —&lt;/span&gt;Acción&lt;/h2&gt;
+&lt;p&gt;Diseñamos &lt;em&gt;Los Galus&lt;/em&gt; como una sala inmersiva en la que los visitantes entraban a un espacio liminal de visuales, texturas y sonidos superpuestos, que reflejaba la lógica textil en capas de las molas. Inspirada en la idea de cruzar umbrales entre reinos espirituales, la instalación usó video mapping, paisajes sonoros ambientales y superficies espejadas para generar una sensación de espacio infinito y profundidad simbólica.&lt;/p&gt;
+&lt;p&gt;Nuestro equipo colaboró con antropólogos, curadores y asesores guna para asegurar la precisión y la sensibilidad cultural. La estructura narrativa evitó el relato lineal y privilegió un ritmo abierto y sensorial que hacía eco de las secuencias oníricas descritas por los Neles. El lenguaje visual se basó en formas abstractas tomadas de la iconografía tradicional de las molas, que se desplegaban en ciclos para simular el ritual y la ensoñación. Lo complementamos con &lt;em&gt;La Mujer y la Mola&lt;/em&gt;, una segunda experiencia audiovisual centrada en la sabiduría de las mujeres guna y en el acto de creación.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;04 —&lt;/span&gt;Resultado&lt;/h2&gt;
+&lt;p&gt;La exposición ofreció a los visitantes del museo una experiencia profunda y contemplativa, que iba más allá de la explicación hacia la inmersión. &lt;em&gt;Los Galus&lt;/em&gt; se convirtió en uno de los puntos más destacados de la muestra, elogiada por su interpretación poética de la cosmología guna. El proyecto reafirmó cómo los medios inmersivos pueden honrar las narrativas indígenas al abrazar la ambigüedad, el simbolismo y la resonancia emocional por encima de los formatos didácticos.&lt;/p&gt;
+&lt;figure class="c-video"&gt;&lt;iframe src="https://www.youtube-nocookie.com/embed/WQmOwhhE5Vk" title="Video" loading="lazy" allow="accelerometer; encrypted-media; picture-in-picture" allowfullscreen&gt;&lt;/iframe&gt;&lt;/figure&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;05 —&lt;/span&gt;La mujer y la mola&lt;/h2&gt;
+&lt;figure class="c-video"&gt;&lt;iframe src="https://www.youtube-nocookie.com/embed/sT1iB5tOBgY" title="Video" loading="lazy" allow="accelerometer; encrypted-media; picture-in-picture" allowfullscreen&gt;&lt;/iframe&gt;&lt;/figure&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
@@ -4286,7 +4910,21 @@
       </c>
       <c r="S43" s="2" t="inlineStr"/>
       <c r="T43" s="2" t="inlineStr"/>
-      <c r="U43" s="2" t="inlineStr"/>
+      <c r="U43" s="2" t="inlineStr">
+        <is>
+          <t>&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;01 —&lt;/span&gt;Situación&lt;/h2&gt;
+&lt;p&gt;A medida que Colombia profundizaba su estrategia nacional de ciencia, tecnología e innovación inclusivas, crecía la necesidad de orientar la creación y el fortalecimiento de Centros de Ciencia en todo el país. Respaldada por Colciencias y desarrollada en alianza con Parque Explora, esta guía nacional buscaba alinear los centros nuevos y existentes con los referentes globales de instituciones de cuarta y quinta generación: espacios enfocados en el aprendizaje experiencial, la participación pública y la participación ciudadana en la ciencia y la tecnología. El desafío era traducir estas ambiciones en orientaciones prácticas y escalables.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;02 —&lt;/span&gt;Tarea&lt;/h2&gt;
+&lt;p&gt;Formé parte de la autoría de la guía y lideré el componente de &lt;strong&gt;diseño interior y ambientes de aprendizaje&lt;/strong&gt;. Mi responsabilidad era definir los principios espaciales y experienciales que ayudarían a los Centros de Ciencia a ir más allá de la exhibición para convertirse en ecosistemas participativos y educativos. Colaboré de cerca con museólogos, expertos en diseño arquitectónico y técnico, y especialistas en participación pública para integrar la intención pedagógica en la lógica espacial de estos centros.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;03 —&lt;/span&gt;Acción&lt;/h2&gt;
+&lt;p&gt;&lt;strong&gt;Diseño conceptual de los lineamientos espaciales.&lt;/strong&gt; Comenzamos analizando modelos globales (ASTC, ECSITE, RedPOP) y tendencias emergentes como la &lt;em&gt;apropiación pública de la ciencia y la tecnología&lt;/em&gt; (public engagement). Estos insumos dieron lugar a un conjunto de principios de diseño espacial basados en la flexibilidad, la interacción multisensorial, la accesibilidad y el diseño inclusivo, que traducen los valores educativos en entornos físicos.&lt;/p&gt;
+&lt;p&gt;&lt;strong&gt;Desarrollo de la guía y validación en campo.&lt;/strong&gt; Trabajando en conjunto con los equipos de Diseño y de curaduría de Parque Explora, estructuramos la guía en rutas temáticas. Mi aporte se centró en las secciones de &lt;strong&gt;Diseño Interior&lt;/strong&gt; y &lt;strong&gt;Ambientes de Aprendizaje&lt;/strong&gt;, alineando las distribuciones físicas con prácticas de aprendizaje informales y participativas. Los principios de diseño se plantearon como herramientas para dar forma no solo al espacio, sino también al comportamiento y a la participación dentro de él.&lt;/p&gt;
+&lt;p&gt;&lt;strong&gt;Aplicación piloto: Proyecto Malva.&lt;/strong&gt; Los lineamientos se probaron en el &lt;strong&gt;fortalecimiento de dos Centros de Ciencia del Valle del Cauca&lt;/strong&gt;, como parte del proyecto Malva. Esto sirvió como un piloto real para evaluar cómo el diseño espacial influía en la experiencia de aprendizaje y en la apropiación de los centros por parte de la comunidad.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;04 —&lt;/span&gt;Resultado&lt;/h2&gt;
+&lt;p&gt;La guía estableció un marco nacional compartido para diseñar Centros de Ciencia de nueva generación en Colombia. Su adopción ha ayudado a elevar la calidad y la coherencia de los proyectos en todo el país, tendiendo un puente entre el diseño físico y la misión educativa. Un aprendizaje clave fue el valor de integrar el pensamiento espacial y pedagógico desde el inicio del proceso para asegurar que los espacios no solo funcionen, sino que transformen la forma en que las personas se relacionan con la ciencia y entre sí.&lt;/p&gt;
+&lt;p&gt;&lt;strong&gt;Escalabilidad y adopción nacional.&lt;/strong&gt; Desde su publicación, la guía se ha convertido en una referencia nacional. Fue determinante para dar forma a la visión y a las estrategias espaciales del &lt;strong&gt;Centro de Ciencia CIBI en Dosquebradas&lt;/strong&gt; y se usó como herramienta de diagnóstico y planeación en el &lt;strong&gt;Centro de Ciencia de la Universidad Tecnológica de Pereira&lt;/strong&gt;. Muchas otras iniciativas en el país siguen basándose en su marco.&lt;/p&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
@@ -4370,7 +5008,14 @@
         </is>
       </c>
       <c r="T44" s="2" t="inlineStr"/>
-      <c r="U44" s="2" t="inlineStr"/>
+      <c r="U44" s="2" t="inlineStr">
+        <is>
+          <t>&lt;figure class="c-video"&gt;&lt;iframe src="https://www.youtube-nocookie.com/embed/lDZhGe6-89M" title="Video" loading="lazy" allow="accelerometer; encrypted-media; picture-in-picture" allowfullscreen&gt;&lt;/iframe&gt;&lt;/figure&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;01 —&lt;/span&gt;El concepto&lt;/h2&gt;
+&lt;p&gt;MOVA es el centro de innovación para docentes de Medellín. Conceptualizamos este novedoso ambiente como la intersección de tres dimensiones: ser, saber y crear; lo que permite desarrollar y nutrir habilidades personales y profesionales orientadas a la generación de experiencias educativas, con prácticas pedagógicas diversas y contextualizadas, basadas en el diálogo y el intercambio de ideas y experiencias.&lt;/p&gt;
+&lt;p&gt;Aprender haciendo y enseñar mostrando es un compromiso metodológico común que se define en las relaciones espaciales y en las formas de habitar el proyecto. Criterios como la simultaneidad espacial, los vacíos y las transparencias, y la mezcla de actividades permiten generar relaciones más complejas al dar visibilidad a todas las experiencias que ocurren, encontrando un entorno fértil para la creación.&lt;/p&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
@@ -4439,7 +5084,11 @@
       </c>
       <c r="S45" s="2" t="inlineStr"/>
       <c r="T45" s="2" t="inlineStr"/>
-      <c r="U45" s="2" t="inlineStr"/>
+      <c r="U45" s="2" t="inlineStr">
+        <is>
+          <t>&lt;figure class="c-video"&gt;&lt;iframe src="https://www.youtube-nocookie.com/embed/9GzNzIdNakc" title="Video" loading="lazy" allow="accelerometer; encrypted-media; picture-in-picture" allowfullscreen&gt;&lt;/iframe&gt;&lt;/figure&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
@@ -4517,7 +5166,12 @@
         </is>
       </c>
       <c r="T46" s="2" t="inlineStr"/>
-      <c r="U46" s="2" t="inlineStr"/>
+      <c r="U46" s="2" t="inlineStr">
+        <is>
+          <t>&lt;blockquote class="c-quote"&gt;“Una exhibición sobre métodos antiguos y modernos de autoexpresión: una idea bastante abstracta y audaz. Varias piezas interactivas que usan una variedad de tecnologías para lograr que los visitantes se expresen de forma individual y colectiva. Fuerte sentido de interactividad, muy divertida y atractiva, con mucha personalización. Altamente atractiva, con insights experienciales sobre el proceso creativo.” — Muse Awards 2017, mención honorífica&lt;/blockquote&gt;
+&lt;figure class="c-video"&gt;&lt;iframe src="https://www.youtube-nocookie.com/embed/DPe9s-1SppQ" title="Video" loading="lazy" allow="accelerometer; encrypted-media; picture-in-picture" allowfullscreen&gt;&lt;/iframe&gt;&lt;/figure&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
@@ -4602,7 +5256,15 @@
         </is>
       </c>
       <c r="T47" s="2" t="inlineStr"/>
-      <c r="U47" s="2" t="inlineStr"/>
+      <c r="U47" s="2" t="inlineStr">
+        <is>
+          <t>&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;01 —&lt;/span&gt;Historias menores&lt;/h2&gt;
+&lt;p&gt;Historias menores (Minor stories) es una exhibición interactiva equipada con una interfaz tangible que usa una técnica de video mapping sobre una mesa en relieve.&lt;/p&gt;
+&lt;p&gt;Se crea una comunidad aborigen en una isla, con plantas, animales, aldeanos y un chamán que le reza al cielo cuando enfrenta un verano intenso o un invierno crudo. Los visitantes comparten el control total de la situación, moviendo y rotando fichas sobre la superficie proyectada. Al manipular dichos objetos, los visitantes pueden crear distintas situaciones: pueden convertir el día en noche, el verano en invierno, generar efectos de aves y ovnis, e incluso provocar desastres naturales en regiones específicas.&lt;/p&gt;
+&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Participación sensorial:&lt;/strong&gt; La proyección de video sobre una superficie en relieve sorprende al visitante, que además encuentra algunos objetos que le permiten interactuar con el juego de una manera nueva y tangible.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Participación creativa:&lt;/strong&gt; Cada visitante está invitado a experimentar y crear su propia historia corta.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Participación social:&lt;/strong&gt; Tres personas pueden compartir la experiencia al mismo tiempo y observar los resultados.&lt;/li&gt;&lt;/ul&gt;
+&lt;figure class="c-video"&gt;&lt;iframe src="https://www.youtube-nocookie.com/embed/ZcotQQtb2Gg" title="Video" loading="lazy" allow="accelerometer; encrypted-media; picture-in-picture" allowfullscreen&gt;&lt;/iframe&gt;&lt;/figure&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
@@ -4698,7 +5360,22 @@
         </is>
       </c>
       <c r="T48" s="2" t="inlineStr"/>
-      <c r="U48" s="2" t="inlineStr"/>
+      <c r="U48" s="2" t="inlineStr">
+        <is>
+          <t>&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;01 —&lt;/span&gt;Situación&lt;/h2&gt;
+&lt;p&gt;Parque Explora buscaba renovar una de sus salas más emblemáticas: la &lt;em&gt;Sala Mente&lt;/em&gt; (The Mind Gallery). Desarrollada originalmente en 2011 en colaboración con el Grupo de Neurociencias de la Universidad de Antioquia, la sala necesitaba evolucionar hacia una experiencia más atractiva, inclusiva y contemporánea. El objetivo era traducir la investigación de vanguardia sobre el cerebro en un entorno de aprendizaje interactivo y emocional, que estimulara la curiosidad, la imaginación y la autorreflexión en todos los públicos.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;02 —&lt;/span&gt;Tarea&lt;/h2&gt;
+&lt;p&gt;Fui responsable del diseño interactivo de la sala. Mi rol cubrió el desarrollo integral de las experiencias del visitante: desde el concepto y la lógica de interacción hasta el detallado técnico, el prototipado y la coordinación de la producción y la instalación. Trabajé de cerca con científicos, fabricantes de exhibiciones y el equipo interno de Explora para asegurar que cada componente fuera a la vez científicamente preciso y emocionalmente resonante.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;03 —&lt;/span&gt;Acción&lt;/h2&gt;
+&lt;p&gt;&lt;strong&gt;Investigación colaborativa y encuadre del concepto.&lt;/strong&gt; La base del proyecto fue una alianza estrecha con neurocientíficos de la Universidad de Antioquia. Realizamos sesiones de trabajo regulares para traducir investigación compleja en narrativas claras y cercanas. Esta colaboración aseguró que cada exhibición hablara de experiencias cotidianas sin dejar de estar fundamentada en el rigor científico.&lt;/p&gt;
+&lt;p&gt;&lt;strong&gt;Diseño de la interacción y la experiencia.&lt;/strong&gt; Reimaginamos la sala no como una exhibición estática, sino como un "medio en movimiento" para el diálogo. En lugar de organizar los contenidos por anatomía cerebral, estructuramos el espacio en torno a las &lt;em&gt;habilidades humanas&lt;/em&gt; —como soñar, sentir, imaginar y comunicar—, haciendo el tema más accesible y emocionalmente resonante.&lt;/p&gt;
+&lt;p&gt;&lt;strong&gt;Arquitectura de la exposición y zonas temáticas.&lt;/strong&gt; El espacio se dividió con un sistema codificado por colores, en el que cada zona invitaba a explorar distintas funciones cognitivas. Cada interacción se diseñó para ser intuitiva y abierta, animando a los visitantes a poner a prueba su memoria, su percepción o su creatividad a su propio ritmo. La sala se construyó en torno a un modelo de aprendizaje de libre elección, que permite una exploración no lineal y una experimentación lúdica.&lt;/p&gt;
+&lt;p&gt;&lt;strong&gt;Prototipado, detallado e instalación.&lt;/strong&gt; Lideré el detallado técnico y la coordinación de la producción de las estaciones interactivas, asegurando que cada pieza pudiera resistir un uso público intenso sin perder fidelidad a la experiencia prevista. Esto incluyó exhibiciones mecánicas, interfaces digitales, disparadores físicos e interacciones basadas en sensores. También supervisé el ensamblaje final y la instalación en sitio.&lt;/p&gt;
+&lt;h2 class="c-h2"&gt;&lt;span class="idx"&gt;04 —&lt;/span&gt;Resultado&lt;/h2&gt;
+&lt;p&gt;La Sala Mente se convirtió en uno de los espacios más queridos de Parque Explora, elogiada por su capacidad de despertar asombro y autoindagación. La sala logró tender un puente entre la neurociencia y la vida cotidiana, convirtiendo conceptos abstractos en experiencias tangibles, alegres y, a veces, surrealistas. Un aprendizaje clave: diseñar para la mente exige involucrar tanto al intelecto como al cuerpo, ofreciendo no solo información, sino oportunidades de sentir, imaginar y cuestionar.&lt;/p&gt;
+&lt;figure class="c-video"&gt;&lt;iframe src="https://www.youtube-nocookie.com/embed/a5zf8eEe4wU" title="Video" loading="lazy" allow="accelerometer; encrypted-media; picture-in-picture" allowfullscreen&gt;&lt;/iframe&gt;&lt;/figure&gt;</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Home: What is HIPERNOVA? particle section + latest Substack articles
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/database/hipernova-portafolio-db.xlsx
+++ b/database/hipernova-portafolio-db.xlsx
@@ -6210,7 +6210,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B142"/>
+  <dimension ref="A1:B172"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -7408,514 +7408,874 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>CPG</t>
+          <t>Highlights</t>
         </is>
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>Bienes de consumo</t>
+          <t>Destacados</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
         <is>
-          <t>Culture &amp; Museums</t>
+          <t>Practice</t>
         </is>
       </c>
       <c r="B101" s="2" t="inlineStr">
         <is>
-          <t>Cultura y museos</t>
+          <t>Práctica</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Principles</t>
         </is>
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Principios</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Clients &amp; partners</t>
         </is>
       </c>
       <c r="B103" s="2" t="inlineStr">
         <is>
-          <t>Energía</t>
+          <t>Clientes y aliados</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>Financial Services</t>
+          <t>Next</t>
         </is>
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>Servicios financieros</t>
+          <t>Siguiente</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
         <is>
-          <t>Goverment / Public</t>
+          <t>02 — What is HIPERNOVA?</t>
         </is>
       </c>
       <c r="B105" s="2" t="inlineStr">
         <is>
-          <t>Gobierno / Público</t>
+          <t>02 — ¿Qué es HIPERNOVA?</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
         <is>
-          <t>Retail</t>
+          <t>Latest writing</t>
         </is>
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
-          <t>Retail</t>
+          <t>Últimos escritos</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
         <is>
-          <t>Science - Research</t>
+          <t>From the Substack.</t>
         </is>
       </c>
       <c r="B107" s="2" t="inlineStr">
         <is>
-          <t>Ciencia - Investigación</t>
+          <t>Desde el Substack.</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
         <is>
-          <t>Third Sector / NGOs</t>
+          <t>All writing</t>
         </is>
       </c>
       <c r="B108" s="2" t="inlineStr">
         <is>
-          <t>Tercer sector / ONG</t>
+          <t>Todos los escritos</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
         <is>
-          <t>CX Strategy</t>
+          <t>A hypernova is a concentration of energy capable of altering what surrounds it. I'm not interested in the astronomical phenomenon, but in its behavior.</t>
         </is>
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>Estrategia de CX</t>
+          <t>Una hipernova es una concentración de energía capaz de alterar lo que la rodea. No me interesa el fenómeno astronómico, sino su comportamiento.</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
         <is>
-          <t>Creative space</t>
+          <t>Scroll to move through the behavior of a hypernova.</t>
         </is>
       </c>
       <c r="B110" s="2" t="inlineStr">
         <is>
-          <t>Espacio creativo</t>
+          <t>Desliza para recorrer el comportamiento de una hipernova.</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
         <is>
-          <t>Customer Experience and Innovation</t>
+          <t>Accumulation.</t>
         </is>
       </c>
       <c r="B111" s="2" t="inlineStr">
         <is>
-          <t>Experiencia de cliente e innovación</t>
+          <t>Acumulación.</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
         <is>
-          <t>Data visualization</t>
+          <t>Tension.</t>
         </is>
       </c>
       <c r="B112" s="2" t="inlineStr">
         <is>
-          <t>Visualización de datos</t>
+          <t>Tensión.</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
         <is>
-          <t>Digital experience</t>
+          <t>Release.</t>
         </is>
       </c>
       <c r="B113" s="2" t="inlineStr">
         <is>
-          <t>Experiencia digital</t>
+          <t>Liberación.</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
         <is>
-          <t>Digital product</t>
+          <t>Expansion.</t>
         </is>
       </c>
       <c r="B114" s="2" t="inlineStr">
         <is>
-          <t>Producto digital</t>
+          <t>Expansión.</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
         <is>
-          <t>Exhibition</t>
+          <t>Transformation.</t>
         </is>
       </c>
       <c r="B115" s="2" t="inlineStr">
         <is>
-          <t>Exposición</t>
+          <t>Transformación.</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
         <is>
-          <t>Immersive media</t>
+          <t>Emergence.</t>
         </is>
       </c>
       <c r="B116" s="2" t="inlineStr">
         <is>
-          <t>Medios inmersivos</t>
+          <t>Emergencia.</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
         <is>
-          <t>Interactives</t>
+          <t>Accumulation</t>
         </is>
       </c>
       <c r="B117" s="2" t="inlineStr">
         <is>
-          <t>Interactivos</t>
+          <t>Acumulación</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
         <is>
-          <t>Learning environment</t>
+          <t>Tension</t>
         </is>
       </c>
       <c r="B118" s="2" t="inlineStr">
         <is>
-          <t>Entorno de aprendizaje</t>
+          <t>Tensión</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
         <is>
-          <t>Master Planning</t>
+          <t>Release</t>
         </is>
       </c>
       <c r="B119" s="2" t="inlineStr">
         <is>
-          <t>Plan maestro</t>
+          <t>Liberación</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
         <is>
-          <t>Policy making</t>
+          <t>Expansion</t>
         </is>
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
-          <t>Política pública</t>
+          <t>Expansión</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
         <is>
-          <t>Product Design and Strategy</t>
+          <t>Emergence</t>
         </is>
       </c>
       <c r="B121" s="2" t="inlineStr">
         <is>
-          <t>Diseño y estrategia de producto</t>
+          <t>Emergencia</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
         <is>
-          <t>Purpose-driven strategy</t>
+          <t>Energy concentrates before something changes. Questions, signals and discomforts build up, often without a name.</t>
         </is>
       </c>
       <c r="B122" s="2" t="inlineStr">
         <is>
-          <t>Estrategia con propósito</t>
+          <t>La energía se concentra antes de que algo cambie. Preguntas, señales e incomodidades se acumulan, muchas veces sin nombre.</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
         <is>
-          <t>Science center</t>
+          <t>What exists no longer suffices to contain what is starting to appear. Tension isn't a problem to eliminate: it's information.</t>
         </is>
       </c>
       <c r="B123" s="2" t="inlineStr">
         <is>
-          <t>Centro de ciencia</t>
+          <t>Lo que existe ya no alcanza para contener lo que empieza a aparecer. La tensión no es un problema que eliminar: es información.</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
         <is>
-          <t>Strategy</t>
+          <t>Something lets go: an assumption, a way of seeing, a way of deciding. The contained energy finds a way out.</t>
         </is>
       </c>
       <c r="B124" s="2" t="inlineStr">
         <is>
-          <t>Estrategia</t>
+          <t>Algo se suelta: un supuesto, una manera de mirar, una forma de decidir. La energía contenida encuentra salida.</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
         <is>
-          <t>Sustainable Futures</t>
+          <t>What is released alters its surroundings. Perspectives, relationships and futures appear that weren't available before.</t>
         </is>
       </c>
       <c r="B125" s="2" t="inlineStr">
         <is>
-          <t>Futuros sostenibles</t>
+          <t>Lo liberado altera su entorno. Aparecen perspectivas, relaciones y futuros que antes no estaban disponibles.</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
         <is>
-          <t>Temporary exhibition</t>
+          <t>Conditions change, and so do the people who inhabit them. It isn't an improvement on what came before: it's another configuration.</t>
         </is>
       </c>
       <c r="B126" s="2" t="inlineStr">
         <is>
-          <t>Exposición temporal</t>
+          <t>Cambian las condiciones y cambian quienes las habitan. No es una mejora de lo anterior: es otra configuración.</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
         <is>
-          <t>Transformation</t>
+          <t>Something emerges that couldn't have been planned in advance. A new order born from everything that moved.</t>
         </is>
       </c>
       <c r="B127" s="2" t="inlineStr">
         <is>
-          <t>Transformación</t>
+          <t>Surge algo que no podía planificarse de antemano. Un orden nuevo que nace de todo lo que se movió.</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
         <is>
-          <t>Traveling exhibition</t>
+          <t>My intention isn't to produce change.</t>
         </is>
       </c>
       <c r="B128" s="2" t="inlineStr">
         <is>
-          <t>Exposición itinerante</t>
+          <t>Mi intención no es producir cambio.</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
         <is>
-          <t>Ux</t>
+          <t>It's to alter trajectories.</t>
         </is>
       </c>
       <c r="B129" s="2" t="inlineStr">
         <is>
-          <t>UX</t>
+          <t>Es alterar trayectorias.</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
         <is>
-          <t>Workshop / Bootcamp</t>
+          <t>CPG</t>
         </is>
       </c>
       <c r="B130" s="2" t="inlineStr">
         <is>
-          <t>Taller / Bootcamp</t>
+          <t>Bienes de consumo</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
         <is>
-          <t>Author</t>
+          <t>Culture &amp; Museums</t>
         </is>
       </c>
       <c r="B131" s="2" t="inlineStr">
         <is>
-          <t>Autor</t>
+          <t>Cultura y museos</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
         <is>
-          <t>Creative director</t>
+          <t>Education</t>
         </is>
       </c>
       <c r="B132" s="2" t="inlineStr">
         <is>
-          <t>Director creativo</t>
+          <t>Educación</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
         <is>
-          <t>Exhibition Designer</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="B133" s="2" t="inlineStr">
         <is>
-          <t>Diseñador de exposiciones</t>
+          <t>Energía</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
         <is>
-          <t>Interior designer</t>
+          <t>Financial Services</t>
         </is>
       </c>
       <c r="B134" s="2" t="inlineStr">
         <is>
-          <t>Diseñador de interiores</t>
+          <t>Servicios financieros</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
         <is>
-          <t>Project leader</t>
+          <t>Goverment / Public</t>
         </is>
       </c>
       <c r="B135" s="2" t="inlineStr">
         <is>
-          <t>Líder de proyecto</t>
+          <t>Gobierno / Público</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
         <is>
-          <t>Researcher</t>
+          <t>Retail</t>
         </is>
       </c>
       <c r="B136" s="2" t="inlineStr">
         <is>
-          <t>Investigador</t>
+          <t>Retail</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
         <is>
-          <t>Senior Exhibition Designer</t>
+          <t>Science - Research</t>
         </is>
       </c>
       <c r="B137" s="2" t="inlineStr">
         <is>
-          <t>Diseñador sénior de exposiciones</t>
+          <t>Ciencia - Investigación</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
         <is>
-          <t>Senior designer</t>
+          <t>Third Sector / NGOs</t>
         </is>
       </c>
       <c r="B138" s="2" t="inlineStr">
         <is>
-          <t>Diseñador sénior</t>
+          <t>Tercer sector / ONG</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
         <is>
-          <t>Strategic Design &amp; CX Lead</t>
+          <t>CX Strategy</t>
         </is>
       </c>
       <c r="B139" s="2" t="inlineStr">
         <is>
-          <t>Líder de diseño estratégico y CX</t>
+          <t>Estrategia de CX</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
         <is>
-          <t>Strategic Design Consultant</t>
+          <t>Creative space</t>
         </is>
       </c>
       <c r="B140" s="2" t="inlineStr">
         <is>
-          <t>Consultor de diseño estratégico</t>
+          <t>Espacio creativo</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
         <is>
-          <t>Strategy Consulting Director</t>
+          <t>Customer Experience and Innovation</t>
         </is>
       </c>
       <c r="B141" s="2" t="inlineStr">
         <is>
-          <t>Director de consultoría estratégica</t>
+          <t>Experiencia de cliente e innovación</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
         <is>
+          <t>Data visualization</t>
+        </is>
+      </c>
+      <c r="B142" s="2" t="inlineStr">
+        <is>
+          <t>Visualización de datos</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="2" t="inlineStr">
+        <is>
+          <t>Digital experience</t>
+        </is>
+      </c>
+      <c r="B143" s="2" t="inlineStr">
+        <is>
+          <t>Experiencia digital</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="2" t="inlineStr">
+        <is>
+          <t>Digital product</t>
+        </is>
+      </c>
+      <c r="B144" s="2" t="inlineStr">
+        <is>
+          <t>Producto digital</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="2" t="inlineStr">
+        <is>
+          <t>Exhibition</t>
+        </is>
+      </c>
+      <c r="B145" s="2" t="inlineStr">
+        <is>
+          <t>Exposición</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="2" t="inlineStr">
+        <is>
+          <t>Immersive media</t>
+        </is>
+      </c>
+      <c r="B146" s="2" t="inlineStr">
+        <is>
+          <t>Medios inmersivos</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="2" t="inlineStr">
+        <is>
+          <t>Interactives</t>
+        </is>
+      </c>
+      <c r="B147" s="2" t="inlineStr">
+        <is>
+          <t>Interactivos</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="2" t="inlineStr">
+        <is>
+          <t>Learning environment</t>
+        </is>
+      </c>
+      <c r="B148" s="2" t="inlineStr">
+        <is>
+          <t>Entorno de aprendizaje</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="2" t="inlineStr">
+        <is>
+          <t>Master Planning</t>
+        </is>
+      </c>
+      <c r="B149" s="2" t="inlineStr">
+        <is>
+          <t>Plan maestro</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="2" t="inlineStr">
+        <is>
+          <t>Policy making</t>
+        </is>
+      </c>
+      <c r="B150" s="2" t="inlineStr">
+        <is>
+          <t>Política pública</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="2" t="inlineStr">
+        <is>
+          <t>Product Design and Strategy</t>
+        </is>
+      </c>
+      <c r="B151" s="2" t="inlineStr">
+        <is>
+          <t>Diseño y estrategia de producto</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="2" t="inlineStr">
+        <is>
+          <t>Purpose-driven strategy</t>
+        </is>
+      </c>
+      <c r="B152" s="2" t="inlineStr">
+        <is>
+          <t>Estrategia con propósito</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="2" t="inlineStr">
+        <is>
+          <t>Science center</t>
+        </is>
+      </c>
+      <c r="B153" s="2" t="inlineStr">
+        <is>
+          <t>Centro de ciencia</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="2" t="inlineStr">
+        <is>
+          <t>Strategy</t>
+        </is>
+      </c>
+      <c r="B154" s="2" t="inlineStr">
+        <is>
+          <t>Estrategia</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="2" t="inlineStr">
+        <is>
+          <t>Sustainable Futures</t>
+        </is>
+      </c>
+      <c r="B155" s="2" t="inlineStr">
+        <is>
+          <t>Futuros sostenibles</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="2" t="inlineStr">
+        <is>
+          <t>Temporary exhibition</t>
+        </is>
+      </c>
+      <c r="B156" s="2" t="inlineStr">
+        <is>
+          <t>Exposición temporal</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="2" t="inlineStr">
+        <is>
+          <t>Transformation</t>
+        </is>
+      </c>
+      <c r="B157" s="2" t="inlineStr">
+        <is>
+          <t>Transformación</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="2" t="inlineStr">
+        <is>
+          <t>Traveling exhibition</t>
+        </is>
+      </c>
+      <c r="B158" s="2" t="inlineStr">
+        <is>
+          <t>Exposición itinerante</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="2" t="inlineStr">
+        <is>
+          <t>Ux</t>
+        </is>
+      </c>
+      <c r="B159" s="2" t="inlineStr">
+        <is>
+          <t>UX</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="2" t="inlineStr">
+        <is>
+          <t>Workshop / Bootcamp</t>
+        </is>
+      </c>
+      <c r="B160" s="2" t="inlineStr">
+        <is>
+          <t>Taller / Bootcamp</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="2" t="inlineStr">
+        <is>
+          <t>Author</t>
+        </is>
+      </c>
+      <c r="B161" s="2" t="inlineStr">
+        <is>
+          <t>Autor</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="2" t="inlineStr">
+        <is>
+          <t>Creative director</t>
+        </is>
+      </c>
+      <c r="B162" s="2" t="inlineStr">
+        <is>
+          <t>Director creativo</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="2" t="inlineStr">
+        <is>
+          <t>Exhibition Designer</t>
+        </is>
+      </c>
+      <c r="B163" s="2" t="inlineStr">
+        <is>
+          <t>Diseñador de exposiciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="2" t="inlineStr">
+        <is>
+          <t>Interior designer</t>
+        </is>
+      </c>
+      <c r="B164" s="2" t="inlineStr">
+        <is>
+          <t>Diseñador de interiores</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="2" t="inlineStr">
+        <is>
+          <t>Project leader</t>
+        </is>
+      </c>
+      <c r="B165" s="2" t="inlineStr">
+        <is>
+          <t>Líder de proyecto</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="2" t="inlineStr">
+        <is>
+          <t>Researcher</t>
+        </is>
+      </c>
+      <c r="B166" s="2" t="inlineStr">
+        <is>
+          <t>Investigador</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="2" t="inlineStr">
+        <is>
+          <t>Senior Exhibition Designer</t>
+        </is>
+      </c>
+      <c r="B167" s="2" t="inlineStr">
+        <is>
+          <t>Diseñador sénior de exposiciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="2" t="inlineStr">
+        <is>
+          <t>Senior designer</t>
+        </is>
+      </c>
+      <c r="B168" s="2" t="inlineStr">
+        <is>
+          <t>Diseñador sénior</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="2" t="inlineStr">
+        <is>
+          <t>Strategic Design &amp; CX Lead</t>
+        </is>
+      </c>
+      <c r="B169" s="2" t="inlineStr">
+        <is>
+          <t>Líder de diseño estratégico y CX</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="2" t="inlineStr">
+        <is>
+          <t>Strategic Design Consultant</t>
+        </is>
+      </c>
+      <c r="B170" s="2" t="inlineStr">
+        <is>
+          <t>Consultor de diseño estratégico</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="2" t="inlineStr">
+        <is>
+          <t>Strategy Consulting Director</t>
+        </is>
+      </c>
+      <c r="B171" s="2" t="inlineStr">
+        <is>
+          <t>Director de consultoría estratégica</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="2" t="inlineStr">
+        <is>
           <t>Volunteer</t>
         </is>
       </c>
-      <c r="B142" s="2" t="inlineStr">
+      <c r="B172" s="2" t="inlineStr">
         <is>
           <t>Voluntario</t>
         </is>

</xml_diff>

<commit_message>
Home: clients as 5 counter-moving marquee rows ordered by priority
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/database/hipernova-portafolio-db.xlsx
+++ b/database/hipernova-portafolio-db.xlsx
@@ -6091,7 +6091,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -6145,33 +6145,37 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>disciplines</t>
+          <t>clients</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Strategic Design | Design Futures | Transformation Design | CX Strategy</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Diseño estratégico | Prospectiva de diseño | Diseño de transformación | Estrategia de CX</t>
-        </is>
-      </c>
+          <t>Ecopetrol | Parque Explora | MTS | FAIN | Itaú Bank | The Bogotá Chamber of Commerce (CCB) | Afore Coppel | Coca-Cola Company | Coca-Cola FEMSA | Coppel - Retail | Zoológico de Barranquilla | Audubon | CIAT | Fundación Puerto Colombia | Ministry of Culture | Alcaldía de Cúcuta | Biblioteca Pública Piloto | Ministry of Education | Biblioteca Departamental | INCIVA | Panama Canal Authority | Embajada de Francia en Colombia | Secretaría Distrital de Cultura Recreación y Deporte (Bogotá) | Comfama | Gold Museum of Bogotá | Colciencias | Alcaldía de Medellín</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>substack</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr"/>
-      <c r="C5" s="2" t="inlineStr"/>
+          <t>disciplines</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Strategic Design | Design Futures | Transformation Design | CX Strategy</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Diseño estratégico | Prospectiva de diseño | Diseño de transformación | Estrategia de CX</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>linkedin</t>
+          <t>substack</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr"/>
@@ -6180,7 +6184,7 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>email</t>
+          <t>linkedin</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr"/>
@@ -6189,15 +6193,24 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr"/>
+      <c r="C8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
           <t>date</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>08.10.2026</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr"/>
+      <c r="C9" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Fix typo: Goverment -> Government
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/database/hipernova-portafolio-db.xlsx
+++ b/database/hipernova-portafolio-db.xlsx
@@ -1238,7 +1238,7 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Goverment / Public</t>
+          <t>Government / Public</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
@@ -2371,7 +2371,7 @@
       <c r="G19" s="2" t="inlineStr"/>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>Goverment / Public</t>
+          <t>Government / Public</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
@@ -3284,7 +3284,7 @@
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>Culture &amp; Museums | Goverment / Public</t>
+          <t>Culture &amp; Museums | Government / Public</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
@@ -3522,7 +3522,7 @@
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>Goverment / Public | Culture &amp; Museums</t>
+          <t>Government / Public | Culture &amp; Museums</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
@@ -4017,7 +4017,7 @@
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>Goverment / Public | Culture &amp; Museums</t>
+          <t>Government / Public | Culture &amp; Museums</t>
         </is>
       </c>
       <c r="I35" s="2" t="inlineStr">
@@ -4124,7 +4124,7 @@
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>Goverment / Public</t>
+          <t>Government / Public</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr">
@@ -4334,7 +4334,7 @@
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>Goverment / Public | Culture &amp; Museums</t>
+          <t>Government / Public | Culture &amp; Museums</t>
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr">
@@ -4748,7 +4748,7 @@
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>Culture &amp; Museums | Goverment / Public</t>
+          <t>Culture &amp; Museums | Government / Public</t>
         </is>
       </c>
       <c r="I42" s="2" t="inlineStr">
@@ -4960,7 +4960,7 @@
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>Goverment / Public | Education</t>
+          <t>Government / Public | Education</t>
         </is>
       </c>
       <c r="I44" s="2" t="inlineStr">
@@ -6223,7 +6223,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B172"/>
+  <dimension ref="A1:B173"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -7841,7 +7841,7 @@
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
         <is>
-          <t>Goverment / Public</t>
+          <t>Government / Public</t>
         </is>
       </c>
       <c r="B135" s="2" t="inlineStr">
@@ -7853,442 +7853,454 @@
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
         <is>
-          <t>Retail</t>
+          <t>Goverment / Public</t>
         </is>
       </c>
       <c r="B136" s="2" t="inlineStr">
         <is>
-          <t>Retail</t>
+          <t>Gobierno / Público</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
         <is>
-          <t>Science - Research</t>
+          <t>Retail</t>
         </is>
       </c>
       <c r="B137" s="2" t="inlineStr">
         <is>
-          <t>Ciencia - Investigación</t>
+          <t>Retail</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
         <is>
-          <t>Third Sector / NGOs</t>
+          <t>Science - Research</t>
         </is>
       </c>
       <c r="B138" s="2" t="inlineStr">
         <is>
-          <t>Tercer sector / ONG</t>
+          <t>Ciencia - Investigación</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
         <is>
-          <t>CX Strategy</t>
+          <t>Third Sector / NGOs</t>
         </is>
       </c>
       <c r="B139" s="2" t="inlineStr">
         <is>
-          <t>Estrategia de CX</t>
+          <t>Tercer sector / ONG</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
         <is>
-          <t>Creative space</t>
+          <t>CX Strategy</t>
         </is>
       </c>
       <c r="B140" s="2" t="inlineStr">
         <is>
-          <t>Espacio creativo</t>
+          <t>Estrategia de CX</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
         <is>
-          <t>Customer Experience and Innovation</t>
+          <t>Creative space</t>
         </is>
       </c>
       <c r="B141" s="2" t="inlineStr">
         <is>
-          <t>Experiencia de cliente e innovación</t>
+          <t>Espacio creativo</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
         <is>
-          <t>Data visualization</t>
+          <t>Customer Experience and Innovation</t>
         </is>
       </c>
       <c r="B142" s="2" t="inlineStr">
         <is>
-          <t>Visualización de datos</t>
+          <t>Experiencia de cliente e innovación</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
         <is>
-          <t>Digital experience</t>
+          <t>Data visualization</t>
         </is>
       </c>
       <c r="B143" s="2" t="inlineStr">
         <is>
-          <t>Experiencia digital</t>
+          <t>Visualización de datos</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
         <is>
-          <t>Digital product</t>
+          <t>Digital experience</t>
         </is>
       </c>
       <c r="B144" s="2" t="inlineStr">
         <is>
-          <t>Producto digital</t>
+          <t>Experiencia digital</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
         <is>
-          <t>Exhibition</t>
+          <t>Digital product</t>
         </is>
       </c>
       <c r="B145" s="2" t="inlineStr">
         <is>
-          <t>Exposición</t>
+          <t>Producto digital</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
         <is>
-          <t>Immersive media</t>
+          <t>Exhibition</t>
         </is>
       </c>
       <c r="B146" s="2" t="inlineStr">
         <is>
-          <t>Medios inmersivos</t>
+          <t>Exposición</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
         <is>
-          <t>Interactives</t>
+          <t>Immersive media</t>
         </is>
       </c>
       <c r="B147" s="2" t="inlineStr">
         <is>
-          <t>Interactivos</t>
+          <t>Medios inmersivos</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
         <is>
-          <t>Learning environment</t>
+          <t>Interactives</t>
         </is>
       </c>
       <c r="B148" s="2" t="inlineStr">
         <is>
-          <t>Entorno de aprendizaje</t>
+          <t>Interactivos</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
         <is>
-          <t>Master Planning</t>
+          <t>Learning environment</t>
         </is>
       </c>
       <c r="B149" s="2" t="inlineStr">
         <is>
-          <t>Plan maestro</t>
+          <t>Entorno de aprendizaje</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
         <is>
-          <t>Policy making</t>
+          <t>Master Planning</t>
         </is>
       </c>
       <c r="B150" s="2" t="inlineStr">
         <is>
-          <t>Política pública</t>
+          <t>Plan maestro</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
         <is>
-          <t>Product Design and Strategy</t>
+          <t>Policy making</t>
         </is>
       </c>
       <c r="B151" s="2" t="inlineStr">
         <is>
-          <t>Diseño y estrategia de producto</t>
+          <t>Política pública</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
         <is>
-          <t>Purpose-driven strategy</t>
+          <t>Product Design and Strategy</t>
         </is>
       </c>
       <c r="B152" s="2" t="inlineStr">
         <is>
-          <t>Estrategia con propósito</t>
+          <t>Diseño y estrategia de producto</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
         <is>
-          <t>Science center</t>
+          <t>Purpose-driven strategy</t>
         </is>
       </c>
       <c r="B153" s="2" t="inlineStr">
         <is>
-          <t>Centro de ciencia</t>
+          <t>Estrategia con propósito</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
         <is>
-          <t>Strategy</t>
+          <t>Science center</t>
         </is>
       </c>
       <c r="B154" s="2" t="inlineStr">
         <is>
-          <t>Estrategia</t>
+          <t>Centro de ciencia</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
         <is>
-          <t>Sustainable Futures</t>
+          <t>Strategy</t>
         </is>
       </c>
       <c r="B155" s="2" t="inlineStr">
         <is>
-          <t>Futuros sostenibles</t>
+          <t>Estrategia</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
         <is>
-          <t>Temporary exhibition</t>
+          <t>Sustainable Futures</t>
         </is>
       </c>
       <c r="B156" s="2" t="inlineStr">
         <is>
-          <t>Exposición temporal</t>
+          <t>Futuros sostenibles</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
         <is>
-          <t>Transformation</t>
+          <t>Temporary exhibition</t>
         </is>
       </c>
       <c r="B157" s="2" t="inlineStr">
         <is>
-          <t>Transformación</t>
+          <t>Exposición temporal</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
         <is>
-          <t>Traveling exhibition</t>
+          <t>Transformation</t>
         </is>
       </c>
       <c r="B158" s="2" t="inlineStr">
         <is>
-          <t>Exposición itinerante</t>
+          <t>Transformación</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
         <is>
-          <t>Ux</t>
+          <t>Traveling exhibition</t>
         </is>
       </c>
       <c r="B159" s="2" t="inlineStr">
         <is>
-          <t>UX</t>
+          <t>Exposición itinerante</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
         <is>
-          <t>Workshop / Bootcamp</t>
+          <t>Ux</t>
         </is>
       </c>
       <c r="B160" s="2" t="inlineStr">
         <is>
-          <t>Taller / Bootcamp</t>
+          <t>UX</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
         <is>
-          <t>Author</t>
+          <t>Workshop / Bootcamp</t>
         </is>
       </c>
       <c r="B161" s="2" t="inlineStr">
         <is>
-          <t>Autor</t>
+          <t>Taller / Bootcamp</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
         <is>
-          <t>Creative director</t>
+          <t>Author</t>
         </is>
       </c>
       <c r="B162" s="2" t="inlineStr">
         <is>
-          <t>Director creativo</t>
+          <t>Autor</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
         <is>
-          <t>Exhibition Designer</t>
+          <t>Creative director</t>
         </is>
       </c>
       <c r="B163" s="2" t="inlineStr">
         <is>
-          <t>Diseñador de exposiciones</t>
+          <t>Director creativo</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
         <is>
-          <t>Interior designer</t>
+          <t>Exhibition Designer</t>
         </is>
       </c>
       <c r="B164" s="2" t="inlineStr">
         <is>
-          <t>Diseñador de interiores</t>
+          <t>Diseñador de exposiciones</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
         <is>
-          <t>Project leader</t>
+          <t>Interior designer</t>
         </is>
       </c>
       <c r="B165" s="2" t="inlineStr">
         <is>
-          <t>Líder de proyecto</t>
+          <t>Diseñador de interiores</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" s="2" t="inlineStr">
         <is>
-          <t>Researcher</t>
+          <t>Project leader</t>
         </is>
       </c>
       <c r="B166" s="2" t="inlineStr">
         <is>
-          <t>Investigador</t>
+          <t>Líder de proyecto</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" s="2" t="inlineStr">
         <is>
-          <t>Senior Exhibition Designer</t>
+          <t>Researcher</t>
         </is>
       </c>
       <c r="B167" s="2" t="inlineStr">
         <is>
-          <t>Diseñador sénior de exposiciones</t>
+          <t>Investigador</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" s="2" t="inlineStr">
         <is>
-          <t>Senior designer</t>
+          <t>Senior Exhibition Designer</t>
         </is>
       </c>
       <c r="B168" s="2" t="inlineStr">
         <is>
-          <t>Diseñador sénior</t>
+          <t>Diseñador sénior de exposiciones</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" s="2" t="inlineStr">
         <is>
-          <t>Strategic Design &amp; CX Lead</t>
+          <t>Senior designer</t>
         </is>
       </c>
       <c r="B169" s="2" t="inlineStr">
         <is>
-          <t>Líder de diseño estratégico y CX</t>
+          <t>Diseñador sénior</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" s="2" t="inlineStr">
         <is>
-          <t>Strategic Design Consultant</t>
+          <t>Strategic Design &amp; CX Lead</t>
         </is>
       </c>
       <c r="B170" s="2" t="inlineStr">
         <is>
-          <t>Consultor de diseño estratégico</t>
+          <t>Líder de diseño estratégico y CX</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" s="2" t="inlineStr">
         <is>
-          <t>Strategy Consulting Director</t>
+          <t>Strategic Design Consultant</t>
         </is>
       </c>
       <c r="B171" s="2" t="inlineStr">
         <is>
-          <t>Director de consultoría estratégica</t>
+          <t>Consultor de diseño estratégico</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" s="2" t="inlineStr">
         <is>
+          <t>Strategy Consulting Director</t>
+        </is>
+      </c>
+      <c r="B172" s="2" t="inlineStr">
+        <is>
+          <t>Director de consultoría estratégica</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="2" t="inlineStr">
+        <is>
           <t>Volunteer</t>
         </is>
       </c>
-      <c r="B172" s="2" t="inlineStr">
+      <c r="B173" s="2" t="inlineStr">
         <is>
           <t>Voluntario</t>
         </is>

</xml_diff>

<commit_message>
Translations: new tags/clients, ES fixes (OPEX title, Shell VAX image + accent), safe overwrite mechanism
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/database/hipernova-portafolio-db.xlsx
+++ b/database/hipernova-portafolio-db.xlsx
@@ -6223,7 +6223,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B173"/>
+  <dimension ref="A1:B181"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -7781,526 +7781,622 @@
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
         <is>
-          <t>CPG</t>
+          <t>Energy &amp; Construction</t>
         </is>
       </c>
       <c r="B130" s="2" t="inlineStr">
         <is>
-          <t>Bienes de consumo</t>
+          <t>Energía y construcción</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
         <is>
-          <t>Culture &amp; Museums</t>
+          <t>AI &amp; Strategic Design</t>
         </is>
       </c>
       <c r="B131" s="2" t="inlineStr">
         <is>
-          <t>Cultura y museos</t>
+          <t>IA y diseño estratégico</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Consulting Director / Strategic Lead</t>
         </is>
       </c>
       <c r="B132" s="2" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Director de consultoría / Líder estratégico</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Ministry of Culture</t>
         </is>
       </c>
       <c r="B133" s="2" t="inlineStr">
         <is>
-          <t>Energía</t>
+          <t>Ministerio de Cultura</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
         <is>
-          <t>Financial Services</t>
+          <t>Ministry of Education</t>
         </is>
       </c>
       <c r="B134" s="2" t="inlineStr">
         <is>
-          <t>Servicios financieros</t>
+          <t>Ministerio de Educación</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
         <is>
-          <t>Government / Public</t>
+          <t>Gold Museum of Bogotá</t>
         </is>
       </c>
       <c r="B135" s="2" t="inlineStr">
         <is>
-          <t>Gobierno / Público</t>
+          <t>Museo del Oro de Bogotá</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
         <is>
-          <t>Goverment / Public</t>
+          <t>The Bogotá Chamber of Commerce (CCB)</t>
         </is>
       </c>
       <c r="B136" s="2" t="inlineStr">
         <is>
-          <t>Gobierno / Público</t>
+          <t>Cámara de Comercio de Bogotá (CCB)</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
         <is>
-          <t>Retail</t>
+          <t>Panama Canal Authority</t>
         </is>
       </c>
       <c r="B137" s="2" t="inlineStr">
         <is>
-          <t>Retail</t>
+          <t>Autoridad del Canal de Panamá</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
         <is>
-          <t>Science - Research</t>
+          <t>CPG</t>
         </is>
       </c>
       <c r="B138" s="2" t="inlineStr">
         <is>
-          <t>Ciencia - Investigación</t>
+          <t>Bienes de consumo</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
         <is>
-          <t>Third Sector / NGOs</t>
+          <t>Culture &amp; Museums</t>
         </is>
       </c>
       <c r="B139" s="2" t="inlineStr">
         <is>
-          <t>Tercer sector / ONG</t>
+          <t>Cultura y museos</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
         <is>
-          <t>CX Strategy</t>
+          <t>Education</t>
         </is>
       </c>
       <c r="B140" s="2" t="inlineStr">
         <is>
-          <t>Estrategia de CX</t>
+          <t>Educación</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
         <is>
-          <t>Creative space</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="B141" s="2" t="inlineStr">
         <is>
-          <t>Espacio creativo</t>
+          <t>Energía</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
         <is>
-          <t>Customer Experience and Innovation</t>
+          <t>Financial Services</t>
         </is>
       </c>
       <c r="B142" s="2" t="inlineStr">
         <is>
-          <t>Experiencia de cliente e innovación</t>
+          <t>Servicios financieros</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
         <is>
-          <t>Data visualization</t>
+          <t>Government / Public</t>
         </is>
       </c>
       <c r="B143" s="2" t="inlineStr">
         <is>
-          <t>Visualización de datos</t>
+          <t>Gobierno / Público</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
         <is>
-          <t>Digital experience</t>
+          <t>Goverment / Public</t>
         </is>
       </c>
       <c r="B144" s="2" t="inlineStr">
         <is>
-          <t>Experiencia digital</t>
+          <t>Gobierno / Público</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
         <is>
-          <t>Digital product</t>
+          <t>Retail</t>
         </is>
       </c>
       <c r="B145" s="2" t="inlineStr">
         <is>
-          <t>Producto digital</t>
+          <t>Retail</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
         <is>
-          <t>Exhibition</t>
+          <t>Science - Research</t>
         </is>
       </c>
       <c r="B146" s="2" t="inlineStr">
         <is>
-          <t>Exposición</t>
+          <t>Ciencia - Investigación</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
         <is>
-          <t>Immersive media</t>
+          <t>Third Sector / NGOs</t>
         </is>
       </c>
       <c r="B147" s="2" t="inlineStr">
         <is>
-          <t>Medios inmersivos</t>
+          <t>Tercer sector / ONG</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
         <is>
-          <t>Interactives</t>
+          <t>CX Strategy</t>
         </is>
       </c>
       <c r="B148" s="2" t="inlineStr">
         <is>
-          <t>Interactivos</t>
+          <t>Estrategia de CX</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
         <is>
-          <t>Learning environment</t>
+          <t>Creative space</t>
         </is>
       </c>
       <c r="B149" s="2" t="inlineStr">
         <is>
-          <t>Entorno de aprendizaje</t>
+          <t>Espacio creativo</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
         <is>
-          <t>Master Planning</t>
+          <t>Customer Experience and Innovation</t>
         </is>
       </c>
       <c r="B150" s="2" t="inlineStr">
         <is>
-          <t>Plan maestro</t>
+          <t>Experiencia de cliente e innovación</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
         <is>
-          <t>Policy making</t>
+          <t>Data visualization</t>
         </is>
       </c>
       <c r="B151" s="2" t="inlineStr">
         <is>
-          <t>Política pública</t>
+          <t>Visualización de datos</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
         <is>
-          <t>Product Design and Strategy</t>
+          <t>Digital experience</t>
         </is>
       </c>
       <c r="B152" s="2" t="inlineStr">
         <is>
-          <t>Diseño y estrategia de producto</t>
+          <t>Experiencia digital</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
         <is>
-          <t>Purpose-driven strategy</t>
+          <t>Digital product</t>
         </is>
       </c>
       <c r="B153" s="2" t="inlineStr">
         <is>
-          <t>Estrategia con propósito</t>
+          <t>Producto digital</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
         <is>
-          <t>Science center</t>
+          <t>Exhibition</t>
         </is>
       </c>
       <c r="B154" s="2" t="inlineStr">
         <is>
-          <t>Centro de ciencia</t>
+          <t>Exposición</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
         <is>
-          <t>Strategy</t>
+          <t>Immersive media</t>
         </is>
       </c>
       <c r="B155" s="2" t="inlineStr">
         <is>
-          <t>Estrategia</t>
+          <t>Medios inmersivos</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
         <is>
-          <t>Sustainable Futures</t>
+          <t>Interactives</t>
         </is>
       </c>
       <c r="B156" s="2" t="inlineStr">
         <is>
-          <t>Futuros sostenibles</t>
+          <t>Interactivos</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
         <is>
-          <t>Temporary exhibition</t>
+          <t>Learning environment</t>
         </is>
       </c>
       <c r="B157" s="2" t="inlineStr">
         <is>
-          <t>Exposición temporal</t>
+          <t>Entorno de aprendizaje</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
         <is>
-          <t>Transformation</t>
+          <t>Master Planning</t>
         </is>
       </c>
       <c r="B158" s="2" t="inlineStr">
         <is>
-          <t>Transformación</t>
+          <t>Plan maestro</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
         <is>
-          <t>Traveling exhibition</t>
+          <t>Policy making</t>
         </is>
       </c>
       <c r="B159" s="2" t="inlineStr">
         <is>
-          <t>Exposición itinerante</t>
+          <t>Política pública</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
         <is>
-          <t>Ux</t>
+          <t>Product Design and Strategy</t>
         </is>
       </c>
       <c r="B160" s="2" t="inlineStr">
         <is>
-          <t>UX</t>
+          <t>Diseño y estrategia de producto</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
         <is>
-          <t>Workshop / Bootcamp</t>
+          <t>Purpose-driven strategy</t>
         </is>
       </c>
       <c r="B161" s="2" t="inlineStr">
         <is>
-          <t>Taller / Bootcamp</t>
+          <t>Estrategia con propósito</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
         <is>
-          <t>Author</t>
+          <t>Science center</t>
         </is>
       </c>
       <c r="B162" s="2" t="inlineStr">
         <is>
-          <t>Autor</t>
+          <t>Centro de ciencia</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
         <is>
-          <t>Creative director</t>
+          <t>Strategy</t>
         </is>
       </c>
       <c r="B163" s="2" t="inlineStr">
         <is>
-          <t>Director creativo</t>
+          <t>Estrategia</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
         <is>
-          <t>Exhibition Designer</t>
+          <t>Sustainable Futures</t>
         </is>
       </c>
       <c r="B164" s="2" t="inlineStr">
         <is>
-          <t>Diseñador de exposiciones</t>
+          <t>Futuros sostenibles</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
         <is>
-          <t>Interior designer</t>
+          <t>Temporary exhibition</t>
         </is>
       </c>
       <c r="B165" s="2" t="inlineStr">
         <is>
-          <t>Diseñador de interiores</t>
+          <t>Exposición temporal</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" s="2" t="inlineStr">
         <is>
-          <t>Project leader</t>
+          <t>Transformation</t>
         </is>
       </c>
       <c r="B166" s="2" t="inlineStr">
         <is>
-          <t>Líder de proyecto</t>
+          <t>Transformación</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" s="2" t="inlineStr">
         <is>
-          <t>Researcher</t>
+          <t>Traveling exhibition</t>
         </is>
       </c>
       <c r="B167" s="2" t="inlineStr">
         <is>
-          <t>Investigador</t>
+          <t>Exposición itinerante</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" s="2" t="inlineStr">
         <is>
-          <t>Senior Exhibition Designer</t>
+          <t>Ux</t>
         </is>
       </c>
       <c r="B168" s="2" t="inlineStr">
         <is>
-          <t>Diseñador sénior de exposiciones</t>
+          <t>UX</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" s="2" t="inlineStr">
         <is>
-          <t>Senior designer</t>
+          <t>Workshop / Bootcamp</t>
         </is>
       </c>
       <c r="B169" s="2" t="inlineStr">
         <is>
-          <t>Diseñador sénior</t>
+          <t>Taller / Bootcamp</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" s="2" t="inlineStr">
         <is>
-          <t>Strategic Design &amp; CX Lead</t>
+          <t>Author</t>
         </is>
       </c>
       <c r="B170" s="2" t="inlineStr">
         <is>
-          <t>Líder de diseño estratégico y CX</t>
+          <t>Autor</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" s="2" t="inlineStr">
         <is>
-          <t>Strategic Design Consultant</t>
+          <t>Creative director</t>
         </is>
       </c>
       <c r="B171" s="2" t="inlineStr">
         <is>
-          <t>Consultor de diseño estratégico</t>
+          <t>Director creativo</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" s="2" t="inlineStr">
         <is>
-          <t>Strategy Consulting Director</t>
+          <t>Exhibition Designer</t>
         </is>
       </c>
       <c r="B172" s="2" t="inlineStr">
         <is>
-          <t>Director de consultoría estratégica</t>
+          <t>Diseñador de exposiciones</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" s="2" t="inlineStr">
         <is>
+          <t>Interior designer</t>
+        </is>
+      </c>
+      <c r="B173" s="2" t="inlineStr">
+        <is>
+          <t>Diseñador de interiores</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="2" t="inlineStr">
+        <is>
+          <t>Project leader</t>
+        </is>
+      </c>
+      <c r="B174" s="2" t="inlineStr">
+        <is>
+          <t>Líder de proyecto</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="2" t="inlineStr">
+        <is>
+          <t>Researcher</t>
+        </is>
+      </c>
+      <c r="B175" s="2" t="inlineStr">
+        <is>
+          <t>Investigador</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="2" t="inlineStr">
+        <is>
+          <t>Senior Exhibition Designer</t>
+        </is>
+      </c>
+      <c r="B176" s="2" t="inlineStr">
+        <is>
+          <t>Diseñador sénior de exposiciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="2" t="inlineStr">
+        <is>
+          <t>Senior designer</t>
+        </is>
+      </c>
+      <c r="B177" s="2" t="inlineStr">
+        <is>
+          <t>Diseñador sénior</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="2" t="inlineStr">
+        <is>
+          <t>Strategic Design &amp; CX Lead</t>
+        </is>
+      </c>
+      <c r="B178" s="2" t="inlineStr">
+        <is>
+          <t>Líder de diseño estratégico y CX</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="2" t="inlineStr">
+        <is>
+          <t>Strategic Design Consultant</t>
+        </is>
+      </c>
+      <c r="B179" s="2" t="inlineStr">
+        <is>
+          <t>Consultor de diseño estratégico</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="2" t="inlineStr">
+        <is>
+          <t>Strategy Consulting Director</t>
+        </is>
+      </c>
+      <c r="B180" s="2" t="inlineStr">
+        <is>
+          <t>Director de consultoría estratégica</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="2" t="inlineStr">
+        <is>
           <t>Volunteer</t>
         </is>
       </c>
-      <c r="B173" s="2" t="inlineStr">
+      <c r="B181" s="2" t="inlineStr">
         <is>
           <t>Voluntario</t>
         </is>

</xml_diff>